<commit_message>
Close Day 9 and log Day 10 breakfast
Day 9 closes at 1,998 kcal - the closing scoops and the grilled chicken
were discussed but never confirmed, so neither is logged. That makes it
a -671 day at 89.5 g of protein, the lowest since Day 1.

Day 10 is Sunday, the roomiest menu of the week: halve the ghee rice at
lunch and three scoops clears the protein floor at a 664 deficit.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N54"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3361,6 +3361,61 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="4" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>2 wheat porotta + kadala curry</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="n">
+        <v>520</v>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>750</v>
+      </c>
+      <c r="F55" s="8">
+        <f>AVERAGE(D55:E55)</f>
+        <v/>
+      </c>
+      <c r="G55" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="H55" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="I55" s="10">
+        <f>AVERAGE(G55:H55)</f>
+        <v/>
+      </c>
+      <c r="J55" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="K55" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="L55" s="10">
+        <f>AVERAGE(J55:K55)</f>
+        <v/>
+      </c>
+      <c r="M55" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N55" s="6" t="inlineStr">
+        <is>
+          <t>Sunday mess breakfast; kadala poured over. A second container in the photo was not identifiable and is not counted</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -3375,7 +3430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3479,11 +3534,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3491,11 +3546,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3503,11 +3558,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3515,11 +3570,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3532,11 +3587,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3544,11 +3599,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3556,11 +3611,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3568,11 +3623,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3585,11 +3640,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3597,11 +3652,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3609,11 +3664,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3621,11 +3676,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3638,11 +3693,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3650,11 +3705,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3662,11 +3717,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3674,11 +3729,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3691,11 +3746,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3703,11 +3758,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3715,11 +3770,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3727,11 +3782,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3744,11 +3799,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3756,11 +3811,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3768,11 +3823,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3780,11 +3835,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3797,11 +3852,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3809,11 +3864,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3821,11 +3876,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3833,11 +3888,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -3850,11 +3905,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -3862,11 +3917,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -3874,11 +3929,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -3886,11 +3941,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -3903,11 +3958,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -3915,11 +3970,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -3927,11 +3982,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -3939,15 +3994,68 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
         <f>D13-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B14" s="21">
+        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"logged")</f>
+        <v/>
+      </c>
+      <c r="C14" s="21">
+        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"logged")</f>
+        <v/>
+      </c>
+      <c r="D14" s="21">
+        <f>AVERAGE(B14:C14)</f>
+        <v/>
+      </c>
+      <c r="E14" s="22">
+        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"logged")</f>
+        <v/>
+      </c>
+      <c r="F14" s="22">
+        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"logged")</f>
+        <v/>
+      </c>
+      <c r="G14" s="22">
+        <f>AVERAGE(E14:F14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="22">
+        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"logged")</f>
+        <v/>
+      </c>
+      <c r="I14" s="22">
+        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"logged")</f>
+        <v/>
+      </c>
+      <c r="J14" s="22">
+        <f>AVERAGE(H14:I14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"logged")</f>
+        <v/>
+      </c>
+      <c r="L14" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"pending")</f>
+        <v/>
+      </c>
+      <c r="M14" s="23">
+        <f>D14-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -4881,7 +4989,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$13)</f>
+        <f>COUNT(Daily!$A$5:$A$14)</f>
         <v/>
       </c>
     </row>
@@ -4892,7 +5000,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$13),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$14),0)</f>
         <v/>
       </c>
     </row>
@@ -4903,7 +5011,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$13),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$14),0)</f>
         <v/>
       </c>
     </row>
@@ -4914,7 +5022,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$13),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$14),0)</f>
         <v/>
       </c>
     </row>
@@ -4958,7 +5066,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$13,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$14,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -4969,7 +5077,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$13)</f>
+        <f>SUM(Daily!$L$5:$L$14)</f>
         <v/>
       </c>
     </row>
@@ -5020,19 +5128,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$13,"&gt;="&amp;$A17,Daily!$A$5:$A$13,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$14,"&gt;="&amp;$A17,Daily!$A$5:$A$14,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$13,Daily!$A$5:$A$13,"&gt;="&amp;$A17,Daily!$A$5:$A$13,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$14,Daily!$A$5:$A$14,"&gt;="&amp;$A17,Daily!$A$5:$A$14,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$13,Daily!$A$5:$A$13,"&gt;="&amp;$A17,Daily!$A$5:$A$13,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$14,Daily!$A$5:$A$14,"&gt;="&amp;$A17,Daily!$A$5:$A$14,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$13,Daily!$A$5:$A$13,"&gt;="&amp;$A17,Daily!$A$5:$A$13,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$14,Daily!$A$5:$A$14,"&gt;="&amp;$A17,Daily!$A$5:$A$14,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -5044,19 +5152,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$13,"&gt;="&amp;$A18,Daily!$A$5:$A$13,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$14,"&gt;="&amp;$A18,Daily!$A$5:$A$14,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$13,Daily!$A$5:$A$13,"&gt;="&amp;$A18,Daily!$A$5:$A$13,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$14,Daily!$A$5:$A$14,"&gt;="&amp;$A18,Daily!$A$5:$A$14,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$13,Daily!$A$5:$A$13,"&gt;="&amp;$A18,Daily!$A$5:$A$13,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$14,Daily!$A$5:$A$14,"&gt;="&amp;$A18,Daily!$A$5:$A$14,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$13,Daily!$A$5:$A$13,"&gt;="&amp;$A18,Daily!$A$5:$A$13,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$14,Daily!$A$5:$A$14,"&gt;="&amp;$A18,Daily!$A$5:$A$14,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -5107,19 +5215,19 @@
         <v>46295</v>
       </c>
       <c r="C22" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$13,"&gt;="&amp;$A22,Daily!$A$5:$A$13,"&lt;="&amp;$B22)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$14,"&gt;="&amp;$A22,Daily!$A$5:$A$14,"&lt;="&amp;$B22)</f>
         <v/>
       </c>
       <c r="D22" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$13,Daily!$A$5:$A$13,"&gt;="&amp;$A22,Daily!$A$5:$A$13,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$14,Daily!$A$5:$A$14,"&gt;="&amp;$A22,Daily!$A$5:$A$14,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
       <c r="E22" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$13,Daily!$A$5:$A$13,"&gt;="&amp;$A22,Daily!$A$5:$A$13,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$14,Daily!$A$5:$A$14,"&gt;="&amp;$A22,Daily!$A$5:$A$14,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
       <c r="F22" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$13,Daily!$A$5:$A$13,"&gt;="&amp;$A22,Daily!$A$5:$A$13,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$14,Daily!$A$5:$A$14,"&gt;="&amp;$A22,Daily!$A$5:$A$14,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Day 10 lunch: halved ghee rice with chicken curry
Rice halved again, coming in ~40 kcal under plan. The curry container
is counted in full since the photo cannot distinguish a lifted-out
chicken from a poured one.

Lands the evening on 4 scoops rather than 3: a third consecutive
large-deficit day at low protein is the wrong shape on a six-day split.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N55"/>
+  <dimension ref="A1:N56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3413,6 +3413,61 @@
       <c r="N55" s="6" t="inlineStr">
         <is>
           <t>Sunday mess breakfast; kadala poured over. A second container in the photo was not identifiable and is not counted</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>Ghee rice (halved) + chicken curry + curd</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="n">
+        <v>440</v>
+      </c>
+      <c r="E56" s="7" t="n">
+        <v>630</v>
+      </c>
+      <c r="F56" s="8">
+        <f>AVERAGE(D56:E56)</f>
+        <v/>
+      </c>
+      <c r="G56" s="9" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="H56" s="9" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="I56" s="10">
+        <f>AVERAGE(G56:H56)</f>
+        <v/>
+      </c>
+      <c r="J56" s="9" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="K56" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="L56" s="10">
+        <f>AVERAGE(J56:K56)</f>
+        <v/>
+      </c>
+      <c r="M56" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N56" s="6" t="inlineStr">
+        <is>
+          <t>Rice halved. Curry container photographed near-empty - counted as eaten in full</t>
         </is>
       </c>
     </row>
@@ -3534,11 +3589,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3546,11 +3601,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3558,11 +3613,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3570,11 +3625,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A5,Meals!$M$5:$M$55,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3587,11 +3642,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3599,11 +3654,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3611,11 +3666,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3623,11 +3678,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A6,Meals!$M$5:$M$55,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3640,11 +3695,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3652,11 +3707,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3664,11 +3719,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3676,11 +3731,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A7,Meals!$M$5:$M$55,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3693,11 +3748,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3705,11 +3760,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3717,11 +3772,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3729,11 +3784,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A8,Meals!$M$5:$M$55,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3746,11 +3801,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3758,11 +3813,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3770,11 +3825,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3782,11 +3837,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A9,Meals!$M$5:$M$55,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3799,11 +3854,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3811,11 +3866,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3823,11 +3878,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3835,11 +3890,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A10,Meals!$M$5:$M$55,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3852,11 +3907,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3864,11 +3919,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3876,11 +3931,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3888,11 +3943,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A11,Meals!$M$5:$M$55,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -3905,11 +3960,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -3917,11 +3972,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -3929,11 +3984,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -3941,11 +3996,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A12,Meals!$M$5:$M$55,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -3958,11 +4013,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -3970,11 +4025,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -3982,11 +4037,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -3994,11 +4049,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A13,Meals!$M$5:$M$55,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4011,11 +4066,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$55,Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$55,Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4023,11 +4078,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$55,Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$55,Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4035,11 +4090,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$55,Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$55,Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4047,11 +4102,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$55,$A14,Meals!$M$5:$M$55,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">

</xml_diff>

<commit_message>
Log 2 boiled eggs on Day 10 and settle the evening on 3 scoops
Eggs taken over the fourth scoop, which is the middle option from this
morning's plan. The day lands within 7 kcal of target at 145.5 g of
protein.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N56"/>
+  <dimension ref="A1:N57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3468,6 +3468,61 @@
       <c r="N56" s="6" t="inlineStr">
         <is>
           <t>Rice halved. Curry container photographed near-empty - counted as eaten in full</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>2 boiled eggs</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="E57" s="7" t="n">
+        <v>156</v>
+      </c>
+      <c r="F57" s="8">
+        <f>AVERAGE(D57:E57)</f>
+        <v/>
+      </c>
+      <c r="G57" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H57" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="I57" s="10">
+        <f>AVERAGE(G57:H57)</f>
+        <v/>
+      </c>
+      <c r="J57" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="K57" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="L57" s="10">
+        <f>AVERAGE(J57:K57)</f>
+        <v/>
+      </c>
+      <c r="M57" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N57" s="6" t="inlineStr">
+        <is>
+          <t>Took the eggs over the fourth scoop</t>
         </is>
       </c>
     </row>
@@ -3589,11 +3644,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3601,11 +3656,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3613,11 +3668,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3625,11 +3680,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A5,Meals!$M$5:$M$56,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3642,11 +3697,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3654,11 +3709,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3666,11 +3721,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3678,11 +3733,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A6,Meals!$M$5:$M$56,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3695,11 +3750,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3707,11 +3762,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3719,11 +3774,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3731,11 +3786,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A7,Meals!$M$5:$M$56,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3748,11 +3803,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3760,11 +3815,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3772,11 +3827,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3784,11 +3839,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A8,Meals!$M$5:$M$56,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3801,11 +3856,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3813,11 +3868,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3825,11 +3880,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3837,11 +3892,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A9,Meals!$M$5:$M$56,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3854,11 +3909,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3866,11 +3921,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3878,11 +3933,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3890,11 +3945,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A10,Meals!$M$5:$M$56,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3907,11 +3962,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3919,11 +3974,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3931,11 +3986,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3943,11 +3998,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A11,Meals!$M$5:$M$56,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -3960,11 +4015,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -3972,11 +4027,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -3984,11 +4039,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -3996,11 +4051,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A12,Meals!$M$5:$M$56,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4013,11 +4068,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4025,11 +4080,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4037,11 +4092,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4049,11 +4104,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A13,Meals!$M$5:$M$56,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4066,11 +4121,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$56,Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$56,Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4078,11 +4133,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$56,Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$56,Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4090,11 +4145,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$56,Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$56,Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4102,11 +4157,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$56,$A14,Meals!$M$5:$M$56,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">

</xml_diff>

<commit_message>
Log Day 10 dinner: 2 chapati, egg roast and 2 extra boiled eggs
Dinner ran ~170 kcal over the menu on two extra boiled eggs and an oily
roast masala, so the day lands at ~101 g of fat rather than the ~90
projected this morning. Closes on 2 scoops.

Adds the finding that this was not a coconut-gravy day and still came in
over 100 g of fat - five eggs carry ~26 g of it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N57"/>
+  <dimension ref="A1:N58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3422,39 +3422,39 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>Ghee rice (halved) + chicken curry + curd</t>
+          <t>2 chapati + egg roast (1 egg) + 2 boiled eggs</t>
         </is>
       </c>
       <c r="D56" s="7" t="n">
-        <v>440</v>
+        <v>540</v>
       </c>
       <c r="E56" s="7" t="n">
-        <v>630</v>
+        <v>696</v>
       </c>
       <c r="F56" s="8">
         <f>AVERAGE(D56:E56)</f>
         <v/>
       </c>
       <c r="G56" s="9" t="n">
-        <v>21.5</v>
+        <v>26</v>
       </c>
       <c r="H56" s="9" t="n">
-        <v>29.5</v>
+        <v>31</v>
       </c>
       <c r="I56" s="10">
         <f>AVERAGE(G56:H56)</f>
         <v/>
       </c>
       <c r="J56" s="9" t="n">
-        <v>18.5</v>
+        <v>28</v>
       </c>
       <c r="K56" s="9" t="n">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="L56" s="10">
         <f>AVERAGE(J56:K56)</f>
@@ -3467,7 +3467,7 @@
       </c>
       <c r="N56" s="6" t="inlineStr">
         <is>
-          <t>Rice halved. Curry container photographed near-empty - counted as eaten in full</t>
+          <t>Two extra boiled eggs on the side beyond the mess portion; roast masala visibly oily</t>
         </is>
       </c>
     </row>
@@ -3477,39 +3477,39 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>2 boiled eggs</t>
+          <t>Ghee rice (halved) + chicken curry + curd</t>
         </is>
       </c>
       <c r="D57" s="7" t="n">
-        <v>140</v>
+        <v>440</v>
       </c>
       <c r="E57" s="7" t="n">
-        <v>156</v>
+        <v>630</v>
       </c>
       <c r="F57" s="8">
         <f>AVERAGE(D57:E57)</f>
         <v/>
       </c>
       <c r="G57" s="9" t="n">
-        <v>12</v>
+        <v>21.5</v>
       </c>
       <c r="H57" s="9" t="n">
-        <v>13</v>
+        <v>29.5</v>
       </c>
       <c r="I57" s="10">
         <f>AVERAGE(G57:H57)</f>
         <v/>
       </c>
       <c r="J57" s="9" t="n">
-        <v>10</v>
+        <v>18.5</v>
       </c>
       <c r="K57" s="9" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="L57" s="10">
         <f>AVERAGE(J57:K57)</f>
@@ -3521,6 +3521,61 @@
         </is>
       </c>
       <c r="N57" s="6" t="inlineStr">
+        <is>
+          <t>Rice halved. Curry container photographed near-empty - counted as eaten in full</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>2 boiled eggs</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="E58" s="7" t="n">
+        <v>156</v>
+      </c>
+      <c r="F58" s="8">
+        <f>AVERAGE(D58:E58)</f>
+        <v/>
+      </c>
+      <c r="G58" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H58" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="I58" s="10">
+        <f>AVERAGE(G58:H58)</f>
+        <v/>
+      </c>
+      <c r="J58" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="K58" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="L58" s="10">
+        <f>AVERAGE(J58:K58)</f>
+        <v/>
+      </c>
+      <c r="M58" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N58" s="6" t="inlineStr">
         <is>
           <t>Took the eggs over the fourth scoop</t>
         </is>
@@ -3644,11 +3699,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3656,11 +3711,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3668,11 +3723,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3680,11 +3735,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A5,Meals!$M$5:$M$57,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3697,11 +3752,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3709,11 +3764,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3721,11 +3776,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3733,11 +3788,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A6,Meals!$M$5:$M$57,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3750,11 +3805,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3762,11 +3817,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3774,11 +3829,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3786,11 +3841,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A7,Meals!$M$5:$M$57,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3803,11 +3858,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3815,11 +3870,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3827,11 +3882,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3839,11 +3894,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A8,Meals!$M$5:$M$57,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3856,11 +3911,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3868,11 +3923,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3880,11 +3935,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3892,11 +3947,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A9,Meals!$M$5:$M$57,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3909,11 +3964,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3921,11 +3976,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3933,11 +3988,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3945,11 +4000,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A10,Meals!$M$5:$M$57,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3962,11 +4017,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3974,11 +4029,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3986,11 +4041,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3998,11 +4053,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A11,Meals!$M$5:$M$57,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4015,11 +4070,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4027,11 +4082,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4039,11 +4094,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4051,11 +4106,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A12,Meals!$M$5:$M$57,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4068,11 +4123,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4080,11 +4135,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4092,11 +4147,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4104,11 +4159,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A13,Meals!$M$5:$M$57,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4121,11 +4176,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$57,Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$57,Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4133,11 +4188,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$57,Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$57,Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4145,11 +4200,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$57,Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$57,Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4157,11 +4212,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$57,$A14,Meals!$M$5:$M$57,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">

</xml_diff>

<commit_message>
Close Day 10, log Day 11 breakfast, and correct the macro priority
Nine complete days average 2,154 kcal (on target), 108.2 g protein
(22 g under the floor) and 90.8 g fat.

Corrects several days of misplaced emphasis: 55 g of fat is a floor,
not a ceiling, so 91 g displaces carbohydrate rather than adding body
fat. The line that is actually wrong is protein, and the cause is the
closing whey scoops going unlogged three days running.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N58"/>
+  <dimension ref="A1:N59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3581,6 +3581,61 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="4" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Large restaurant dosa + sambar + red chutney (white coconut chutney skipped)</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="n">
+        <v>380</v>
+      </c>
+      <c r="E59" s="7" t="n">
+        <v>590</v>
+      </c>
+      <c r="F59" s="8">
+        <f>AVERAGE(D59:E59)</f>
+        <v/>
+      </c>
+      <c r="G59" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H59" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="I59" s="10">
+        <f>AVERAGE(G59:H59)</f>
+        <v/>
+      </c>
+      <c r="J59" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="K59" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="L59" s="10">
+        <f>AVERAGE(J59:K59)</f>
+        <v/>
+      </c>
+      <c r="M59" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N59" s="6" t="inlineStr">
+        <is>
+          <t>Sixth skip of the coconut chutney; eaten out rather than from the mess</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -3595,7 +3650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3699,11 +3754,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3711,11 +3766,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3723,11 +3778,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3735,11 +3790,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A5,Meals!$M$5:$M$58,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3752,11 +3807,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3764,11 +3819,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3776,11 +3831,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3788,11 +3843,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A6,Meals!$M$5:$M$58,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3805,11 +3860,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3817,11 +3872,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3829,11 +3884,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3841,11 +3896,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A7,Meals!$M$5:$M$58,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3858,11 +3913,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3870,11 +3925,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3882,11 +3937,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3894,11 +3949,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A8,Meals!$M$5:$M$58,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3911,11 +3966,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3923,11 +3978,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3935,11 +3990,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3947,11 +4002,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A9,Meals!$M$5:$M$58,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3964,11 +4019,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3976,11 +4031,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3988,11 +4043,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4000,11 +4055,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A10,Meals!$M$5:$M$58,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4017,11 +4072,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4029,11 +4084,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4041,11 +4096,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4053,11 +4108,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A11,Meals!$M$5:$M$58,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4070,11 +4125,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4082,11 +4137,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4094,11 +4149,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4106,11 +4161,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A12,Meals!$M$5:$M$58,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4123,11 +4178,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4135,11 +4190,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4147,11 +4202,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4159,11 +4214,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A13,Meals!$M$5:$M$58,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4176,11 +4231,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$58,Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$58,Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4188,11 +4243,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$58,Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$58,Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4200,11 +4255,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$58,Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$58,Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4212,15 +4267,68 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$58,$A14,Meals!$M$5:$M$58,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
         <f>D14-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B15" s="8">
+        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"logged")</f>
+        <v/>
+      </c>
+      <c r="C15" s="8">
+        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"logged")</f>
+        <v/>
+      </c>
+      <c r="D15" s="8">
+        <f>AVERAGE(B15:C15)</f>
+        <v/>
+      </c>
+      <c r="E15" s="10">
+        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"logged")</f>
+        <v/>
+      </c>
+      <c r="F15" s="10">
+        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"logged")</f>
+        <v/>
+      </c>
+      <c r="G15" s="10">
+        <f>AVERAGE(E15:F15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="10">
+        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"logged")</f>
+        <v/>
+      </c>
+      <c r="I15" s="10">
+        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"logged")</f>
+        <v/>
+      </c>
+      <c r="J15" s="10">
+        <f>AVERAGE(H15:I15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"logged")</f>
+        <v/>
+      </c>
+      <c r="L15" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"pending")</f>
+        <v/>
+      </c>
+      <c r="M15" s="19">
+        <f>D15-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -5115,7 +5223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5154,7 +5262,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$14)</f>
+        <f>COUNT(Daily!$A$5:$A$15)</f>
         <v/>
       </c>
     </row>
@@ -5165,7 +5273,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$14),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$15),0)</f>
         <v/>
       </c>
     </row>
@@ -5176,7 +5284,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$14),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$15),0)</f>
         <v/>
       </c>
     </row>
@@ -5187,7 +5295,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$14),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$15),0)</f>
         <v/>
       </c>
     </row>
@@ -5231,7 +5339,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$14,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$15,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -5242,7 +5350,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$14)</f>
+        <f>SUM(Daily!$L$5:$L$15)</f>
         <v/>
       </c>
     </row>
@@ -5293,19 +5401,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$14,"&gt;="&amp;$A17,Daily!$A$5:$A$14,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$15,"&gt;="&amp;$A17,Daily!$A$5:$A$15,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$14,Daily!$A$5:$A$14,"&gt;="&amp;$A17,Daily!$A$5:$A$14,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$15,Daily!$A$5:$A$15,"&gt;="&amp;$A17,Daily!$A$5:$A$15,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$14,Daily!$A$5:$A$14,"&gt;="&amp;$A17,Daily!$A$5:$A$14,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$15,Daily!$A$5:$A$15,"&gt;="&amp;$A17,Daily!$A$5:$A$15,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$14,Daily!$A$5:$A$14,"&gt;="&amp;$A17,Daily!$A$5:$A$14,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$15,Daily!$A$5:$A$15,"&gt;="&amp;$A17,Daily!$A$5:$A$15,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -5317,87 +5425,111 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$14,"&gt;="&amp;$A18,Daily!$A$5:$A$14,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$15,"&gt;="&amp;$A18,Daily!$A$5:$A$15,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$14,Daily!$A$5:$A$14,"&gt;="&amp;$A18,Daily!$A$5:$A$14,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$15,Daily!$A$5:$A$15,"&gt;="&amp;$A18,Daily!$A$5:$A$15,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$14,Daily!$A$5:$A$14,"&gt;="&amp;$A18,Daily!$A$5:$A$14,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$15,Daily!$A$5:$A$15,"&gt;="&amp;$A18,Daily!$A$5:$A$15,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$14,Daily!$A$5:$A$14,"&gt;="&amp;$A18,Daily!$A$5:$A$14,"&lt;="&amp;$B18),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="28" t="inlineStr">
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$15,Daily!$A$5:$A$15,"&gt;="&amp;$A18,Daily!$A$5:$A$15,"&lt;="&amp;$B18),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>46285</v>
+      </c>
+      <c r="C19" s="18">
+        <f>COUNTIFS(Daily!$A$5:$A$15,"&gt;="&amp;$A19,Daily!$A$5:$A$15,"&lt;="&amp;$B19)</f>
+        <v/>
+      </c>
+      <c r="D19" s="8">
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$15,Daily!$A$5:$A$15,"&gt;="&amp;$A19,Daily!$A$5:$A$15,"&lt;="&amp;$B19),0)</f>
+        <v/>
+      </c>
+      <c r="E19" s="10">
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$15,Daily!$A$5:$A$15,"&gt;="&amp;$A19,Daily!$A$5:$A$15,"&lt;="&amp;$B19),0)</f>
+        <v/>
+      </c>
+      <c r="F19" s="10">
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$15,Daily!$A$5:$A$15,"&gt;="&amp;$A19,Daily!$A$5:$A$15,"&lt;="&amp;$B19),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="28" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Month start</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Month end</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Days logged</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Avg cal/day (mid)</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Avg protein/day (mid, g)</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Avg fat/day (mid, g)</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
+    <row r="23">
+      <c r="A23" s="4" t="n">
         <v>46266</v>
       </c>
-      <c r="B22" s="4" t="n">
+      <c r="B23" s="4" t="n">
         <v>46295</v>
       </c>
-      <c r="C22" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$14,"&gt;="&amp;$A22,Daily!$A$5:$A$14,"&lt;="&amp;$B22)</f>
-        <v/>
-      </c>
-      <c r="D22" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$14,Daily!$A$5:$A$14,"&gt;="&amp;$A22,Daily!$A$5:$A$14,"&lt;="&amp;$B22),0)</f>
-        <v/>
-      </c>
-      <c r="E22" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$14,Daily!$A$5:$A$14,"&gt;="&amp;$A22,Daily!$A$5:$A$14,"&lt;="&amp;$B22),0)</f>
-        <v/>
-      </c>
-      <c r="F22" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$14,Daily!$A$5:$A$14,"&gt;="&amp;$A22,Daily!$A$5:$A$14,"&lt;="&amp;$B22),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="27" t="inlineStr">
+      <c r="C23" s="18">
+        <f>COUNTIFS(Daily!$A$5:$A$15,"&gt;="&amp;$A23,Daily!$A$5:$A$15,"&lt;="&amp;$B23)</f>
+        <v/>
+      </c>
+      <c r="D23" s="8">
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$15,Daily!$A$5:$A$15,"&gt;="&amp;$A23,Daily!$A$5:$A$15,"&lt;="&amp;$B23),0)</f>
+        <v/>
+      </c>
+      <c r="E23" s="10">
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$15,Daily!$A$5:$A$15,"&gt;="&amp;$A23,Daily!$A$5:$A$15,"&lt;="&amp;$B23),0)</f>
+        <v/>
+      </c>
+      <c r="F23" s="10">
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$15,Daily!$A$5:$A$15,"&gt;="&amp;$A23,Daily!$A$5:$A$15,"&lt;="&amp;$B23),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="27" t="inlineStr">
         <is>
           <t>Averages cover only the days present in the log; a part-logged day (today's dinner still to come) drags its average down.</t>
         </is>

</xml_diff>

<commit_message>
Log Day 11 lunch: lightest plate of the eleven days
457 kcal against the ~760 budgeted - rice halved, one fish piece, one
veg curry, and the four side containers still sealed and uncounted.

The light lunch leaves a 1,177 kcal evening, so the usual 3 scoops would
produce an 801 deficit at barely 130 g of protein. Lands on 3 scoops
plus 3 eggs instead.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N59"/>
+  <dimension ref="A1:N60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3633,6 +3633,61 @@
       <c r="N59" s="6" t="inlineStr">
         <is>
           <t>Sixth skip of the coconut chutney; eaten out rather than from the mess</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>Mess meals plate (rice halved) + 1 fried fish piece + 1 veg curry</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="n">
+        <v>365</v>
+      </c>
+      <c r="E60" s="7" t="n">
+        <v>550</v>
+      </c>
+      <c r="F60" s="8">
+        <f>AVERAGE(D60:E60)</f>
+        <v/>
+      </c>
+      <c r="G60" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="H60" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="I60" s="10">
+        <f>AVERAGE(G60:H60)</f>
+        <v/>
+      </c>
+      <c r="J60" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="K60" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="L60" s="10">
+        <f>AVERAGE(J60:K60)</f>
+        <v/>
+      </c>
+      <c r="M60" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N60" s="6" t="inlineStr">
+        <is>
+          <t>Plate only - four unopened side containers in the photo are not counted</t>
         </is>
       </c>
     </row>
@@ -3754,11 +3809,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3766,11 +3821,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3778,11 +3833,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3790,11 +3845,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A5,Meals!$M$5:$M$59,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3807,11 +3862,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3819,11 +3874,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3831,11 +3886,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3843,11 +3898,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A6,Meals!$M$5:$M$59,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3860,11 +3915,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3872,11 +3927,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3884,11 +3939,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3896,11 +3951,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A7,Meals!$M$5:$M$59,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3913,11 +3968,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3925,11 +3980,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3937,11 +3992,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3949,11 +4004,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A8,Meals!$M$5:$M$59,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3966,11 +4021,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3978,11 +4033,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3990,11 +4045,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4002,11 +4057,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A9,Meals!$M$5:$M$59,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4019,11 +4074,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4031,11 +4086,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4043,11 +4098,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4055,11 +4110,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A10,Meals!$M$5:$M$59,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4072,11 +4127,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4084,11 +4139,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4096,11 +4151,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4108,11 +4163,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A11,Meals!$M$5:$M$59,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4125,11 +4180,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4137,11 +4192,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4149,11 +4204,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4161,11 +4216,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A12,Meals!$M$5:$M$59,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4178,11 +4233,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4190,11 +4245,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4202,11 +4257,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4214,11 +4269,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A13,Meals!$M$5:$M$59,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4231,11 +4286,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4243,11 +4298,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4255,11 +4310,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4267,11 +4322,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A14,Meals!$M$5:$M$59,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -4284,11 +4339,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$59,Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$59,Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -4296,11 +4351,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$59,Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$59,Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4308,11 +4363,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$59,Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$59,Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -4320,11 +4375,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$59,$A15,Meals!$M$5:$M$59,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">

</xml_diff>

<commit_message>
Fold the four side containers into Day 11 lunch
Confirmed opened and eaten, adding ~300 kcal, ~10 g protein and ~19.5 g
fat. Lunch lands at 757 kcal - within 3 of the figure originally
budgeted for a halved meals plate, so the evening returns to the
standard 3 scoops and the extra eggs are no longer needed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -3647,34 +3647,34 @@
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate (rice halved) + 1 fried fish piece + 1 veg curry</t>
+          <t>Mess meals plate (rice halved) + 1 fried fish piece + veg curry, sambar, thin curry, white side, green side</t>
         </is>
       </c>
       <c r="D60" s="7" t="n">
-        <v>365</v>
+        <v>565</v>
       </c>
       <c r="E60" s="7" t="n">
-        <v>550</v>
+        <v>950</v>
       </c>
       <c r="F60" s="8">
         <f>AVERAGE(D60:E60)</f>
         <v/>
       </c>
       <c r="G60" s="9" t="n">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="H60" s="9" t="n">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="I60" s="10">
         <f>AVERAGE(G60:H60)</f>
         <v/>
       </c>
       <c r="J60" s="9" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="K60" s="9" t="n">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="L60" s="10">
         <f>AVERAGE(J60:K60)</f>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="N60" s="6" t="inlineStr">
         <is>
-          <t>Plate only - four unopened side containers in the photo are not counted</t>
+          <t>All four side containers opened and eaten - confirmed by the user</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Day 11 scoop 1
First logged whey scoop in four days. Two more to go for the standard
Monday shape.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N60"/>
+  <dimension ref="A1:N61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3688,6 +3688,61 @@
       <c r="N60" s="6" t="inlineStr">
         <is>
           <t>All four side containers opened and eaten - confirmed by the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1 whey scoop</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E61" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F61" s="8">
+        <f>AVERAGE(D61:E61)</f>
+        <v/>
+      </c>
+      <c r="G61" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H61" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I61" s="10">
+        <f>AVERAGE(G61:H61)</f>
+        <v/>
+      </c>
+      <c r="J61" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K61" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L61" s="10">
+        <f>AVERAGE(J61:K61)</f>
+        <v/>
+      </c>
+      <c r="M61" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N61" s="6" t="inlineStr">
+        <is>
+          <t>Scoop 1 of the 3 planned for today</t>
         </is>
       </c>
     </row>
@@ -3809,11 +3864,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3821,11 +3876,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3833,11 +3888,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3845,11 +3900,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A5,Meals!$M$5:$M$60,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3862,11 +3917,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3874,11 +3929,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3886,11 +3941,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3898,11 +3953,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A6,Meals!$M$5:$M$60,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3915,11 +3970,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3927,11 +3982,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3939,11 +3994,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3951,11 +4006,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A7,Meals!$M$5:$M$60,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3968,11 +4023,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3980,11 +4035,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3992,11 +4047,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4004,11 +4059,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A8,Meals!$M$5:$M$60,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4021,11 +4076,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4033,11 +4088,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4045,11 +4100,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4057,11 +4112,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A9,Meals!$M$5:$M$60,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4074,11 +4129,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4086,11 +4141,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4098,11 +4153,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4110,11 +4165,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A10,Meals!$M$5:$M$60,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4127,11 +4182,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4139,11 +4194,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4151,11 +4206,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4163,11 +4218,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A11,Meals!$M$5:$M$60,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4180,11 +4235,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4192,11 +4247,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4204,11 +4259,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4216,11 +4271,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A12,Meals!$M$5:$M$60,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4233,11 +4288,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4245,11 +4300,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4257,11 +4312,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4269,11 +4324,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A13,Meals!$M$5:$M$60,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4286,11 +4341,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4298,11 +4353,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4310,11 +4365,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4322,11 +4377,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A14,Meals!$M$5:$M$60,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -4339,11 +4394,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$60,Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$60,Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -4351,11 +4406,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$60,Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$60,Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4363,11 +4418,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$60,Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$60,Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -4375,11 +4430,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$60,$A15,Meals!$M$5:$M$60,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">

</xml_diff>

<commit_message>
Log Day 11 dinner: leftover half rice with chicken curry
The rice swap saved ~112 kcal over three chapati for only ~6 g of
protein, and the saving buys a scoop worth 22.5 g. Dinner came with
three or four chicken pieces rather than the usual two.

A green 330 ml can in the photo is unidentified and uncounted.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N61"/>
+  <dimension ref="A1:N62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3642,39 +3642,39 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate (rice halved) + 1 fried fish piece + veg curry, sambar, thin curry, white side, green side</t>
+          <t>Leftover half rice from lunch + chicken curry</t>
         </is>
       </c>
       <c r="D60" s="7" t="n">
-        <v>565</v>
+        <v>375</v>
       </c>
       <c r="E60" s="7" t="n">
-        <v>950</v>
+        <v>560</v>
       </c>
       <c r="F60" s="8">
         <f>AVERAGE(D60:E60)</f>
         <v/>
       </c>
       <c r="G60" s="9" t="n">
-        <v>22.5</v>
+        <v>20</v>
       </c>
       <c r="H60" s="9" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="I60" s="10">
         <f>AVERAGE(G60:H60)</f>
         <v/>
       </c>
       <c r="J60" s="9" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="K60" s="9" t="n">
-        <v>48</v>
+        <v>19</v>
       </c>
       <c r="L60" s="10">
         <f>AVERAGE(J60:K60)</f>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="N60" s="6" t="inlineStr">
         <is>
-          <t>All four side containers opened and eaten - confirmed by the user</t>
+          <t>Rice reused from the lunch container; green 330 ml can in the photo not identified and not counted</t>
         </is>
       </c>
     </row>
@@ -3697,39 +3697,39 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Black coffee + 1 whey scoop</t>
+          <t>Mess meals plate (rice halved) + 1 fried fish piece + veg curry, sambar, thin curry, white side, green side</t>
         </is>
       </c>
       <c r="D61" s="7" t="n">
-        <v>100</v>
+        <v>565</v>
       </c>
       <c r="E61" s="7" t="n">
-        <v>130</v>
+        <v>950</v>
       </c>
       <c r="F61" s="8">
         <f>AVERAGE(D61:E61)</f>
         <v/>
       </c>
       <c r="G61" s="9" t="n">
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="H61" s="9" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="I61" s="10">
         <f>AVERAGE(G61:H61)</f>
         <v/>
       </c>
       <c r="J61" s="9" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="K61" s="9" t="n">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="L61" s="10">
         <f>AVERAGE(J61:K61)</f>
@@ -3741,6 +3741,61 @@
         </is>
       </c>
       <c r="N61" s="6" t="inlineStr">
+        <is>
+          <t>All four side containers opened and eaten - confirmed by the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1 whey scoop</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E62" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F62" s="8">
+        <f>AVERAGE(D62:E62)</f>
+        <v/>
+      </c>
+      <c r="G62" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H62" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I62" s="10">
+        <f>AVERAGE(G62:H62)</f>
+        <v/>
+      </c>
+      <c r="J62" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K62" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L62" s="10">
+        <f>AVERAGE(J62:K62)</f>
+        <v/>
+      </c>
+      <c r="M62" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N62" s="6" t="inlineStr">
         <is>
           <t>Scoop 1 of the 3 planned for today</t>
         </is>
@@ -3864,11 +3919,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3876,11 +3931,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3888,11 +3943,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3900,11 +3955,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A5,Meals!$M$5:$M$61,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3917,11 +3972,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3929,11 +3984,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3941,11 +3996,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3953,11 +4008,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A6,Meals!$M$5:$M$61,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3970,11 +4025,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3982,11 +4037,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3994,11 +4049,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4006,11 +4061,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A7,Meals!$M$5:$M$61,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4023,11 +4078,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4035,11 +4090,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4047,11 +4102,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4059,11 +4114,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A8,Meals!$M$5:$M$61,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4076,11 +4131,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4088,11 +4143,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4100,11 +4155,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4112,11 +4167,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A9,Meals!$M$5:$M$61,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4129,11 +4184,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4141,11 +4196,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4153,11 +4208,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4165,11 +4220,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A10,Meals!$M$5:$M$61,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4182,11 +4237,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4194,11 +4249,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4206,11 +4261,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4218,11 +4273,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A11,Meals!$M$5:$M$61,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4235,11 +4290,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4247,11 +4302,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4259,11 +4314,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4271,11 +4326,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A12,Meals!$M$5:$M$61,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4288,11 +4343,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4300,11 +4355,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4312,11 +4367,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4324,11 +4379,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A13,Meals!$M$5:$M$61,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4341,11 +4396,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4353,11 +4408,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4365,11 +4420,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4377,11 +4432,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A14,Meals!$M$5:$M$61,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -4394,11 +4449,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$61,Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$61,Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -4406,11 +4461,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$61,Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$61,Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4418,11 +4473,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$61,Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$61,Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -4430,11 +4485,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$61,$A15,Meals!$M$5:$M$61,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">

</xml_diff>

<commit_message>
Close Day 11 and log Day 12 breakfast
Day 11 closes at 1,825 kcal - scoops 2 and 3 unconfirmed, making it the
largest deficit of the twelve at 87.25 g of protein.

Day 12 is Tuesday, the menu's protein desert: 54.5 g as served with no
meat at dinner. Lands on 4 scoops plus 2 eggs to reach 159.5 g on target.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N62"/>
+  <dimension ref="A1:N63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3801,6 +3801,61 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="4" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>Large restaurant dosa + sambar + red chutney (white chutney skipped)</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="n">
+        <v>380</v>
+      </c>
+      <c r="E63" s="7" t="n">
+        <v>590</v>
+      </c>
+      <c r="F63" s="8">
+        <f>AVERAGE(D63:E63)</f>
+        <v/>
+      </c>
+      <c r="G63" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H63" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="I63" s="10">
+        <f>AVERAGE(G63:H63)</f>
+        <v/>
+      </c>
+      <c r="J63" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="K63" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="L63" s="10">
+        <f>AVERAGE(J63:K63)</f>
+        <v/>
+      </c>
+      <c r="M63" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N63" s="6" t="inlineStr">
+        <is>
+          <t>Seventh skip of the white chutney; eaten out again</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -3815,7 +3870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3919,11 +3974,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3931,11 +3986,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3943,11 +3998,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3955,11 +4010,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A5,Meals!$M$5:$M$62,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3972,11 +4027,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3984,11 +4039,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3996,11 +4051,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4008,11 +4063,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A6,Meals!$M$5:$M$62,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4025,11 +4080,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4037,11 +4092,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4049,11 +4104,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4061,11 +4116,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A7,Meals!$M$5:$M$62,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4078,11 +4133,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4090,11 +4145,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4102,11 +4157,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4114,11 +4169,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A8,Meals!$M$5:$M$62,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4131,11 +4186,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4143,11 +4198,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4155,11 +4210,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4167,11 +4222,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A9,Meals!$M$5:$M$62,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4184,11 +4239,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4196,11 +4251,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4208,11 +4263,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4220,11 +4275,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A10,Meals!$M$5:$M$62,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4237,11 +4292,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4249,11 +4304,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4261,11 +4316,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4273,11 +4328,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A11,Meals!$M$5:$M$62,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4290,11 +4345,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4302,11 +4357,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4314,11 +4369,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4326,11 +4381,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A12,Meals!$M$5:$M$62,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4343,11 +4398,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4355,11 +4410,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4367,11 +4422,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4379,11 +4434,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A13,Meals!$M$5:$M$62,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4396,11 +4451,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4408,11 +4463,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4420,11 +4475,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4432,11 +4487,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A14,Meals!$M$5:$M$62,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -4449,11 +4504,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$62,Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$62,Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -4461,11 +4516,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$62,Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$62,Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4473,11 +4528,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$62,Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$62,Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -4485,15 +4540,68 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$62,$A15,Meals!$M$5:$M$62,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
         <f>D15-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B16" s="21">
+        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"logged")</f>
+        <v/>
+      </c>
+      <c r="C16" s="21">
+        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"logged")</f>
+        <v/>
+      </c>
+      <c r="D16" s="21">
+        <f>AVERAGE(B16:C16)</f>
+        <v/>
+      </c>
+      <c r="E16" s="22">
+        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"logged")</f>
+        <v/>
+      </c>
+      <c r="F16" s="22">
+        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"logged")</f>
+        <v/>
+      </c>
+      <c r="G16" s="22">
+        <f>AVERAGE(E16:F16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="22">
+        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"logged")</f>
+        <v/>
+      </c>
+      <c r="I16" s="22">
+        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"logged")</f>
+        <v/>
+      </c>
+      <c r="J16" s="22">
+        <f>AVERAGE(H16:I16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"logged")</f>
+        <v/>
+      </c>
+      <c r="L16" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"pending")</f>
+        <v/>
+      </c>
+      <c r="M16" s="23">
+        <f>D16-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -5427,7 +5535,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$15)</f>
+        <f>COUNT(Daily!$A$5:$A$16)</f>
         <v/>
       </c>
     </row>
@@ -5438,7 +5546,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$15),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$16),0)</f>
         <v/>
       </c>
     </row>
@@ -5449,7 +5557,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$15),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$16),0)</f>
         <v/>
       </c>
     </row>
@@ -5460,7 +5568,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$15),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$16),0)</f>
         <v/>
       </c>
     </row>
@@ -5504,7 +5612,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$15,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$16,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -5515,7 +5623,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$15)</f>
+        <f>SUM(Daily!$L$5:$L$16)</f>
         <v/>
       </c>
     </row>
@@ -5566,19 +5674,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$15,"&gt;="&amp;$A17,Daily!$A$5:$A$15,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$16,"&gt;="&amp;$A17,Daily!$A$5:$A$16,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$15,Daily!$A$5:$A$15,"&gt;="&amp;$A17,Daily!$A$5:$A$15,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$16,Daily!$A$5:$A$16,"&gt;="&amp;$A17,Daily!$A$5:$A$16,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$15,Daily!$A$5:$A$15,"&gt;="&amp;$A17,Daily!$A$5:$A$15,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$16,Daily!$A$5:$A$16,"&gt;="&amp;$A17,Daily!$A$5:$A$16,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$15,Daily!$A$5:$A$15,"&gt;="&amp;$A17,Daily!$A$5:$A$15,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$16,Daily!$A$5:$A$16,"&gt;="&amp;$A17,Daily!$A$5:$A$16,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -5590,19 +5698,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$15,"&gt;="&amp;$A18,Daily!$A$5:$A$15,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$16,"&gt;="&amp;$A18,Daily!$A$5:$A$16,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$15,Daily!$A$5:$A$15,"&gt;="&amp;$A18,Daily!$A$5:$A$15,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$16,Daily!$A$5:$A$16,"&gt;="&amp;$A18,Daily!$A$5:$A$16,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$15,Daily!$A$5:$A$15,"&gt;="&amp;$A18,Daily!$A$5:$A$15,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$16,Daily!$A$5:$A$16,"&gt;="&amp;$A18,Daily!$A$5:$A$16,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$15,Daily!$A$5:$A$15,"&gt;="&amp;$A18,Daily!$A$5:$A$15,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$16,Daily!$A$5:$A$16,"&gt;="&amp;$A18,Daily!$A$5:$A$16,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -5614,19 +5722,19 @@
         <v>46285</v>
       </c>
       <c r="C19" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$15,"&gt;="&amp;$A19,Daily!$A$5:$A$15,"&lt;="&amp;$B19)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$16,"&gt;="&amp;$A19,Daily!$A$5:$A$16,"&lt;="&amp;$B19)</f>
         <v/>
       </c>
       <c r="D19" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$15,Daily!$A$5:$A$15,"&gt;="&amp;$A19,Daily!$A$5:$A$15,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$16,Daily!$A$5:$A$16,"&gt;="&amp;$A19,Daily!$A$5:$A$16,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$15,Daily!$A$5:$A$15,"&gt;="&amp;$A19,Daily!$A$5:$A$15,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$16,Daily!$A$5:$A$16,"&gt;="&amp;$A19,Daily!$A$5:$A$16,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$15,Daily!$A$5:$A$15,"&gt;="&amp;$A19,Daily!$A$5:$A$15,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$16,Daily!$A$5:$A$16,"&gt;="&amp;$A19,Daily!$A$5:$A$16,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
     </row>
@@ -5677,19 +5785,19 @@
         <v>46295</v>
       </c>
       <c r="C23" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$15,"&gt;="&amp;$A23,Daily!$A$5:$A$15,"&lt;="&amp;$B23)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$16,"&gt;="&amp;$A23,Daily!$A$5:$A$16,"&lt;="&amp;$B23)</f>
         <v/>
       </c>
       <c r="D23" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$15,Daily!$A$5:$A$15,"&gt;="&amp;$A23,Daily!$A$5:$A$15,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$16,Daily!$A$5:$A$16,"&gt;="&amp;$A23,Daily!$A$5:$A$16,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$15,Daily!$A$5:$A$15,"&gt;="&amp;$A23,Daily!$A$5:$A$15,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$16,Daily!$A$5:$A$16,"&gt;="&amp;$A23,Daily!$A$5:$A$16,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$15,Daily!$A$5:$A$15,"&gt;="&amp;$A23,Daily!$A$5:$A$15,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$16,Daily!$A$5:$A$16,"&gt;="&amp;$A23,Daily!$A$5:$A$16,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Day 12 lunch and birthday cake
Chapati taken instead of Tuesday's ghee rice: 510 kcal against ~575 for
a halved rice plate, with more protein since rice carries almost none.
That saving plus four chicken pieces is what leaves room for the cake.

The day still lands 5 kcal under target on 3 scoops. The slice cost
protein rather than calories - 132.5 g instead of the 159.5 g planned.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N63"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3853,6 +3853,116 @@
       <c r="N63" s="6" t="inlineStr">
         <is>
           <t>Seventh skip of the white chutney; eaten out again</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>2 chapati + chicken curry with 4 chicken pieces</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="E64" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="F64" s="8">
+        <f>AVERAGE(D64:E64)</f>
+        <v/>
+      </c>
+      <c r="G64" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="H64" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I64" s="10">
+        <f>AVERAGE(G64:H64)</f>
+        <v/>
+      </c>
+      <c r="J64" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="K64" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="L64" s="10">
+        <f>AVERAGE(J64:K64)</f>
+        <v/>
+      </c>
+      <c r="M64" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N64" s="6" t="inlineStr">
+        <is>
+          <t>Chapati taken instead of the menu's ghee rice - cheaper and more protein</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>1 slice birthday cake</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="E65" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="F65" s="8">
+        <f>AVERAGE(D65:E65)</f>
+        <v/>
+      </c>
+      <c r="G65" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H65" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I65" s="10">
+        <f>AVERAGE(G65:H65)</f>
+        <v/>
+      </c>
+      <c r="J65" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="K65" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="L65" s="10">
+        <f>AVERAGE(J65:K65)</f>
+        <v/>
+      </c>
+      <c r="M65" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N65" s="6" t="inlineStr">
+        <is>
+          <t>33rd birthday</t>
         </is>
       </c>
     </row>
@@ -3974,11 +4084,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3986,11 +4096,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3998,11 +4108,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4010,11 +4120,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A5,Meals!$M$5:$M$63,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4027,11 +4137,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4039,11 +4149,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4051,11 +4161,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4063,11 +4173,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A6,Meals!$M$5:$M$63,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4080,11 +4190,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4092,11 +4202,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4104,11 +4214,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4116,11 +4226,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A7,Meals!$M$5:$M$63,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4133,11 +4243,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4145,11 +4255,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4157,11 +4267,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4169,11 +4279,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A8,Meals!$M$5:$M$63,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4186,11 +4296,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4198,11 +4308,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4210,11 +4320,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4222,11 +4332,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A9,Meals!$M$5:$M$63,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4239,11 +4349,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4251,11 +4361,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4263,11 +4373,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4275,11 +4385,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A10,Meals!$M$5:$M$63,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4292,11 +4402,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4304,11 +4414,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4316,11 +4426,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4328,11 +4438,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A11,Meals!$M$5:$M$63,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4345,11 +4455,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4357,11 +4467,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4369,11 +4479,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4381,11 +4491,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A12,Meals!$M$5:$M$63,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4398,11 +4508,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4410,11 +4520,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4422,11 +4532,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4434,11 +4544,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A13,Meals!$M$5:$M$63,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4451,11 +4561,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4463,11 +4573,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4475,11 +4585,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4487,11 +4597,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A14,Meals!$M$5:$M$63,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -4504,11 +4614,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -4516,11 +4626,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4528,11 +4638,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -4540,11 +4650,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A15,Meals!$M$5:$M$63,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -4557,11 +4667,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$63,Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$63,Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -4569,11 +4679,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$63,Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$63,Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -4581,11 +4691,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$63,Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$63,Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -4593,11 +4703,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$63,$A16,Meals!$M$5:$M$63,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">

</xml_diff>

<commit_message>
Log Day 12 dinner: half ghee rice, chicken curry and beef varattiyathu
Not the menu's meatless green peas - 53 g of protein from one meal, the
best dinner of the twelve days, and 410 kcal over what the morning plan
assumed.

The birthday still lands within 175 kcal of target with a 374 deficit,
on one closing scoop.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:N66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3862,39 +3862,39 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>2 chapati + chicken curry with 4 chicken pieces</t>
+          <t>Half ghee rice + chicken curry + 2 pieces beef varattiyathu + raita</t>
         </is>
       </c>
       <c r="D64" s="7" t="n">
-        <v>420</v>
+        <v>690</v>
       </c>
       <c r="E64" s="7" t="n">
-        <v>600</v>
+        <v>1030</v>
       </c>
       <c r="F64" s="8">
         <f>AVERAGE(D64:E64)</f>
         <v/>
       </c>
       <c r="G64" s="9" t="n">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H64" s="9" t="n">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="I64" s="10">
         <f>AVERAGE(G64:H64)</f>
         <v/>
       </c>
       <c r="J64" s="9" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="K64" s="9" t="n">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="L64" s="10">
         <f>AVERAGE(J64:K64)</f>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="N64" s="6" t="inlineStr">
         <is>
-          <t>Chapati taken instead of the menu's ghee rice - cheaper and more protein</t>
+          <t>Not the menu's green peas - chicken and beef both on the plate; best protein dinner of the twelve days</t>
         </is>
       </c>
     </row>
@@ -3917,39 +3917,39 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>1 slice birthday cake</t>
+          <t>2 chapati + chicken curry with 4 chicken pieces</t>
         </is>
       </c>
       <c r="D65" s="7" t="n">
-        <v>250</v>
+        <v>420</v>
       </c>
       <c r="E65" s="7" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="F65" s="8">
         <f>AVERAGE(D65:E65)</f>
         <v/>
       </c>
       <c r="G65" s="9" t="n">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="H65" s="9" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="I65" s="10">
         <f>AVERAGE(G65:H65)</f>
         <v/>
       </c>
       <c r="J65" s="9" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="K65" s="9" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="L65" s="10">
         <f>AVERAGE(J65:K65)</f>
@@ -3961,6 +3961,61 @@
         </is>
       </c>
       <c r="N65" s="6" t="inlineStr">
+        <is>
+          <t>Chapati taken instead of the menu's ghee rice - cheaper and more protein</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>1 slice birthday cake</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="E66" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="F66" s="8">
+        <f>AVERAGE(D66:E66)</f>
+        <v/>
+      </c>
+      <c r="G66" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H66" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I66" s="10">
+        <f>AVERAGE(G66:H66)</f>
+        <v/>
+      </c>
+      <c r="J66" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="K66" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="L66" s="10">
+        <f>AVERAGE(J66:K66)</f>
+        <v/>
+      </c>
+      <c r="M66" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N66" s="6" t="inlineStr">
         <is>
           <t>33rd birthday</t>
         </is>
@@ -4084,11 +4139,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4096,11 +4151,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4108,11 +4163,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4120,11 +4175,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A5,Meals!$M$5:$M$65,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4137,11 +4192,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4149,11 +4204,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4161,11 +4216,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4173,11 +4228,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A6,Meals!$M$5:$M$65,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4190,11 +4245,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4202,11 +4257,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4214,11 +4269,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4226,11 +4281,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A7,Meals!$M$5:$M$65,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4243,11 +4298,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4255,11 +4310,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4267,11 +4322,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4279,11 +4334,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A8,Meals!$M$5:$M$65,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4296,11 +4351,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4308,11 +4363,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4320,11 +4375,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4332,11 +4387,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A9,Meals!$M$5:$M$65,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4349,11 +4404,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4361,11 +4416,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4373,11 +4428,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4385,11 +4440,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A10,Meals!$M$5:$M$65,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4402,11 +4457,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4414,11 +4469,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4426,11 +4481,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4438,11 +4493,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A11,Meals!$M$5:$M$65,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4455,11 +4510,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4467,11 +4522,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4479,11 +4534,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4491,11 +4546,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A12,Meals!$M$5:$M$65,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4508,11 +4563,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4520,11 +4575,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4532,11 +4587,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4544,11 +4599,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A13,Meals!$M$5:$M$65,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4561,11 +4616,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4573,11 +4628,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4585,11 +4640,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4597,11 +4652,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A14,Meals!$M$5:$M$65,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -4614,11 +4669,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -4626,11 +4681,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4638,11 +4693,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -4650,11 +4705,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A15,Meals!$M$5:$M$65,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -4667,11 +4722,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$65,Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$65,Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -4679,11 +4734,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$65,Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$65,Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -4691,11 +4746,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$65,Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$65,Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -4703,11 +4758,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$65,$A16,Meals!$M$5:$M$65,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">

</xml_diff>

<commit_message>
Close Day 12 and log Day 13 breakfast with the second puttu pending
Day 12 closed within 60 kcal of target at a -489 deficit despite cake
and a beef dinner; the closing scoop was unconfirmed so protein stands
at 101 g.

Day 13 is Wednesday, a tight day. The second puttu piece is ~215 kcal
for ~4 g of protein - 1.9 g per 100 kcal, the worst rate logged - and
forces the day to miss either the target or the protein floor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N66"/>
+  <dimension ref="A1:N68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4021,6 +4021,116 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="4" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>1 puttu piece + kadala curry</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="n">
+        <v>380</v>
+      </c>
+      <c r="E67" s="7" t="n">
+        <v>550</v>
+      </c>
+      <c r="F67" s="8">
+        <f>AVERAGE(D67:E67)</f>
+        <v/>
+      </c>
+      <c r="G67" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="H67" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="I67" s="10">
+        <f>AVERAGE(G67:H67)</f>
+        <v/>
+      </c>
+      <c r="J67" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="K67" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="L67" s="10">
+        <f>AVERAGE(J67:K67)</f>
+        <v/>
+      </c>
+      <c r="M67" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N67" s="6" t="inlineStr">
+        <is>
+          <t>Eaten out at Grill Spot; the second puttu piece is pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
+        <is>
+          <t>2nd puttu piece</t>
+        </is>
+      </c>
+      <c r="D68" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="E68" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F68" s="15">
+        <f>AVERAGE(D68:E68)</f>
+        <v/>
+      </c>
+      <c r="G68" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="H68" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="I68" s="17">
+        <f>AVERAGE(G68:H68)</f>
+        <v/>
+      </c>
+      <c r="J68" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="K68" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="L68" s="17">
+        <f>AVERAGE(J68:K68)</f>
+        <v/>
+      </c>
+      <c r="M68" s="12" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N68" s="13" t="inlineStr">
+        <is>
+          <t>Asked about but not yet eaten</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -4035,7 +4145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4139,11 +4249,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4151,11 +4261,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4163,11 +4273,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4175,11 +4285,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A5,Meals!$M$5:$M$66,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4192,11 +4302,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4204,11 +4314,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4216,11 +4326,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4228,11 +4338,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A6,Meals!$M$5:$M$66,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4245,11 +4355,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4257,11 +4367,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4269,11 +4379,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4281,11 +4391,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A7,Meals!$M$5:$M$66,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4298,11 +4408,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4310,11 +4420,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4322,11 +4432,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4334,11 +4444,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A8,Meals!$M$5:$M$66,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4351,11 +4461,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4363,11 +4473,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4375,11 +4485,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4387,11 +4497,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A9,Meals!$M$5:$M$66,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4404,11 +4514,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4416,11 +4526,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4428,11 +4538,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4440,11 +4550,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A10,Meals!$M$5:$M$66,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4457,11 +4567,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4469,11 +4579,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4481,11 +4591,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4493,11 +4603,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A11,Meals!$M$5:$M$66,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4510,11 +4620,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4522,11 +4632,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4534,11 +4644,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4546,11 +4656,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A12,Meals!$M$5:$M$66,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4563,11 +4673,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4575,11 +4685,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4587,11 +4697,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4599,11 +4709,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A13,Meals!$M$5:$M$66,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4616,11 +4726,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4628,11 +4738,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4640,11 +4750,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4652,11 +4762,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A14,Meals!$M$5:$M$66,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -4669,11 +4779,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -4681,11 +4791,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4693,11 +4803,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -4705,11 +4815,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A15,Meals!$M$5:$M$66,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -4722,11 +4832,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$66,Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$66,Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -4734,11 +4844,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$66,Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$66,Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -4746,11 +4856,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$66,Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$66,Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -4758,15 +4868,68 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$66,$A16,Meals!$M$5:$M$66,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
         <f>D16-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B17" s="8">
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <v/>
+      </c>
+      <c r="C17" s="8">
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <v/>
+      </c>
+      <c r="D17" s="8">
+        <f>AVERAGE(B17:C17)</f>
+        <v/>
+      </c>
+      <c r="E17" s="10">
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <v/>
+      </c>
+      <c r="F17" s="10">
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <v/>
+      </c>
+      <c r="G17" s="10">
+        <f>AVERAGE(E17:F17)</f>
+        <v/>
+      </c>
+      <c r="H17" s="10">
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <v/>
+      </c>
+      <c r="I17" s="10">
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <v/>
+      </c>
+      <c r="J17" s="10">
+        <f>AVERAGE(H17:I17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <v/>
+      </c>
+      <c r="L17" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"pending")</f>
+        <v/>
+      </c>
+      <c r="M17" s="19">
+        <f>D17-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -5700,7 +5863,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$16)</f>
+        <f>COUNT(Daily!$A$5:$A$17)</f>
         <v/>
       </c>
     </row>
@@ -5711,7 +5874,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$16),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$17),0)</f>
         <v/>
       </c>
     </row>
@@ -5722,7 +5885,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$16),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$17),0)</f>
         <v/>
       </c>
     </row>
@@ -5733,7 +5896,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$16),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$17),0)</f>
         <v/>
       </c>
     </row>
@@ -5777,7 +5940,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$16,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$17,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -5788,7 +5951,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$16)</f>
+        <f>SUM(Daily!$L$5:$L$17)</f>
         <v/>
       </c>
     </row>
@@ -5839,19 +6002,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$16,"&gt;="&amp;$A17,Daily!$A$5:$A$16,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$17,"&gt;="&amp;$A17,Daily!$A$5:$A$17,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$16,Daily!$A$5:$A$16,"&gt;="&amp;$A17,Daily!$A$5:$A$16,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$17,Daily!$A$5:$A$17,"&gt;="&amp;$A17,Daily!$A$5:$A$17,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$16,Daily!$A$5:$A$16,"&gt;="&amp;$A17,Daily!$A$5:$A$16,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$17,Daily!$A$5:$A$17,"&gt;="&amp;$A17,Daily!$A$5:$A$17,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$16,Daily!$A$5:$A$16,"&gt;="&amp;$A17,Daily!$A$5:$A$16,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$17,Daily!$A$5:$A$17,"&gt;="&amp;$A17,Daily!$A$5:$A$17,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -5863,19 +6026,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$16,"&gt;="&amp;$A18,Daily!$A$5:$A$16,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$17,"&gt;="&amp;$A18,Daily!$A$5:$A$17,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$16,Daily!$A$5:$A$16,"&gt;="&amp;$A18,Daily!$A$5:$A$16,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$17,Daily!$A$5:$A$17,"&gt;="&amp;$A18,Daily!$A$5:$A$17,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$16,Daily!$A$5:$A$16,"&gt;="&amp;$A18,Daily!$A$5:$A$16,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$17,Daily!$A$5:$A$17,"&gt;="&amp;$A18,Daily!$A$5:$A$17,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$16,Daily!$A$5:$A$16,"&gt;="&amp;$A18,Daily!$A$5:$A$16,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$17,Daily!$A$5:$A$17,"&gt;="&amp;$A18,Daily!$A$5:$A$17,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -5887,19 +6050,19 @@
         <v>46285</v>
       </c>
       <c r="C19" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$16,"&gt;="&amp;$A19,Daily!$A$5:$A$16,"&lt;="&amp;$B19)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$17,"&gt;="&amp;$A19,Daily!$A$5:$A$17,"&lt;="&amp;$B19)</f>
         <v/>
       </c>
       <c r="D19" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$16,Daily!$A$5:$A$16,"&gt;="&amp;$A19,Daily!$A$5:$A$16,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$17,Daily!$A$5:$A$17,"&gt;="&amp;$A19,Daily!$A$5:$A$17,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$16,Daily!$A$5:$A$16,"&gt;="&amp;$A19,Daily!$A$5:$A$16,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$17,Daily!$A$5:$A$17,"&gt;="&amp;$A19,Daily!$A$5:$A$17,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$16,Daily!$A$5:$A$16,"&gt;="&amp;$A19,Daily!$A$5:$A$16,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$17,Daily!$A$5:$A$17,"&gt;="&amp;$A19,Daily!$A$5:$A$17,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
     </row>
@@ -5950,19 +6113,19 @@
         <v>46295</v>
       </c>
       <c r="C23" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$16,"&gt;="&amp;$A23,Daily!$A$5:$A$16,"&lt;="&amp;$B23)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$17,"&gt;="&amp;$A23,Daily!$A$5:$A$17,"&lt;="&amp;$B23)</f>
         <v/>
       </c>
       <c r="D23" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$16,Daily!$A$5:$A$16,"&gt;="&amp;$A23,Daily!$A$5:$A$16,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$17,Daily!$A$5:$A$17,"&gt;="&amp;$A23,Daily!$A$5:$A$17,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$16,Daily!$A$5:$A$16,"&gt;="&amp;$A23,Daily!$A$5:$A$16,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$17,Daily!$A$5:$A$17,"&gt;="&amp;$A23,Daily!$A$5:$A$17,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$16,Daily!$A$5:$A$16,"&gt;="&amp;$A23,Daily!$A$5:$A$16,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$17,Daily!$A$5:$A$17,"&gt;="&amp;$A23,Daily!$A$5:$A$17,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Confirm both puttu pieces eaten and spend Wednesday's second cut
Breakfast lands at 680 kcal. Two small cuts - leaving the lunch gravies
and taking one chapati instead of two at dinner - put the day back at
2,150 and 141 g of protein, the same place one piece would have.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N68"/>
+  <dimension ref="A1:N67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4032,34 +4032,34 @@
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>1 puttu piece + kadala curry</t>
+          <t>2 puttu pieces + kadala curry</t>
         </is>
       </c>
       <c r="D67" s="7" t="n">
-        <v>380</v>
+        <v>560</v>
       </c>
       <c r="E67" s="7" t="n">
-        <v>550</v>
+        <v>800</v>
       </c>
       <c r="F67" s="8">
         <f>AVERAGE(D67:E67)</f>
         <v/>
       </c>
       <c r="G67" s="9" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H67" s="9" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I67" s="10">
         <f>AVERAGE(G67:H67)</f>
         <v/>
       </c>
       <c r="J67" s="9" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="K67" s="9" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="L67" s="10">
         <f>AVERAGE(J67:K67)</f>
@@ -4072,62 +4072,7 @@
       </c>
       <c r="N67" s="6" t="inlineStr">
         <is>
-          <t>Eaten out at Grill Spot; the second puttu piece is pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="11" t="n">
-        <v>46281</v>
-      </c>
-      <c r="B68" s="12" t="inlineStr">
-        <is>
-          <t>Breakfast</t>
-        </is>
-      </c>
-      <c r="C68" s="13" t="inlineStr">
-        <is>
-          <t>2nd puttu piece</t>
-        </is>
-      </c>
-      <c r="D68" s="14" t="n">
-        <v>180</v>
-      </c>
-      <c r="E68" s="14" t="n">
-        <v>250</v>
-      </c>
-      <c r="F68" s="15">
-        <f>AVERAGE(D68:E68)</f>
-        <v/>
-      </c>
-      <c r="G68" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="H68" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="I68" s="17">
-        <f>AVERAGE(G68:H68)</f>
-        <v/>
-      </c>
-      <c r="J68" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="K68" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="L68" s="17">
-        <f>AVERAGE(J68:K68)</f>
-        <v/>
-      </c>
-      <c r="M68" s="12" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N68" s="13" t="inlineStr">
-        <is>
-          <t>Asked about but not yet eaten</t>
+          <t>Eaten out at Grill Spot; both pieces confirmed eaten</t>
         </is>
       </c>
     </row>
@@ -4249,11 +4194,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4261,11 +4206,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4273,11 +4218,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4285,11 +4230,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4302,11 +4247,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4314,11 +4259,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4326,11 +4271,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4338,11 +4283,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4355,11 +4300,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4367,11 +4312,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4379,11 +4324,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4391,11 +4336,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4408,11 +4353,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4420,11 +4365,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4432,11 +4377,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4444,11 +4389,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4461,11 +4406,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4473,11 +4418,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4485,11 +4430,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4497,11 +4442,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4514,11 +4459,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4526,11 +4471,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4538,11 +4483,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4550,11 +4495,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4567,11 +4512,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4579,11 +4524,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4591,11 +4536,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4603,11 +4548,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4620,11 +4565,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4632,11 +4577,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4644,11 +4589,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4656,11 +4601,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4673,11 +4618,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4685,11 +4630,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4697,11 +4642,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4709,11 +4654,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4726,11 +4671,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4738,11 +4683,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4750,11 +4695,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4762,11 +4707,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -4779,11 +4724,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -4791,11 +4736,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4803,11 +4748,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -4815,11 +4760,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -4832,11 +4777,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -4844,11 +4789,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -4856,11 +4801,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -4868,11 +4813,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -4885,11 +4830,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -4897,11 +4842,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -4909,11 +4854,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -4921,11 +4866,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">

</xml_diff>

<commit_message>
Log omega-3 and vitamin D3 capsules on Day 13
Together ~15 kcal, below the resolution of the other estimates.

Adds a note on the D3: 50,000 IU is a weekly dose strength, not daily,
and the 12-capsule bottle matches a 12-week once-weekly course. Also
notes that 1000 mg of fish oil is only ~300 mg of actual EPA+DHA.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N67"/>
+  <dimension ref="A1:N68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4073,6 +4073,61 @@
       <c r="N67" s="6" t="inlineStr">
         <is>
           <t>Eaten out at Grill Spot; both pieces confirmed eaten</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Supplement</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>1 omega-3 fish oil 1000 mg + 1 vitamin D3 50000 IU capsule</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E68" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F68" s="8">
+        <f>AVERAGE(D68:E68)</f>
+        <v/>
+      </c>
+      <c r="G68" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="10">
+        <f>AVERAGE(G68:H68)</f>
+        <v/>
+      </c>
+      <c r="J68" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K68" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="L68" s="10">
+        <f>AVERAGE(J68:K68)</f>
+        <v/>
+      </c>
+      <c r="M68" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N68" s="6" t="inlineStr">
+        <is>
+          <t>Negligible calories; D3 50000 IU is a weekly-dose strength</t>
         </is>
       </c>
     </row>
@@ -4194,11 +4249,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4206,11 +4261,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4218,11 +4273,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4230,11 +4285,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A5,Meals!$M$5:$M$67,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4247,11 +4302,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4259,11 +4314,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4271,11 +4326,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4283,11 +4338,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A6,Meals!$M$5:$M$67,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4300,11 +4355,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4312,11 +4367,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4324,11 +4379,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4336,11 +4391,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A7,Meals!$M$5:$M$67,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4353,11 +4408,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4365,11 +4420,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4377,11 +4432,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4389,11 +4444,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A8,Meals!$M$5:$M$67,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4406,11 +4461,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4418,11 +4473,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4430,11 +4485,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4442,11 +4497,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A9,Meals!$M$5:$M$67,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4459,11 +4514,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4471,11 +4526,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4483,11 +4538,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4495,11 +4550,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A10,Meals!$M$5:$M$67,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4512,11 +4567,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4524,11 +4579,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4536,11 +4591,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4548,11 +4603,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A11,Meals!$M$5:$M$67,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4565,11 +4620,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4577,11 +4632,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4589,11 +4644,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4601,11 +4656,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A12,Meals!$M$5:$M$67,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4618,11 +4673,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4630,11 +4685,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4642,11 +4697,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4654,11 +4709,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A13,Meals!$M$5:$M$67,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4671,11 +4726,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4683,11 +4738,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4695,11 +4750,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4707,11 +4762,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A14,Meals!$M$5:$M$67,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -4724,11 +4779,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -4736,11 +4791,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4748,11 +4803,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -4760,11 +4815,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A15,Meals!$M$5:$M$67,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -4777,11 +4832,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -4789,11 +4844,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -4801,11 +4856,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -4813,11 +4868,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A16,Meals!$M$5:$M$67,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -4830,11 +4885,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$67,Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$67,Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -4842,11 +4897,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$67,Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$67,Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -4854,11 +4909,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$67,Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$67,Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -4866,11 +4921,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$67,$A17,Meals!$M$5:$M$67,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6588,7 +6643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -7974,6 +8029,60 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>Fish oil capsule (1000 mg)</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C56" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="D56" s="8">
+        <f>AVERAGE(B56:C56)</f>
+        <v/>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>1 g of oil. 1000 mg fish oil is typically only ~300 mg EPA+DHA</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>Vitamin D3 softgel (50000 IU)</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C57" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D57" s="8">
+        <f>AVERAGE(B57:C57)</f>
+        <v/>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>Oil-base softgel. 50000 IU is a weekly or fortnightly dose strength - not daily</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Log Day 13 lunch plate; four side containers held pending
Corrects this morning's costing of "leave the gravies" from ~100 kcal to
~300, measured from yesterday's four containers. Skipping them more than
covers the second puttu piece: the day lands at 2,103 and 154 g of
protein on 4 scoops, better than the pre-puttu plan.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N68"/>
+  <dimension ref="A1:N70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4082,39 +4082,39 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Supplement</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>1 omega-3 fish oil 1000 mg + 1 vitamin D3 50000 IU capsule</t>
+          <t>Mess meals plate (rice halved) + 1 fried fish + sambar/veg curry on the plate</t>
         </is>
       </c>
       <c r="D68" s="7" t="n">
-        <v>10</v>
+        <v>385</v>
       </c>
       <c r="E68" s="7" t="n">
-        <v>20</v>
+        <v>580</v>
       </c>
       <c r="F68" s="8">
         <f>AVERAGE(D68:E68)</f>
         <v/>
       </c>
       <c r="G68" s="9" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="H68" s="9" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="I68" s="10">
         <f>AVERAGE(G68:H68)</f>
         <v/>
       </c>
       <c r="J68" s="9" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="K68" s="9" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="L68" s="10">
         <f>AVERAGE(J68:K68)</f>
@@ -4126,6 +4126,116 @@
         </is>
       </c>
       <c r="N68" s="6" t="inlineStr">
+        <is>
+          <t>Plate only</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>4 side containers</t>
+        </is>
+      </c>
+      <c r="D69" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="E69" s="14" t="n">
+        <v>400</v>
+      </c>
+      <c r="F69" s="15">
+        <f>AVERAGE(D69:E69)</f>
+        <v/>
+      </c>
+      <c r="G69" s="16" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H69" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="I69" s="17">
+        <f>AVERAGE(G69:H69)</f>
+        <v/>
+      </c>
+      <c r="J69" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="K69" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="L69" s="17">
+        <f>AVERAGE(J69:K69)</f>
+        <v/>
+      </c>
+      <c r="M69" s="12" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N69" s="13" t="inlineStr">
+        <is>
+          <t>Cannot tell from the photo whether they were eaten - today's plan turns on this</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Supplement</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>1 omega-3 fish oil 1000 mg + 1 vitamin D3 50000 IU capsule</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E70" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F70" s="8">
+        <f>AVERAGE(D70:E70)</f>
+        <v/>
+      </c>
+      <c r="G70" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" s="10">
+        <f>AVERAGE(G70:H70)</f>
+        <v/>
+      </c>
+      <c r="J70" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K70" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="L70" s="10">
+        <f>AVERAGE(J70:K70)</f>
+        <v/>
+      </c>
+      <c r="M70" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N70" s="6" t="inlineStr">
         <is>
           <t>Negligible calories; D3 50000 IU is a weekly-dose strength</t>
         </is>
@@ -4249,11 +4359,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4261,11 +4371,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4273,11 +4383,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4285,11 +4395,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A5,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4302,11 +4412,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4314,11 +4424,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4326,11 +4436,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4338,11 +4448,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A6,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4355,11 +4465,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4367,11 +4477,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4379,11 +4489,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4391,11 +4501,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A7,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4408,11 +4518,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4420,11 +4530,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4432,11 +4542,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4444,11 +4554,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A8,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4461,11 +4571,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4473,11 +4583,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4485,11 +4595,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4497,11 +4607,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A9,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4514,11 +4624,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4526,11 +4636,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4538,11 +4648,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4550,11 +4660,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A10,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4567,11 +4677,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4579,11 +4689,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4591,11 +4701,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4603,11 +4713,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A11,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4620,11 +4730,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4632,11 +4742,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4644,11 +4754,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4656,11 +4766,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A12,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4673,11 +4783,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4685,11 +4795,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4697,11 +4807,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4709,11 +4819,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A13,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4726,11 +4836,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4738,11 +4848,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4750,11 +4860,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4762,11 +4872,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A14,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -4779,11 +4889,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -4791,11 +4901,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4803,11 +4913,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -4815,11 +4925,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A15,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -4832,11 +4942,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -4844,11 +4954,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -4856,11 +4966,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -4868,11 +4978,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A16,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -4885,11 +4995,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -4897,11 +5007,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -4909,11 +5019,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$68,Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -4921,11 +5031,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$68,$A17,Meals!$M$5:$M$68,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">

</xml_diff>

<commit_message>
Confirm Day 13 sides eaten; they came in ~70 kcal above estimate
The plated photo settles the pending row. This set carried a large
coconut chammanthi dollop and a battered fried item rather than four
thin gravies, so ~370 kcal rather than ~300.

The day is ~285 kcal above the morning plan and the chapati cut is
already spent, so the evening choice is between protein and bread at
identical calories.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -4132,57 +4132,57 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="11" t="n">
+      <c r="A69" s="4" t="n">
         <v>46281</v>
       </c>
-      <c r="B69" s="12" t="inlineStr">
+      <c r="B69" s="5" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="C69" s="13" t="inlineStr">
-        <is>
-          <t>4 side containers</t>
-        </is>
-      </c>
-      <c r="D69" s="14" t="n">
-        <v>200</v>
-      </c>
-      <c r="E69" s="14" t="n">
-        <v>400</v>
-      </c>
-      <c r="F69" s="15">
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>Side containers onto the plate: cabbage-carrot thoran, battered fried pieces, coconut chammanthi</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="n">
+        <v>270</v>
+      </c>
+      <c r="E69" s="7" t="n">
+        <v>470</v>
+      </c>
+      <c r="F69" s="8">
         <f>AVERAGE(D69:E69)</f>
         <v/>
       </c>
-      <c r="G69" s="16" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="H69" s="16" t="n">
-        <v>13</v>
-      </c>
-      <c r="I69" s="17">
+      <c r="G69" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="H69" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="I69" s="10">
         <f>AVERAGE(G69:H69)</f>
         <v/>
       </c>
-      <c r="J69" s="16" t="n">
-        <v>11</v>
-      </c>
-      <c r="K69" s="16" t="n">
-        <v>28</v>
-      </c>
-      <c r="L69" s="17">
+      <c r="J69" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="K69" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="L69" s="10">
         <f>AVERAGE(J69:K69)</f>
         <v/>
       </c>
-      <c r="M69" s="12" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N69" s="13" t="inlineStr">
-        <is>
-          <t>Cannot tell from the photo whether they were eaten - today's plan turns on this</t>
+      <c r="M69" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N69" s="6" t="inlineStr">
+        <is>
+          <t>Confirmed by the plated photo - higher than the 200-400 assumed because of the large chammanthi dollop and a fried item</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Day 13 dinner and close on 2 scoops with skimmed milk
Leftover half rice rather than a chapati. The day sits at 2,015 kcal and
73.5 g of protein before scoops.

Two scoops with the last in skimmed milk reaches 127 g - the first
evening in five where the plan actually hits the floor. The last four
complete days ran -671, -733, -844 and -489, all larger than designed
and three of them at 85-90 g of protein.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N70"/>
+  <dimension ref="A1:N71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4082,39 +4082,39 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate (rice halved) + 1 fried fish + sambar/veg curry on the plate</t>
+          <t>Leftover half rice from lunch + chicken curry</t>
         </is>
       </c>
       <c r="D68" s="7" t="n">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="E68" s="7" t="n">
-        <v>580</v>
+        <v>560</v>
       </c>
       <c r="F68" s="8">
         <f>AVERAGE(D68:E68)</f>
         <v/>
       </c>
       <c r="G68" s="9" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="H68" s="9" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="I68" s="10">
         <f>AVERAGE(G68:H68)</f>
         <v/>
       </c>
       <c r="J68" s="9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K68" s="9" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L68" s="10">
         <f>AVERAGE(J68:K68)</f>
@@ -4127,7 +4127,7 @@
       </c>
       <c r="N68" s="6" t="inlineStr">
         <is>
-          <t>Plate only</t>
+          <t>Rice reused from the lunch container; no chapati</t>
         </is>
       </c>
     </row>
@@ -4142,34 +4142,34 @@
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>Side containers onto the plate: cabbage-carrot thoran, battered fried pieces, coconut chammanthi</t>
+          <t>Mess meals plate (rice halved) + 1 fried fish + sambar/veg curry on the plate</t>
         </is>
       </c>
       <c r="D69" s="7" t="n">
-        <v>270</v>
+        <v>385</v>
       </c>
       <c r="E69" s="7" t="n">
-        <v>470</v>
+        <v>580</v>
       </c>
       <c r="F69" s="8">
         <f>AVERAGE(D69:E69)</f>
         <v/>
       </c>
       <c r="G69" s="9" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="H69" s="9" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="I69" s="10">
         <f>AVERAGE(G69:H69)</f>
         <v/>
       </c>
       <c r="J69" s="9" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="K69" s="9" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="L69" s="10">
         <f>AVERAGE(J69:K69)</f>
@@ -4182,7 +4182,7 @@
       </c>
       <c r="N69" s="6" t="inlineStr">
         <is>
-          <t>Confirmed by the plated photo - higher than the 200-400 assumed because of the large chammanthi dollop and a fried item</t>
+          <t>Plate only</t>
         </is>
       </c>
     </row>
@@ -4192,39 +4192,39 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Supplement</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>1 omega-3 fish oil 1000 mg + 1 vitamin D3 50000 IU capsule</t>
+          <t>Side containers onto the plate: cabbage-carrot thoran, battered fried pieces, coconut chammanthi</t>
         </is>
       </c>
       <c r="D70" s="7" t="n">
-        <v>10</v>
+        <v>270</v>
       </c>
       <c r="E70" s="7" t="n">
-        <v>20</v>
+        <v>470</v>
       </c>
       <c r="F70" s="8">
         <f>AVERAGE(D70:E70)</f>
         <v/>
       </c>
       <c r="G70" s="9" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H70" s="9" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="I70" s="10">
         <f>AVERAGE(G70:H70)</f>
         <v/>
       </c>
       <c r="J70" s="9" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="K70" s="9" t="n">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="L70" s="10">
         <f>AVERAGE(J70:K70)</f>
@@ -4236,6 +4236,61 @@
         </is>
       </c>
       <c r="N70" s="6" t="inlineStr">
+        <is>
+          <t>Confirmed by the plated photo - higher than the 200-400 assumed because of the large chammanthi dollop and a fried item</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>Supplement</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>1 omega-3 fish oil 1000 mg + 1 vitamin D3 50000 IU capsule</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E71" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F71" s="8">
+        <f>AVERAGE(D71:E71)</f>
+        <v/>
+      </c>
+      <c r="G71" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" s="10">
+        <f>AVERAGE(G71:H71)</f>
+        <v/>
+      </c>
+      <c r="J71" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K71" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="L71" s="10">
+        <f>AVERAGE(J71:K71)</f>
+        <v/>
+      </c>
+      <c r="M71" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N71" s="6" t="inlineStr">
         <is>
           <t>Negligible calories; D3 50000 IU is a weekly-dose strength</t>
         </is>
@@ -4359,11 +4414,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4371,11 +4426,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4383,11 +4438,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4395,11 +4450,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A5,Meals!$M$5:$M$70,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4412,11 +4467,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4424,11 +4479,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4436,11 +4491,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4448,11 +4503,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A6,Meals!$M$5:$M$70,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4465,11 +4520,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4477,11 +4532,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4489,11 +4544,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4501,11 +4556,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A7,Meals!$M$5:$M$70,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4518,11 +4573,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4530,11 +4585,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4542,11 +4597,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4554,11 +4609,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A8,Meals!$M$5:$M$70,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4571,11 +4626,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4583,11 +4638,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4595,11 +4650,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4607,11 +4662,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A9,Meals!$M$5:$M$70,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4624,11 +4679,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4636,11 +4691,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4648,11 +4703,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4660,11 +4715,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A10,Meals!$M$5:$M$70,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4677,11 +4732,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4689,11 +4744,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4701,11 +4756,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4713,11 +4768,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A11,Meals!$M$5:$M$70,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4730,11 +4785,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4742,11 +4797,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4754,11 +4809,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4766,11 +4821,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A12,Meals!$M$5:$M$70,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4783,11 +4838,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4795,11 +4850,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4807,11 +4862,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4819,11 +4874,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A13,Meals!$M$5:$M$70,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4836,11 +4891,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4848,11 +4903,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4860,11 +4915,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4872,11 +4927,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A14,Meals!$M$5:$M$70,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -4889,11 +4944,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -4901,11 +4956,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4913,11 +4968,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -4925,11 +4980,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A15,Meals!$M$5:$M$70,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -4942,11 +4997,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -4954,11 +5009,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -4966,11 +5021,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -4978,11 +5033,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A16,Meals!$M$5:$M$70,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -4995,11 +5050,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$70,Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$70,Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5007,11 +5062,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$70,Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$70,Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5019,11 +5074,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$70,Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$70,Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5031,11 +5086,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$70,$A17,Meals!$M$5:$M$70,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">

</xml_diff>

<commit_message>
Add boneless charcoal grilled chicken to the reference table
13 g of protein per 100 kcal - the best whole-food protein source of
anything logged, against whey's 19.6, a boiled egg's 8.5 and the mess
plate's 3.7. A 1 kg order is a 3-4 person portion.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -6808,7 +6808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -8248,6 +8248,60 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Boneless charcoal grilled chicken (100 g cooked)</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="n">
+        <v>190</v>
+      </c>
+      <c r="C58" s="7" t="n">
+        <v>230</v>
+      </c>
+      <c r="D58" s="8">
+        <f>AVERAGE(B58:C58)</f>
+        <v/>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>~27-30 g</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>13 g protein per 100 kcal - the best whole-food protein source on any menu logged</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>Boneless charcoal grilled chicken (1 kg order)</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="n">
+        <v>1400</v>
+      </c>
+      <c r="C59" s="7" t="n">
+        <v>2300</v>
+      </c>
+      <c r="D59" s="8">
+        <f>AVERAGE(B59:C59)</f>
+        <v/>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>~190-300 g</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>A 3-4 person portion. Range depends on whether 1 kg is the raw or the served weight</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Close Day 13 at 141 g of protein, the highest of the thirteen days
Three scoops in water rather than two with milk. The day lands at 2,360
kcal and a 309 deficit - the softest of the twelve read alone, but a
correction read in sequence after four days of -671, -733, -844 and -489
at 85-101 g of protein.

Twelve complete days now average 2,146 kcal, 108.5 g protein, a 523
deficit, 0.48 kg/week.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N71"/>
+  <dimension ref="A1:N72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4247,39 +4247,39 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>Supplement</t>
+          <t>Snack</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>1 omega-3 fish oil 1000 mg + 1 vitamin D3 50000 IU capsule</t>
+          <t>3 whey scoops + water</t>
         </is>
       </c>
       <c r="D71" s="7" t="n">
-        <v>10</v>
+        <v>300</v>
       </c>
       <c r="E71" s="7" t="n">
-        <v>20</v>
+        <v>390</v>
       </c>
       <c r="F71" s="8">
         <f>AVERAGE(D71:E71)</f>
         <v/>
       </c>
       <c r="G71" s="9" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="H71" s="9" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="I71" s="10">
         <f>AVERAGE(G71:H71)</f>
         <v/>
       </c>
       <c r="J71" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K71" s="9" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="L71" s="10">
         <f>AVERAGE(J71:K71)</f>
@@ -4291,6 +4291,61 @@
         </is>
       </c>
       <c r="N71" s="6" t="inlineStr">
+        <is>
+          <t>Closing scoops confirmed - first full evening dose logged in five days</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Supplement</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>1 omega-3 fish oil 1000 mg + 1 vitamin D3 50000 IU capsule</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E72" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F72" s="8">
+        <f>AVERAGE(D72:E72)</f>
+        <v/>
+      </c>
+      <c r="G72" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I72" s="10">
+        <f>AVERAGE(G72:H72)</f>
+        <v/>
+      </c>
+      <c r="J72" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K72" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="L72" s="10">
+        <f>AVERAGE(J72:K72)</f>
+        <v/>
+      </c>
+      <c r="M72" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N72" s="6" t="inlineStr">
         <is>
           <t>Negligible calories; D3 50000 IU is a weekly-dose strength</t>
         </is>
@@ -4414,11 +4469,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4426,11 +4481,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4438,11 +4493,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4450,11 +4505,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A5,Meals!$M$5:$M$71,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4467,11 +4522,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4479,11 +4534,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4491,11 +4546,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4503,11 +4558,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A6,Meals!$M$5:$M$71,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4520,11 +4575,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4532,11 +4587,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4544,11 +4599,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4556,11 +4611,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A7,Meals!$M$5:$M$71,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4573,11 +4628,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4585,11 +4640,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4597,11 +4652,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4609,11 +4664,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A8,Meals!$M$5:$M$71,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4626,11 +4681,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4638,11 +4693,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4650,11 +4705,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4662,11 +4717,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A9,Meals!$M$5:$M$71,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4679,11 +4734,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4691,11 +4746,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4703,11 +4758,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4715,11 +4770,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A10,Meals!$M$5:$M$71,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4732,11 +4787,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4744,11 +4799,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4756,11 +4811,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4768,11 +4823,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A11,Meals!$M$5:$M$71,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4785,11 +4840,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4797,11 +4852,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4809,11 +4864,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4821,11 +4876,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A12,Meals!$M$5:$M$71,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4838,11 +4893,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4850,11 +4905,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4862,11 +4917,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4874,11 +4929,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A13,Meals!$M$5:$M$71,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4891,11 +4946,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4903,11 +4958,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4915,11 +4970,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4927,11 +4982,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A14,Meals!$M$5:$M$71,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -4944,11 +4999,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -4956,11 +5011,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4968,11 +5023,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -4980,11 +5035,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A15,Meals!$M$5:$M$71,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -4997,11 +5052,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5009,11 +5064,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5021,11 +5076,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5033,11 +5088,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A16,Meals!$M$5:$M$71,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5050,11 +5105,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$71,Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$71,Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5062,11 +5117,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$71,Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$71,Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5074,11 +5129,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$71,Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$71,Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5086,11 +5141,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$71,$A17,Meals!$M$5:$M$71,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">

</xml_diff>

<commit_message>
Record the 09-16 weigh-in and confirm the activity multiplier
90.15 kg, up 0.10 over 5 days, taken in different clothing.

Measured from 09-07 after the glycogen flush, the trend is -0.467 kg/wk
over 9 days against -0.476 predicted from twelve logged days. The two
agree to within 2%, so the x1.52 multiplier revised on 09-11 is correct
and the 2,120 target holds.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -5167,7 +5167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5321,8 +5321,33 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B9" s="24" t="n">
+        <v>90.15000000000001</v>
+      </c>
+      <c r="C9" s="25">
+        <f>B9-B8</f>
+        <v/>
+      </c>
+      <c r="D9" s="25">
+        <f>B9-$B$5</f>
+        <v/>
+      </c>
+      <c r="E9" s="26">
+        <f>AVERAGE(B5:B9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Morning weigh-in - user noted different clothing from previous weigh-ins</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>A drop in the first week is mostly water and glycogen, not fat. Judge the trend over 2-3 weeks, and change the activity multiplier on Targets only then.</t>
         </is>

</xml_diff>

<commit_message>
Log Day 14 breakfast and plan the Thursday protein desert
Eighth skip of the white chutney. Thursday serves 54 g of protein with
no meat at dinner, so it is the slot the grilled chicken was bought for:
250 g with two chapati lands the day at 2,115 kcal and 144.5 g on a
single scoop.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N72"/>
+  <dimension ref="A1:N73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4351,6 +4351,61 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="4" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>Large restaurant dosa + sambar + red chutney (white chutney skipped)</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="n">
+        <v>380</v>
+      </c>
+      <c r="E73" s="7" t="n">
+        <v>590</v>
+      </c>
+      <c r="F73" s="8">
+        <f>AVERAGE(D73:E73)</f>
+        <v/>
+      </c>
+      <c r="G73" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H73" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="I73" s="10">
+        <f>AVERAGE(G73:H73)</f>
+        <v/>
+      </c>
+      <c r="J73" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="K73" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="L73" s="10">
+        <f>AVERAGE(J73:K73)</f>
+        <v/>
+      </c>
+      <c r="M73" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N73" s="6" t="inlineStr">
+        <is>
+          <t>Eighth skip of the white chutney</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -4365,7 +4420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4469,11 +4524,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4481,11 +4536,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4493,11 +4548,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4505,11 +4560,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A5,Meals!$M$5:$M$72,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4522,11 +4577,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4534,11 +4589,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4546,11 +4601,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4558,11 +4613,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A6,Meals!$M$5:$M$72,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4575,11 +4630,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4587,11 +4642,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4599,11 +4654,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4611,11 +4666,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A7,Meals!$M$5:$M$72,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4628,11 +4683,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4640,11 +4695,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4652,11 +4707,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4664,11 +4719,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A8,Meals!$M$5:$M$72,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4681,11 +4736,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4693,11 +4748,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4705,11 +4760,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4717,11 +4772,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A9,Meals!$M$5:$M$72,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4734,11 +4789,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4746,11 +4801,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4758,11 +4813,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4770,11 +4825,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A10,Meals!$M$5:$M$72,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4787,11 +4842,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4799,11 +4854,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4811,11 +4866,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4823,11 +4878,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A11,Meals!$M$5:$M$72,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4840,11 +4895,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4852,11 +4907,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4864,11 +4919,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4876,11 +4931,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A12,Meals!$M$5:$M$72,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4893,11 +4948,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4905,11 +4960,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4917,11 +4972,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4929,11 +4984,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A13,Meals!$M$5:$M$72,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -4946,11 +5001,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -4958,11 +5013,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -4970,11 +5025,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -4982,11 +5037,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A14,Meals!$M$5:$M$72,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -4999,11 +5054,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5011,11 +5066,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5023,11 +5078,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5035,11 +5090,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A15,Meals!$M$5:$M$72,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5052,11 +5107,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5064,11 +5119,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5076,11 +5131,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5088,11 +5143,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A16,Meals!$M$5:$M$72,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5105,11 +5160,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$72,Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$72,Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5117,11 +5172,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$72,Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$72,Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5129,11 +5184,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$72,Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$72,Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5141,15 +5196,68 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$72,$A17,Meals!$M$5:$M$72,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
         <f>D17-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B18" s="21">
+        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"logged")</f>
+        <v/>
+      </c>
+      <c r="C18" s="21">
+        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"logged")</f>
+        <v/>
+      </c>
+      <c r="D18" s="21">
+        <f>AVERAGE(B18:C18)</f>
+        <v/>
+      </c>
+      <c r="E18" s="22">
+        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"logged")</f>
+        <v/>
+      </c>
+      <c r="F18" s="22">
+        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"logged")</f>
+        <v/>
+      </c>
+      <c r="G18" s="22">
+        <f>AVERAGE(E18:F18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="22">
+        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"logged")</f>
+        <v/>
+      </c>
+      <c r="I18" s="22">
+        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"logged")</f>
+        <v/>
+      </c>
+      <c r="J18" s="22">
+        <f>AVERAGE(H18:I18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"logged")</f>
+        <v/>
+      </c>
+      <c r="L18" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"pending")</f>
+        <v/>
+      </c>
+      <c r="M18" s="23">
+        <f>D18-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -6108,7 +6216,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$17)</f>
+        <f>COUNT(Daily!$A$5:$A$18)</f>
         <v/>
       </c>
     </row>
@@ -6119,7 +6227,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$17),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$18),0)</f>
         <v/>
       </c>
     </row>
@@ -6130,7 +6238,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$17),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$18),0)</f>
         <v/>
       </c>
     </row>
@@ -6141,7 +6249,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$17),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$18),0)</f>
         <v/>
       </c>
     </row>
@@ -6185,7 +6293,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$17,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$18,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -6196,7 +6304,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$17)</f>
+        <f>SUM(Daily!$L$5:$L$18)</f>
         <v/>
       </c>
     </row>
@@ -6247,19 +6355,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$17,"&gt;="&amp;$A17,Daily!$A$5:$A$17,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$18,"&gt;="&amp;$A17,Daily!$A$5:$A$18,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$17,Daily!$A$5:$A$17,"&gt;="&amp;$A17,Daily!$A$5:$A$17,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$18,Daily!$A$5:$A$18,"&gt;="&amp;$A17,Daily!$A$5:$A$18,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$17,Daily!$A$5:$A$17,"&gt;="&amp;$A17,Daily!$A$5:$A$17,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$18,Daily!$A$5:$A$18,"&gt;="&amp;$A17,Daily!$A$5:$A$18,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$17,Daily!$A$5:$A$17,"&gt;="&amp;$A17,Daily!$A$5:$A$17,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$18,Daily!$A$5:$A$18,"&gt;="&amp;$A17,Daily!$A$5:$A$18,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -6271,19 +6379,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$17,"&gt;="&amp;$A18,Daily!$A$5:$A$17,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$18,"&gt;="&amp;$A18,Daily!$A$5:$A$18,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$17,Daily!$A$5:$A$17,"&gt;="&amp;$A18,Daily!$A$5:$A$17,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$18,Daily!$A$5:$A$18,"&gt;="&amp;$A18,Daily!$A$5:$A$18,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$17,Daily!$A$5:$A$17,"&gt;="&amp;$A18,Daily!$A$5:$A$17,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$18,Daily!$A$5:$A$18,"&gt;="&amp;$A18,Daily!$A$5:$A$18,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$17,Daily!$A$5:$A$17,"&gt;="&amp;$A18,Daily!$A$5:$A$17,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$18,Daily!$A$5:$A$18,"&gt;="&amp;$A18,Daily!$A$5:$A$18,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -6295,19 +6403,19 @@
         <v>46285</v>
       </c>
       <c r="C19" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$17,"&gt;="&amp;$A19,Daily!$A$5:$A$17,"&lt;="&amp;$B19)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$18,"&gt;="&amp;$A19,Daily!$A$5:$A$18,"&lt;="&amp;$B19)</f>
         <v/>
       </c>
       <c r="D19" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$17,Daily!$A$5:$A$17,"&gt;="&amp;$A19,Daily!$A$5:$A$17,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$18,Daily!$A$5:$A$18,"&gt;="&amp;$A19,Daily!$A$5:$A$18,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$17,Daily!$A$5:$A$17,"&gt;="&amp;$A19,Daily!$A$5:$A$17,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$18,Daily!$A$5:$A$18,"&gt;="&amp;$A19,Daily!$A$5:$A$18,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$17,Daily!$A$5:$A$17,"&gt;="&amp;$A19,Daily!$A$5:$A$17,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$18,Daily!$A$5:$A$18,"&gt;="&amp;$A19,Daily!$A$5:$A$18,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
     </row>
@@ -6358,19 +6466,19 @@
         <v>46295</v>
       </c>
       <c r="C23" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$17,"&gt;="&amp;$A23,Daily!$A$5:$A$17,"&lt;="&amp;$B23)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$18,"&gt;="&amp;$A23,Daily!$A$5:$A$18,"&lt;="&amp;$B23)</f>
         <v/>
       </c>
       <c r="D23" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$17,Daily!$A$5:$A$17,"&gt;="&amp;$A23,Daily!$A$5:$A$17,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$18,Daily!$A$5:$A$18,"&gt;="&amp;$A23,Daily!$A$5:$A$18,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$17,Daily!$A$5:$A$17,"&gt;="&amp;$A23,Daily!$A$5:$A$17,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$18,Daily!$A$5:$A$18,"&gt;="&amp;$A23,Daily!$A$5:$A$18,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$17,Daily!$A$5:$A$17,"&gt;="&amp;$A23,Daily!$A$5:$A$17,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$18,Daily!$A$5:$A$18,"&gt;="&amp;$A23,Daily!$A$5:$A$18,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Record the 09-17 weigh-in: 90.05, yesterday's rise reversed
The 09-16 +0.10 was noise, as read - different clothing and two higher
carb days. It came off the next morning with nothing changed.

The trend from 09-07 is now -0.490 kg/wk over 10 days against -0.476
predicted from the logged intake.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -5275,7 +5275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5454,8 +5454,33 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B10" s="24" t="n">
+        <v>90.05</v>
+      </c>
+      <c r="C10" s="25">
+        <f>B10-B9</f>
+        <v/>
+      </c>
+      <c r="D10" s="25">
+        <f>B10-$B$5</f>
+        <v/>
+      </c>
+      <c r="E10" s="26">
+        <f>AVERAGE(B5:B10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Morning weigh-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>A drop in the first week is mostly water and glycogen, not fat. Judge the trend over 2-3 weeks, and change the activity multiplier on Targets only then.</t>
         </is>

</xml_diff>

<commit_message>
Log Day 14 scoop 1
With the grilled chicken at dinner the day needs no further whey: one
scoop total, 144.5 g of protein, on target. Without it, three more.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N73"/>
+  <dimension ref="A1:N74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4403,6 +4403,61 @@
       <c r="N73" s="6" t="inlineStr">
         <is>
           <t>Eighth skip of the white chutney</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1 whey scoop</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E74" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F74" s="8">
+        <f>AVERAGE(D74:E74)</f>
+        <v/>
+      </c>
+      <c r="G74" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H74" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I74" s="10">
+        <f>AVERAGE(G74:H74)</f>
+        <v/>
+      </c>
+      <c r="J74" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K74" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L74" s="10">
+        <f>AVERAGE(J74:K74)</f>
+        <v/>
+      </c>
+      <c r="M74" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N74" s="6" t="inlineStr">
+        <is>
+          <t>Scoop 1</t>
         </is>
       </c>
     </row>
@@ -4524,11 +4579,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4536,11 +4591,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4548,11 +4603,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4560,11 +4615,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A5,Meals!$M$5:$M$73,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4577,11 +4632,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4589,11 +4644,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4601,11 +4656,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4613,11 +4668,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A6,Meals!$M$5:$M$73,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4630,11 +4685,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4642,11 +4697,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4654,11 +4709,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4666,11 +4721,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A7,Meals!$M$5:$M$73,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4683,11 +4738,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4695,11 +4750,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4707,11 +4762,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4719,11 +4774,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A8,Meals!$M$5:$M$73,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4736,11 +4791,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4748,11 +4803,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4760,11 +4815,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4772,11 +4827,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A9,Meals!$M$5:$M$73,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4789,11 +4844,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4801,11 +4856,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4813,11 +4868,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4825,11 +4880,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A10,Meals!$M$5:$M$73,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4842,11 +4897,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4854,11 +4909,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4866,11 +4921,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4878,11 +4933,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A11,Meals!$M$5:$M$73,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4895,11 +4950,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4907,11 +4962,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4919,11 +4974,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4931,11 +4986,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A12,Meals!$M$5:$M$73,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -4948,11 +5003,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -4960,11 +5015,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4972,11 +5027,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -4984,11 +5039,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A13,Meals!$M$5:$M$73,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5001,11 +5056,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5013,11 +5068,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5025,11 +5080,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5037,11 +5092,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A14,Meals!$M$5:$M$73,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5054,11 +5109,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5066,11 +5121,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5078,11 +5133,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5090,11 +5145,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A15,Meals!$M$5:$M$73,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5107,11 +5162,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5119,11 +5174,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5131,11 +5186,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5143,11 +5198,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A16,Meals!$M$5:$M$73,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5160,11 +5215,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5172,11 +5227,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5184,11 +5239,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5196,11 +5251,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A17,Meals!$M$5:$M$73,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -5213,11 +5268,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$73,Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$73,Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -5225,11 +5280,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$73,Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$73,Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -5237,11 +5292,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$73,Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$73,Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -5249,11 +5304,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$73,$A18,Meals!$M$5:$M$73,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">

</xml_diff>

<commit_message>
Log Day 14 lunch: halved plate with one container instead of four
Moru is the right container to pick - yogurt-based, ~85 kcal against the
coconut chammanthi's ~125 for the same protein. Yesterday's four cost
~370.

The grilled chicken did not appear at lunch, so it becomes the dinner
lever: 250 g with two chapati lands the day at 2,192 and 144 g on a
single scoop.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N74"/>
+  <dimension ref="A1:N75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4412,39 +4412,39 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Black coffee + 1 whey scoop</t>
+          <t>Mess meals plate (rice halved) + 1 fried fish + sambar, cabbage thoran, 2 veg curries + moru curry</t>
         </is>
       </c>
       <c r="D74" s="7" t="n">
-        <v>100</v>
+        <v>645</v>
       </c>
       <c r="E74" s="7" t="n">
-        <v>130</v>
+        <v>1030</v>
       </c>
       <c r="F74" s="8">
         <f>AVERAGE(D74:E74)</f>
         <v/>
       </c>
       <c r="G74" s="9" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="H74" s="9" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="I74" s="10">
         <f>AVERAGE(G74:H74)</f>
         <v/>
       </c>
       <c r="J74" s="9" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="K74" s="9" t="n">
-        <v>3</v>
+        <v>52</v>
       </c>
       <c r="L74" s="10">
         <f>AVERAGE(J74:K74)</f>
@@ -4456,6 +4456,61 @@
         </is>
       </c>
       <c r="N74" s="6" t="inlineStr">
+        <is>
+          <t>Only the moru container taken rather than all four</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1 whey scoop</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E75" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F75" s="8">
+        <f>AVERAGE(D75:E75)</f>
+        <v/>
+      </c>
+      <c r="G75" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H75" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I75" s="10">
+        <f>AVERAGE(G75:H75)</f>
+        <v/>
+      </c>
+      <c r="J75" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K75" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L75" s="10">
+        <f>AVERAGE(J75:K75)</f>
+        <v/>
+      </c>
+      <c r="M75" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N75" s="6" t="inlineStr">
         <is>
           <t>Scoop 1</t>
         </is>
@@ -4579,11 +4634,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4591,11 +4646,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4603,11 +4658,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4615,11 +4670,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A5,Meals!$M$5:$M$74,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4632,11 +4687,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4644,11 +4699,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4656,11 +4711,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4668,11 +4723,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A6,Meals!$M$5:$M$74,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4685,11 +4740,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4697,11 +4752,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4709,11 +4764,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4721,11 +4776,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A7,Meals!$M$5:$M$74,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4738,11 +4793,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4750,11 +4805,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4762,11 +4817,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4774,11 +4829,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A8,Meals!$M$5:$M$74,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4791,11 +4846,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4803,11 +4858,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4815,11 +4870,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4827,11 +4882,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A9,Meals!$M$5:$M$74,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4844,11 +4899,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4856,11 +4911,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4868,11 +4923,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4880,11 +4935,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A10,Meals!$M$5:$M$74,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4897,11 +4952,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4909,11 +4964,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4921,11 +4976,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4933,11 +4988,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A11,Meals!$M$5:$M$74,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4950,11 +5005,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -4962,11 +5017,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -4974,11 +5029,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -4986,11 +5041,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A12,Meals!$M$5:$M$74,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5003,11 +5058,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5015,11 +5070,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5027,11 +5082,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5039,11 +5094,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A13,Meals!$M$5:$M$74,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5056,11 +5111,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5068,11 +5123,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5080,11 +5135,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5092,11 +5147,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A14,Meals!$M$5:$M$74,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5109,11 +5164,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5121,11 +5176,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5133,11 +5188,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5145,11 +5200,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A15,Meals!$M$5:$M$74,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5162,11 +5217,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5174,11 +5229,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5186,11 +5241,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5198,11 +5253,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A16,Meals!$M$5:$M$74,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5215,11 +5270,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5227,11 +5282,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5239,11 +5294,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5251,11 +5306,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A17,Meals!$M$5:$M$74,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -5268,11 +5323,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$74,Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$74,Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -5280,11 +5335,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$74,Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$74,Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -5292,11 +5347,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$74,Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$74,Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -5304,11 +5359,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$74,$A18,Meals!$M$5:$M$74,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">

</xml_diff>

<commit_message>
Log Day 14 scoops 2 and 3 and reshape the evening
Three scoops by mid-afternoon puts protein at 111 g before dinner, so
the floor is solved and only 452 kcal of room is left. That makes this
morning's 250 g chicken plus two chapati a 300 kcal overshoot.

200 g of chicken on its own lands 32 under target at 168 g of protein
and a 582 deficit - the best-shaped day of the fourteen.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N75"/>
+  <dimension ref="A1:N76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4513,6 +4513,61 @@
       <c r="N75" s="6" t="inlineStr">
         <is>
           <t>Scoop 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 2 whey scoops</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="E76" s="7" t="n">
+        <v>260</v>
+      </c>
+      <c r="F76" s="8">
+        <f>AVERAGE(D76:E76)</f>
+        <v/>
+      </c>
+      <c r="G76" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="H76" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I76" s="10">
+        <f>AVERAGE(G76:H76)</f>
+        <v/>
+      </c>
+      <c r="J76" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K76" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L76" s="10">
+        <f>AVERAGE(J76:K76)</f>
+        <v/>
+      </c>
+      <c r="M76" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N76" s="6" t="inlineStr">
+        <is>
+          <t>Scoops 2 and 3</t>
         </is>
       </c>
     </row>
@@ -4634,11 +4689,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4646,11 +4701,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4658,11 +4713,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4670,11 +4725,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A5,Meals!$M$5:$M$75,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4687,11 +4742,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4699,11 +4754,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4711,11 +4766,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4723,11 +4778,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A6,Meals!$M$5:$M$75,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4740,11 +4795,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4752,11 +4807,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4764,11 +4819,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4776,11 +4831,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A7,Meals!$M$5:$M$75,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4793,11 +4848,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4805,11 +4860,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4817,11 +4872,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4829,11 +4884,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A8,Meals!$M$5:$M$75,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4846,11 +4901,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4858,11 +4913,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4870,11 +4925,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4882,11 +4937,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A9,Meals!$M$5:$M$75,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4899,11 +4954,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4911,11 +4966,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4923,11 +4978,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4935,11 +4990,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A10,Meals!$M$5:$M$75,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4952,11 +5007,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -4964,11 +5019,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4976,11 +5031,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -4988,11 +5043,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A11,Meals!$M$5:$M$75,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5005,11 +5060,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5017,11 +5072,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5029,11 +5084,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5041,11 +5096,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A12,Meals!$M$5:$M$75,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5058,11 +5113,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5070,11 +5125,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5082,11 +5137,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5094,11 +5149,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A13,Meals!$M$5:$M$75,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5111,11 +5166,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5123,11 +5178,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5135,11 +5190,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5147,11 +5202,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A14,Meals!$M$5:$M$75,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5164,11 +5219,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5176,11 +5231,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5188,11 +5243,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5200,11 +5255,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A15,Meals!$M$5:$M$75,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5217,11 +5272,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5229,11 +5284,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5241,11 +5296,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5253,11 +5308,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A16,Meals!$M$5:$M$75,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5270,11 +5325,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5282,11 +5337,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5294,11 +5349,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5306,11 +5361,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A17,Meals!$M$5:$M$75,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -5323,11 +5378,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$75,Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$75,Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -5335,11 +5390,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$75,Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$75,Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -5347,11 +5402,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$75,Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$75,Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -5359,11 +5414,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$75,$A18,Meals!$M$5:$M$75,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">

</xml_diff>

<commit_message>
Close Day 14: first day of the fourteen with no deficit
2,708 kcal, 38 above maintenance, and 180.75 g of protein - by far the
highest protein day, 40 g clear of the previous best.

The chicken was the right food at 12 g of protein per 100 kcal. The
accompaniments cost ~450 kcal for ~8 g between them, and the three
afternoon scoops had already left only 452 kcal of evening room.

Thirteen complete days now average 2,189 kcal and 114.1 g of protein,
a 480 deficit, 0.44 kg/week.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N76"/>
+  <dimension ref="A1:N77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4412,39 +4412,39 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate (rice halved) + 1 fried fish + sambar, cabbage thoran, 2 veg curries + moru curry</t>
+          <t>Charcoal grilled chicken piece + Malabar porotta + hummus, garlic toum, tomato-onion mezze, pickles</t>
         </is>
       </c>
       <c r="D74" s="7" t="n">
-        <v>645</v>
+        <v>840</v>
       </c>
       <c r="E74" s="7" t="n">
-        <v>1030</v>
+        <v>1240</v>
       </c>
       <c r="F74" s="8">
         <f>AVERAGE(D74:E74)</f>
         <v/>
       </c>
       <c r="G74" s="9" t="n">
-        <v>24</v>
+        <v>60.5</v>
       </c>
       <c r="H74" s="9" t="n">
-        <v>37</v>
+        <v>79</v>
       </c>
       <c r="I74" s="10">
         <f>AVERAGE(G74:H74)</f>
         <v/>
       </c>
       <c r="J74" s="9" t="n">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="K74" s="9" t="n">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="L74" s="10">
         <f>AVERAGE(J74:K74)</f>
@@ -4457,7 +4457,7 @@
       </c>
       <c r="N74" s="6" t="inlineStr">
         <is>
-          <t>Only the moru container taken rather than all four</t>
+          <t>Restaurant grilled chicken meal</t>
         </is>
       </c>
     </row>
@@ -4467,39 +4467,39 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Black coffee + 1 whey scoop</t>
+          <t>Mess meals plate (rice halved) + 1 fried fish + sambar, cabbage thoran, 2 veg curries + moru curry</t>
         </is>
       </c>
       <c r="D75" s="7" t="n">
-        <v>100</v>
+        <v>645</v>
       </c>
       <c r="E75" s="7" t="n">
-        <v>130</v>
+        <v>1030</v>
       </c>
       <c r="F75" s="8">
         <f>AVERAGE(D75:E75)</f>
         <v/>
       </c>
       <c r="G75" s="9" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="H75" s="9" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="I75" s="10">
         <f>AVERAGE(G75:H75)</f>
         <v/>
       </c>
       <c r="J75" s="9" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="K75" s="9" t="n">
-        <v>3</v>
+        <v>52</v>
       </c>
       <c r="L75" s="10">
         <f>AVERAGE(J75:K75)</f>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="N75" s="6" t="inlineStr">
         <is>
-          <t>Scoop 1</t>
+          <t>Only the moru container taken rather than all four</t>
         </is>
       </c>
     </row>
@@ -4527,34 +4527,34 @@
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Black coffee + 2 whey scoops</t>
+          <t>Black coffee + 1 whey scoop</t>
         </is>
       </c>
       <c r="D76" s="7" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>260</v>
+        <v>130</v>
       </c>
       <c r="F76" s="8">
         <f>AVERAGE(D76:E76)</f>
         <v/>
       </c>
       <c r="G76" s="9" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H76" s="9" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="I76" s="10">
         <f>AVERAGE(G76:H76)</f>
         <v/>
       </c>
       <c r="J76" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K76" s="9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L76" s="10">
         <f>AVERAGE(J76:K76)</f>
@@ -4566,6 +4566,61 @@
         </is>
       </c>
       <c r="N76" s="6" t="inlineStr">
+        <is>
+          <t>Scoop 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 2 whey scoops</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="E77" s="7" t="n">
+        <v>260</v>
+      </c>
+      <c r="F77" s="8">
+        <f>AVERAGE(D77:E77)</f>
+        <v/>
+      </c>
+      <c r="G77" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="H77" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I77" s="10">
+        <f>AVERAGE(G77:H77)</f>
+        <v/>
+      </c>
+      <c r="J77" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K77" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L77" s="10">
+        <f>AVERAGE(J77:K77)</f>
+        <v/>
+      </c>
+      <c r="M77" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N77" s="6" t="inlineStr">
         <is>
           <t>Scoops 2 and 3</t>
         </is>
@@ -4689,11 +4744,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4701,11 +4756,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4713,11 +4768,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4725,11 +4780,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A5,Meals!$M$5:$M$76,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4742,11 +4797,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4754,11 +4809,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4766,11 +4821,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4778,11 +4833,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A6,Meals!$M$5:$M$76,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4795,11 +4850,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4807,11 +4862,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4819,11 +4874,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4831,11 +4886,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A7,Meals!$M$5:$M$76,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4848,11 +4903,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4860,11 +4915,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4872,11 +4927,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4884,11 +4939,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A8,Meals!$M$5:$M$76,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4901,11 +4956,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4913,11 +4968,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4925,11 +4980,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4937,11 +4992,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A9,Meals!$M$5:$M$76,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4954,11 +5009,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -4966,11 +5021,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -4978,11 +5033,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -4990,11 +5045,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A10,Meals!$M$5:$M$76,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5007,11 +5062,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5019,11 +5074,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5031,11 +5086,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5043,11 +5098,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A11,Meals!$M$5:$M$76,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5060,11 +5115,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5072,11 +5127,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5084,11 +5139,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5096,11 +5151,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A12,Meals!$M$5:$M$76,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5113,11 +5168,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5125,11 +5180,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5137,11 +5192,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5149,11 +5204,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A13,Meals!$M$5:$M$76,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5166,11 +5221,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5178,11 +5233,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5190,11 +5245,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5202,11 +5257,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A14,Meals!$M$5:$M$76,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5219,11 +5274,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5231,11 +5286,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5243,11 +5298,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5255,11 +5310,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A15,Meals!$M$5:$M$76,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5272,11 +5327,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5284,11 +5339,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5296,11 +5351,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5308,11 +5363,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A16,Meals!$M$5:$M$76,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5325,11 +5380,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5337,11 +5392,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5349,11 +5404,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5361,11 +5416,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A17,Meals!$M$5:$M$76,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -5378,11 +5433,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$76,Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$76,Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -5390,11 +5445,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$76,Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$76,Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -5402,11 +5457,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$76,Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$76,Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -5414,11 +5469,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$76,$A18,Meals!$M$5:$M$76,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">

</xml_diff>

<commit_message>
Record the 09-18 weigh-in: 89.55, first reading under 90 kg
The -0.50 follows a day that finished 38 kcal above maintenance, so it
is water rather than fat. Endpoint rates are unstable at this noise
level - 09-07 to 09-18 reads -0.764 kg/wk, which the intake cannot
support.

Switches the trend measure to a least-squares fit through the six
post-flush points: -0.489 kg/wk against -0.436 predicted from the food
log.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -5495,7 +5495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5699,8 +5699,33 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B11" s="24" t="n">
+        <v>89.55</v>
+      </c>
+      <c r="C11" s="25">
+        <f>B11-B10</f>
+        <v/>
+      </c>
+      <c r="D11" s="25">
+        <f>B11-$B$5</f>
+        <v/>
+      </c>
+      <c r="E11" s="26">
+        <f>AVERAGE(B5:B11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Morning weigh-in - first reading under 90 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>A drop in the first week is mostly water and glycogen, not fat. Judge the trend over 2-3 weeks, and change the activity multiplier on Targets only then.</t>
         </is>

</xml_diff>

<commit_message>
Log Day 15 breakfast and plan Friday
Puttu and kadala in place of the menu's idly set costs 355 kcal and
~18 g of fat - the idly set is the lightest breakfast of the week and
Friday is the roomiest day, so the swap spends most of that advantage
early.

Four scoops lands 40 under target at 153 g of protein and ~70 g of fat,
the lowest fat day since Day 1.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N77"/>
+  <dimension ref="A1:N78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4626,6 +4626,61 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" s="4" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>2 puttu pieces + kadala curry</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>560</v>
+      </c>
+      <c r="E78" s="7" t="n">
+        <v>800</v>
+      </c>
+      <c r="F78" s="8">
+        <f>AVERAGE(D78:E78)</f>
+        <v/>
+      </c>
+      <c r="G78" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="H78" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="I78" s="10">
+        <f>AVERAGE(G78:H78)</f>
+        <v/>
+      </c>
+      <c r="J78" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="K78" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="L78" s="10">
+        <f>AVERAGE(J78:K78)</f>
+        <v/>
+      </c>
+      <c r="M78" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N78" s="6" t="inlineStr">
+        <is>
+          <t>Same breakfast as Day 13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -4640,7 +4695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4744,11 +4799,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4756,11 +4811,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4768,11 +4823,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4780,11 +4835,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A5,Meals!$M$5:$M$77,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4797,11 +4852,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4809,11 +4864,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4821,11 +4876,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4833,11 +4888,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A6,Meals!$M$5:$M$77,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4850,11 +4905,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4862,11 +4917,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4874,11 +4929,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4886,11 +4941,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A7,Meals!$M$5:$M$77,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4903,11 +4958,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4915,11 +4970,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4927,11 +4982,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4939,11 +4994,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A8,Meals!$M$5:$M$77,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -4956,11 +5011,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -4968,11 +5023,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4980,11 +5035,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -4992,11 +5047,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A9,Meals!$M$5:$M$77,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5009,11 +5064,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5021,11 +5076,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5033,11 +5088,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5045,11 +5100,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A10,Meals!$M$5:$M$77,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5062,11 +5117,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5074,11 +5129,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5086,11 +5141,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5098,11 +5153,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A11,Meals!$M$5:$M$77,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5115,11 +5170,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5127,11 +5182,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5139,11 +5194,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5151,11 +5206,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A12,Meals!$M$5:$M$77,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5168,11 +5223,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5180,11 +5235,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5192,11 +5247,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5204,11 +5259,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A13,Meals!$M$5:$M$77,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5221,11 +5276,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5233,11 +5288,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5245,11 +5300,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5257,11 +5312,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A14,Meals!$M$5:$M$77,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5274,11 +5329,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5286,11 +5341,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5298,11 +5353,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5310,11 +5365,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A15,Meals!$M$5:$M$77,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5327,11 +5382,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5339,11 +5394,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5351,11 +5406,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5363,11 +5418,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A16,Meals!$M$5:$M$77,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5380,11 +5435,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5392,11 +5447,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5404,11 +5459,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5416,11 +5471,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A17,Meals!$M$5:$M$77,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -5433,11 +5488,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$77,Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$77,Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -5445,11 +5500,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$77,Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$77,Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -5457,11 +5512,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$77,Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$77,Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -5469,15 +5524,68 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$77,$A18,Meals!$M$5:$M$77,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
         <f>D18-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B19" s="8">
+        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"logged")</f>
+        <v/>
+      </c>
+      <c r="C19" s="8">
+        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"logged")</f>
+        <v/>
+      </c>
+      <c r="D19" s="8">
+        <f>AVERAGE(B19:C19)</f>
+        <v/>
+      </c>
+      <c r="E19" s="10">
+        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"logged")</f>
+        <v/>
+      </c>
+      <c r="F19" s="10">
+        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"logged")</f>
+        <v/>
+      </c>
+      <c r="G19" s="10">
+        <f>AVERAGE(E19:F19)</f>
+        <v/>
+      </c>
+      <c r="H19" s="10">
+        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"logged")</f>
+        <v/>
+      </c>
+      <c r="I19" s="10">
+        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"logged")</f>
+        <v/>
+      </c>
+      <c r="J19" s="10">
+        <f>AVERAGE(H19:I19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"logged")</f>
+        <v/>
+      </c>
+      <c r="L19" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"pending")</f>
+        <v/>
+      </c>
+      <c r="M19" s="19">
+        <f>D19-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -6486,7 +6594,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$18)</f>
+        <f>COUNT(Daily!$A$5:$A$19)</f>
         <v/>
       </c>
     </row>
@@ -6497,7 +6605,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$18),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$19),0)</f>
         <v/>
       </c>
     </row>
@@ -6508,7 +6616,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$18),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$19),0)</f>
         <v/>
       </c>
     </row>
@@ -6519,7 +6627,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$18),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$19),0)</f>
         <v/>
       </c>
     </row>
@@ -6563,7 +6671,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$18,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$19,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -6574,7 +6682,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$18)</f>
+        <f>SUM(Daily!$L$5:$L$19)</f>
         <v/>
       </c>
     </row>
@@ -6625,19 +6733,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$18,"&gt;="&amp;$A17,Daily!$A$5:$A$18,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$19,"&gt;="&amp;$A17,Daily!$A$5:$A$19,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$18,Daily!$A$5:$A$18,"&gt;="&amp;$A17,Daily!$A$5:$A$18,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$19,Daily!$A$5:$A$19,"&gt;="&amp;$A17,Daily!$A$5:$A$19,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$18,Daily!$A$5:$A$18,"&gt;="&amp;$A17,Daily!$A$5:$A$18,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$19,Daily!$A$5:$A$19,"&gt;="&amp;$A17,Daily!$A$5:$A$19,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$18,Daily!$A$5:$A$18,"&gt;="&amp;$A17,Daily!$A$5:$A$18,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$19,Daily!$A$5:$A$19,"&gt;="&amp;$A17,Daily!$A$5:$A$19,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -6649,19 +6757,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$18,"&gt;="&amp;$A18,Daily!$A$5:$A$18,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$19,"&gt;="&amp;$A18,Daily!$A$5:$A$19,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$18,Daily!$A$5:$A$18,"&gt;="&amp;$A18,Daily!$A$5:$A$18,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$19,Daily!$A$5:$A$19,"&gt;="&amp;$A18,Daily!$A$5:$A$19,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$18,Daily!$A$5:$A$18,"&gt;="&amp;$A18,Daily!$A$5:$A$18,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$19,Daily!$A$5:$A$19,"&gt;="&amp;$A18,Daily!$A$5:$A$19,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$18,Daily!$A$5:$A$18,"&gt;="&amp;$A18,Daily!$A$5:$A$18,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$19,Daily!$A$5:$A$19,"&gt;="&amp;$A18,Daily!$A$5:$A$19,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -6673,19 +6781,19 @@
         <v>46285</v>
       </c>
       <c r="C19" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$18,"&gt;="&amp;$A19,Daily!$A$5:$A$18,"&lt;="&amp;$B19)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$19,"&gt;="&amp;$A19,Daily!$A$5:$A$19,"&lt;="&amp;$B19)</f>
         <v/>
       </c>
       <c r="D19" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$18,Daily!$A$5:$A$18,"&gt;="&amp;$A19,Daily!$A$5:$A$18,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$19,Daily!$A$5:$A$19,"&gt;="&amp;$A19,Daily!$A$5:$A$19,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$18,Daily!$A$5:$A$18,"&gt;="&amp;$A19,Daily!$A$5:$A$18,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$19,Daily!$A$5:$A$19,"&gt;="&amp;$A19,Daily!$A$5:$A$19,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$18,Daily!$A$5:$A$18,"&gt;="&amp;$A19,Daily!$A$5:$A$18,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$19,Daily!$A$5:$A$19,"&gt;="&amp;$A19,Daily!$A$5:$A$19,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
     </row>
@@ -6736,19 +6844,19 @@
         <v>46295</v>
       </c>
       <c r="C23" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$18,"&gt;="&amp;$A23,Daily!$A$5:$A$18,"&lt;="&amp;$B23)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$19,"&gt;="&amp;$A23,Daily!$A$5:$A$19,"&lt;="&amp;$B23)</f>
         <v/>
       </c>
       <c r="D23" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$18,Daily!$A$5:$A$18,"&gt;="&amp;$A23,Daily!$A$5:$A$18,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$19,Daily!$A$5:$A$19,"&gt;="&amp;$A23,Daily!$A$5:$A$19,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$18,Daily!$A$5:$A$18,"&gt;="&amp;$A23,Daily!$A$5:$A$18,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$19,Daily!$A$5:$A$19,"&gt;="&amp;$A23,Daily!$A$5:$A$19,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$18,Daily!$A$5:$A$18,"&gt;="&amp;$A23,Daily!$A$5:$A$18,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$19,Daily!$A$5:$A$19,"&gt;="&amp;$A23,Daily!$A$5:$A$19,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Day 15 lunch: halved biriyani with two chicken pieces
Ran ~145 kcal over estimate but delivered ~6 g more protein. Three
scoops lands the day 10 under target at 136.75 g of protein and ~74.5 g
of fat, which would tie Day 11 as the second-lowest of the fifteen.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N78"/>
+  <dimension ref="A1:N79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4678,6 +4678,61 @@
       <c r="N78" s="6" t="inlineStr">
         <is>
           <t>Same breakfast as Day 13</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>Chicken biriyani (rice halved) + 2 chicken pieces + raita + garlic pickle</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="n">
+        <v>480</v>
+      </c>
+      <c r="E79" s="7" t="n">
+        <v>730</v>
+      </c>
+      <c r="F79" s="8">
+        <f>AVERAGE(D79:E79)</f>
+        <v/>
+      </c>
+      <c r="G79" s="9" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="H79" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I79" s="10">
+        <f>AVERAGE(G79:H79)</f>
+        <v/>
+      </c>
+      <c r="J79" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="K79" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="L79" s="10">
+        <f>AVERAGE(J79:K79)</f>
+        <v/>
+      </c>
+      <c r="M79" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N79" s="6" t="inlineStr">
+        <is>
+          <t>Rice halved; 2 chicken pieces</t>
         </is>
       </c>
     </row>
@@ -4799,11 +4854,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4811,11 +4866,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4823,11 +4878,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4835,11 +4890,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A5,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4852,11 +4907,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4864,11 +4919,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4876,11 +4931,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4888,11 +4943,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A6,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4905,11 +4960,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4917,11 +4972,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4929,11 +4984,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4941,11 +4996,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A7,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -4958,11 +5013,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -4970,11 +5025,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -4982,11 +5037,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -4994,11 +5049,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A8,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5011,11 +5066,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5023,11 +5078,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5035,11 +5090,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5047,11 +5102,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A9,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5064,11 +5119,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5076,11 +5131,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5088,11 +5143,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5100,11 +5155,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A10,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5117,11 +5172,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5129,11 +5184,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5141,11 +5196,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5153,11 +5208,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A11,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5170,11 +5225,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5182,11 +5237,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5194,11 +5249,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5206,11 +5261,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A12,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5223,11 +5278,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5235,11 +5290,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5247,11 +5302,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5259,11 +5314,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A13,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5276,11 +5331,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5288,11 +5343,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5300,11 +5355,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5312,11 +5367,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A14,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5329,11 +5384,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5341,11 +5396,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5353,11 +5408,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5365,11 +5420,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A15,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5382,11 +5437,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5394,11 +5449,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5406,11 +5461,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5418,11 +5473,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A16,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5435,11 +5490,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5447,11 +5502,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5459,11 +5514,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5471,11 +5526,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A17,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -5488,11 +5543,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -5500,11 +5555,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -5512,11 +5567,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -5524,11 +5579,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A18,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -5541,11 +5596,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$78,Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$78,Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -5553,11 +5608,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$78,Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$78,Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -5565,11 +5620,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$78,Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$78,Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -5577,11 +5632,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$78,$A19,Meals!$M$5:$M$78,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">

</xml_diff>

<commit_message>
Close Day 15: lowest-fat day since Day 1 at 70.5 g
1,880 kcal, 91.75 g protein, 70.5 g fat. Nothing on a Friday menu is
coconut-based, which did more for the fat line than any deliberate cut
of the past fortnight.

The two closing scoops were not confirmed, so the day closes 38 g under
the protein floor on a 789 deficit rather than at 2,110 and 136.75 g.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N79"/>
+  <dimension ref="A1:N81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4687,39 +4687,39 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Chicken biriyani (rice halved) + 2 chicken pieces + raita + garlic pickle</t>
+          <t>2 chapati + kadala curry</t>
         </is>
       </c>
       <c r="D79" s="7" t="n">
-        <v>480</v>
+        <v>400</v>
       </c>
       <c r="E79" s="7" t="n">
-        <v>730</v>
+        <v>560</v>
       </c>
       <c r="F79" s="8">
         <f>AVERAGE(D79:E79)</f>
         <v/>
       </c>
       <c r="G79" s="9" t="n">
-        <v>29.5</v>
+        <v>14</v>
       </c>
       <c r="H79" s="9" t="n">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I79" s="10">
         <f>AVERAGE(G79:H79)</f>
         <v/>
       </c>
       <c r="J79" s="9" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="K79" s="9" t="n">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="L79" s="10">
         <f>AVERAGE(J79:K79)</f>
@@ -4732,7 +4732,117 @@
       </c>
       <c r="N79" s="6" t="inlineStr">
         <is>
+          <t>Mess Friday dinner</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>Chicken biriyani (rice halved) + 2 chicken pieces + raita + garlic pickle</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>480</v>
+      </c>
+      <c r="E80" s="7" t="n">
+        <v>730</v>
+      </c>
+      <c r="F80" s="8">
+        <f>AVERAGE(D80:E80)</f>
+        <v/>
+      </c>
+      <c r="G80" s="9" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="H80" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="I80" s="10">
+        <f>AVERAGE(G80:H80)</f>
+        <v/>
+      </c>
+      <c r="J80" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="K80" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="L80" s="10">
+        <f>AVERAGE(J80:K80)</f>
+        <v/>
+      </c>
+      <c r="M80" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N80" s="6" t="inlineStr">
+        <is>
           <t>Rice halved; 2 chicken pieces</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1 whey scoop</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E81" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F81" s="8">
+        <f>AVERAGE(D81:E81)</f>
+        <v/>
+      </c>
+      <c r="G81" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H81" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I81" s="10">
+        <f>AVERAGE(G81:H81)</f>
+        <v/>
+      </c>
+      <c r="J81" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K81" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L81" s="10">
+        <f>AVERAGE(J81:K81)</f>
+        <v/>
+      </c>
+      <c r="M81" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N81" s="6" t="inlineStr">
+        <is>
+          <t>Scoop 1</t>
         </is>
       </c>
     </row>
@@ -4854,11 +4964,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4866,11 +4976,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4878,11 +4988,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -4890,11 +5000,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A5,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -4907,11 +5017,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -4919,11 +5029,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -4931,11 +5041,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -4943,11 +5053,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A6,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -4960,11 +5070,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -4972,11 +5082,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4984,11 +5094,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -4996,11 +5106,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A7,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5013,11 +5123,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5025,11 +5135,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5037,11 +5147,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5049,11 +5159,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A8,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5066,11 +5176,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5078,11 +5188,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5090,11 +5200,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5102,11 +5212,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A9,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5119,11 +5229,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5131,11 +5241,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5143,11 +5253,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5155,11 +5265,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A10,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5172,11 +5282,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5184,11 +5294,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5196,11 +5306,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5208,11 +5318,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A11,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5225,11 +5335,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5237,11 +5347,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5249,11 +5359,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5261,11 +5371,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A12,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5278,11 +5388,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5290,11 +5400,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5302,11 +5412,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5314,11 +5424,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A13,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5331,11 +5441,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5343,11 +5453,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5355,11 +5465,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5367,11 +5477,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A14,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5384,11 +5494,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5396,11 +5506,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5408,11 +5518,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5420,11 +5530,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A15,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5437,11 +5547,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5449,11 +5559,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5461,11 +5571,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5473,11 +5583,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A16,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5490,11 +5600,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5502,11 +5612,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5514,11 +5624,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5526,11 +5636,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A17,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -5543,11 +5653,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -5555,11 +5665,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -5567,11 +5677,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -5579,11 +5689,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A18,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -5596,11 +5706,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$79,Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$79,Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -5608,11 +5718,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$79,Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$79,Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -5620,11 +5730,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$79,Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$79,Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -5632,11 +5742,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$79,$A19,Meals!$M$5:$M$79,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">

</xml_diff>

<commit_message>
Record the 09-19 weigh-in: 89.45, and flag the widening trend gap
The fitted line is now -0.560 kg/wk against -0.456 predicted from the
food log - a gap of ~114 kcal/day, up from 0.05 kg/wk two readings ago.

Candidates: photo estimates ~5% high, maintenance above 2,669 with
activity rising, or remaining water noise. Not unlogged whey, which
would push the fit the other way. No target change until another week
of data.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -5768,7 +5768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5997,8 +5997,33 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="27" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B12" s="24" t="n">
+        <v>89.45</v>
+      </c>
+      <c r="C12" s="25">
+        <f>B12-B11</f>
+        <v/>
+      </c>
+      <c r="D12" s="25">
+        <f>B12-$B$5</f>
+        <v/>
+      </c>
+      <c r="E12" s="26">
+        <f>AVERAGE(B6:B12)</f>
+        <v/>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Morning weigh-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="27" t="inlineStr">
         <is>
           <t>A drop in the first week is mostly water and glycogen, not fat. Judge the trend over 2-3 weeks, and change the activity multiplier on Targets only then.</t>
         </is>

</xml_diff>

<commit_message>
Log Day 16 breakfast and plan Saturday
Saturday is one of the two tight days at 2,100 kcal as served. Using the
leftover grilled chicken at dinner lands the day exactly on target at
133.75 g of protein with a single scoop - and it is day three of the
3-4 day refrigerated window, so today or never.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N81"/>
+  <dimension ref="A1:N82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4846,6 +4846,61 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="4" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>2 set dosa + vegetable sambar + red chutney (no white chutney)</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>480</v>
+      </c>
+      <c r="E82" s="7" t="n">
+        <v>710</v>
+      </c>
+      <c r="F82" s="8">
+        <f>AVERAGE(D82:E82)</f>
+        <v/>
+      </c>
+      <c r="G82" s="9" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H82" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="I82" s="10">
+        <f>AVERAGE(G82:H82)</f>
+        <v/>
+      </c>
+      <c r="J82" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="K82" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="L82" s="10">
+        <f>AVERAGE(J82:K82)</f>
+        <v/>
+      </c>
+      <c r="M82" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N82" s="6" t="inlineStr">
+        <is>
+          <t>Eaten out; generous sambar poured over both dosa</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -4860,7 +4915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4964,11 +5019,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -4976,11 +5031,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4988,11 +5043,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5000,11 +5055,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A5,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5017,11 +5072,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5029,11 +5084,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5041,11 +5096,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5053,11 +5108,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A6,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5070,11 +5125,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5082,11 +5137,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5094,11 +5149,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5106,11 +5161,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A7,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5123,11 +5178,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5135,11 +5190,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5147,11 +5202,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5159,11 +5214,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A8,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5176,11 +5231,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5188,11 +5243,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5200,11 +5255,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5212,11 +5267,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A9,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5229,11 +5284,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5241,11 +5296,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5253,11 +5308,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5265,11 +5320,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A10,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5282,11 +5337,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5294,11 +5349,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5306,11 +5361,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5318,11 +5373,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A11,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5335,11 +5390,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5347,11 +5402,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5359,11 +5414,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5371,11 +5426,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A12,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5388,11 +5443,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5400,11 +5455,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5412,11 +5467,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5424,11 +5479,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A13,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5441,11 +5496,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5453,11 +5508,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5465,11 +5520,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5477,11 +5532,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A14,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5494,11 +5549,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5506,11 +5561,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5518,11 +5573,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5530,11 +5585,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A15,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5547,11 +5602,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5559,11 +5614,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5571,11 +5626,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5583,11 +5638,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A16,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5600,11 +5655,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5612,11 +5667,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5624,11 +5679,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5636,11 +5691,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A17,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -5653,11 +5708,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -5665,11 +5720,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -5677,11 +5732,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -5689,11 +5744,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A18,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -5706,11 +5761,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$81,Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$81,Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -5718,11 +5773,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$81,Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$81,Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -5730,11 +5785,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$81,Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$81,Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -5742,15 +5797,68 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$81,$A19,Meals!$M$5:$M$81,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
         <f>D19-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B20" s="21">
+        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"logged")</f>
+        <v/>
+      </c>
+      <c r="C20" s="21">
+        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"logged")</f>
+        <v/>
+      </c>
+      <c r="D20" s="21">
+        <f>AVERAGE(B20:C20)</f>
+        <v/>
+      </c>
+      <c r="E20" s="22">
+        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"logged")</f>
+        <v/>
+      </c>
+      <c r="F20" s="22">
+        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"logged")</f>
+        <v/>
+      </c>
+      <c r="G20" s="22">
+        <f>AVERAGE(E20:F20)</f>
+        <v/>
+      </c>
+      <c r="H20" s="22">
+        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"logged")</f>
+        <v/>
+      </c>
+      <c r="I20" s="22">
+        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"logged")</f>
+        <v/>
+      </c>
+      <c r="J20" s="22">
+        <f>AVERAGE(H20:I20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"logged")</f>
+        <v/>
+      </c>
+      <c r="L20" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"pending")</f>
+        <v/>
+      </c>
+      <c r="M20" s="23">
+        <f>D20-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -6784,7 +6892,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$19)</f>
+        <f>COUNT(Daily!$A$5:$A$20)</f>
         <v/>
       </c>
     </row>
@@ -6795,7 +6903,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$19),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$20),0)</f>
         <v/>
       </c>
     </row>
@@ -6806,7 +6914,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$19),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$20),0)</f>
         <v/>
       </c>
     </row>
@@ -6817,7 +6925,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$19),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$20),0)</f>
         <v/>
       </c>
     </row>
@@ -6861,7 +6969,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$19,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$20,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -6872,7 +6980,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$19)</f>
+        <f>SUM(Daily!$L$5:$L$20)</f>
         <v/>
       </c>
     </row>
@@ -6923,19 +7031,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$19,"&gt;="&amp;$A17,Daily!$A$5:$A$19,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$20,"&gt;="&amp;$A17,Daily!$A$5:$A$20,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$19,Daily!$A$5:$A$19,"&gt;="&amp;$A17,Daily!$A$5:$A$19,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$20,Daily!$A$5:$A$20,"&gt;="&amp;$A17,Daily!$A$5:$A$20,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$19,Daily!$A$5:$A$19,"&gt;="&amp;$A17,Daily!$A$5:$A$19,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$20,Daily!$A$5:$A$20,"&gt;="&amp;$A17,Daily!$A$5:$A$20,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$19,Daily!$A$5:$A$19,"&gt;="&amp;$A17,Daily!$A$5:$A$19,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$20,Daily!$A$5:$A$20,"&gt;="&amp;$A17,Daily!$A$5:$A$20,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -6947,19 +7055,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$19,"&gt;="&amp;$A18,Daily!$A$5:$A$19,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$20,"&gt;="&amp;$A18,Daily!$A$5:$A$20,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$19,Daily!$A$5:$A$19,"&gt;="&amp;$A18,Daily!$A$5:$A$19,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$20,Daily!$A$5:$A$20,"&gt;="&amp;$A18,Daily!$A$5:$A$20,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$19,Daily!$A$5:$A$19,"&gt;="&amp;$A18,Daily!$A$5:$A$19,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$20,Daily!$A$5:$A$20,"&gt;="&amp;$A18,Daily!$A$5:$A$20,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$19,Daily!$A$5:$A$19,"&gt;="&amp;$A18,Daily!$A$5:$A$19,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$20,Daily!$A$5:$A$20,"&gt;="&amp;$A18,Daily!$A$5:$A$20,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -6971,19 +7079,19 @@
         <v>46285</v>
       </c>
       <c r="C19" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$19,"&gt;="&amp;$A19,Daily!$A$5:$A$19,"&lt;="&amp;$B19)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$20,"&gt;="&amp;$A19,Daily!$A$5:$A$20,"&lt;="&amp;$B19)</f>
         <v/>
       </c>
       <c r="D19" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$19,Daily!$A$5:$A$19,"&gt;="&amp;$A19,Daily!$A$5:$A$19,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$20,Daily!$A$5:$A$20,"&gt;="&amp;$A19,Daily!$A$5:$A$20,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$19,Daily!$A$5:$A$19,"&gt;="&amp;$A19,Daily!$A$5:$A$19,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$20,Daily!$A$5:$A$20,"&gt;="&amp;$A19,Daily!$A$5:$A$20,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$19,Daily!$A$5:$A$19,"&gt;="&amp;$A19,Daily!$A$5:$A$19,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$20,Daily!$A$5:$A$20,"&gt;="&amp;$A19,Daily!$A$5:$A$20,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
     </row>
@@ -7034,19 +7142,19 @@
         <v>46295</v>
       </c>
       <c r="C23" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$19,"&gt;="&amp;$A23,Daily!$A$5:$A$19,"&lt;="&amp;$B23)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$20,"&gt;="&amp;$A23,Daily!$A$5:$A$20,"&lt;="&amp;$B23)</f>
         <v/>
       </c>
       <c r="D23" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$19,Daily!$A$5:$A$19,"&gt;="&amp;$A23,Daily!$A$5:$A$19,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$20,Daily!$A$5:$A$20,"&gt;="&amp;$A23,Daily!$A$5:$A$20,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$19,Daily!$A$5:$A$19,"&gt;="&amp;$A23,Daily!$A$5:$A$19,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$20,Daily!$A$5:$A$20,"&gt;="&amp;$A23,Daily!$A$5:$A$20,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$19,Daily!$A$5:$A$19,"&gt;="&amp;$A23,Daily!$A$5:$A$19,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$20,Daily!$A$5:$A$20,"&gt;="&amp;$A23,Daily!$A$5:$A$20,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Day 16 lunch: first all-vegetarian mess plate of the sixteen days
742 kcal for 23.5 g of protein - 3.2 g per 100 kcal, below the mess
weekly average, because no fried fish or chicken piece was on the plate.
That leaves 90 g of protein for the evening.

Lands on the leftover grilled chicken plus two scoops: 148.75 g and a
451 deficit, which is corrective given the fitted trend is already
running ahead of prediction.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N82"/>
+  <dimension ref="A1:N83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4898,6 +4898,61 @@
       <c r="N82" s="6" t="inlineStr">
         <is>
           <t>Eaten out; generous sambar poured over both dosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>Mess meals plate (rice halved) + sambar, pappadam, cabbage thoran, veg curry, curd</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="n">
+        <v>575</v>
+      </c>
+      <c r="E83" s="7" t="n">
+        <v>910</v>
+      </c>
+      <c r="F83" s="8">
+        <f>AVERAGE(D83:E83)</f>
+        <v/>
+      </c>
+      <c r="G83" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="H83" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="I83" s="10">
+        <f>AVERAGE(G83:H83)</f>
+        <v/>
+      </c>
+      <c r="J83" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="K83" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="L83" s="10">
+        <f>AVERAGE(J83:K83)</f>
+        <v/>
+      </c>
+      <c r="M83" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N83" s="6" t="inlineStr">
+        <is>
+          <t>No fish or meat on the plate - first all-vegetarian mess lunch logged</t>
         </is>
       </c>
     </row>
@@ -5019,11 +5074,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5031,11 +5086,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5043,11 +5098,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5055,11 +5110,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A5,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5072,11 +5127,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5084,11 +5139,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5096,11 +5151,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5108,11 +5163,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A6,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5125,11 +5180,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5137,11 +5192,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5149,11 +5204,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5161,11 +5216,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A7,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5178,11 +5233,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5190,11 +5245,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5202,11 +5257,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5214,11 +5269,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A8,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5231,11 +5286,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5243,11 +5298,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5255,11 +5310,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5267,11 +5322,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A9,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5284,11 +5339,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5296,11 +5351,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5308,11 +5363,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5320,11 +5375,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A10,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5337,11 +5392,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5349,11 +5404,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5361,11 +5416,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5373,11 +5428,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A11,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5390,11 +5445,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5402,11 +5457,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5414,11 +5469,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5426,11 +5481,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A12,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5443,11 +5498,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5455,11 +5510,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5467,11 +5522,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5479,11 +5534,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A13,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5496,11 +5551,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5508,11 +5563,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5520,11 +5575,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5532,11 +5587,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A14,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5549,11 +5604,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5561,11 +5616,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5573,11 +5628,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5585,11 +5640,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A15,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5602,11 +5657,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5614,11 +5669,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5626,11 +5681,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5638,11 +5693,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A16,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5655,11 +5710,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5667,11 +5722,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5679,11 +5734,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5691,11 +5746,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A17,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -5708,11 +5763,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -5720,11 +5775,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -5732,11 +5787,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -5744,11 +5799,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A18,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -5761,11 +5816,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -5773,11 +5828,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -5785,11 +5840,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -5797,11 +5852,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A19,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -5814,11 +5869,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$82,Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$82,Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -5826,11 +5881,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$82,Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$82,Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -5838,11 +5893,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$82,Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$82,Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -5850,11 +5905,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$82,$A20,Meals!$M$5:$M$82,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">

</xml_diff>

<commit_message>
Correct Day 16 lunch: the flat item was a 1-egg omelette, not pappadam
+45 kcal, +4.5 g protein, +4.5 g fat. Retires the "first all-vegetarian
plate" reading - at 3.6 g of protein per 100 kcal the plate is at the
mess average, not below it.

The evening now needs one scoop rather than two: 2,148 kcal and 130.75 g,
27 over target.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -4912,34 +4912,34 @@
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate (rice halved) + sambar, pappadam, cabbage thoran, veg curry, curd</t>
+          <t>Mess meals plate (rice halved) + 1-egg omelette + sambar, cabbage thoran, veg curry, curd</t>
         </is>
       </c>
       <c r="D83" s="7" t="n">
-        <v>575</v>
+        <v>615</v>
       </c>
       <c r="E83" s="7" t="n">
-        <v>910</v>
+        <v>960</v>
       </c>
       <c r="F83" s="8">
         <f>AVERAGE(D83:E83)</f>
         <v/>
       </c>
       <c r="G83" s="9" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="H83" s="9" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="I83" s="10">
         <f>AVERAGE(G83:H83)</f>
         <v/>
       </c>
       <c r="J83" s="9" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K83" s="9" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="L83" s="10">
         <f>AVERAGE(J83:K83)</f>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="N83" s="6" t="inlineStr">
         <is>
-          <t>No fish or meat on the plate - first all-vegetarian mess lunch logged</t>
+          <t>Corrected - the flat item was a thin 1-egg omelette</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Day 16 whey (1.5 scoops) and close the evening on the chicken
565 kcal to target and 52 g of protein to the floor, both covered by
200 g of the leftover grilled chicken with two chapati: 2,205 kcal,
142 g of protein, a 464 deficit. No further whey needed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N83"/>
+  <dimension ref="A1:N84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4953,6 +4953,61 @@
       <c r="N83" s="6" t="inlineStr">
         <is>
           <t>Corrected - the flat item was a thin 1-egg omelette</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1.5 whey scoops</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="E84" s="7" t="n">
+        <v>195</v>
+      </c>
+      <c r="F84" s="8">
+        <f>AVERAGE(D84:E84)</f>
+        <v/>
+      </c>
+      <c r="G84" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="H84" s="9" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="I84" s="10">
+        <f>AVERAGE(G84:H84)</f>
+        <v/>
+      </c>
+      <c r="J84" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K84" s="9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L84" s="10">
+        <f>AVERAGE(J84:K84)</f>
+        <v/>
+      </c>
+      <c r="M84" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N84" s="6" t="inlineStr">
+        <is>
+          <t>Scoop 1 and a half</t>
         </is>
       </c>
     </row>
@@ -5074,11 +5129,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5086,11 +5141,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5098,11 +5153,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5110,11 +5165,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A5,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5127,11 +5182,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5139,11 +5194,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5151,11 +5206,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5163,11 +5218,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A6,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5180,11 +5235,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5192,11 +5247,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5204,11 +5259,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5216,11 +5271,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A7,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5233,11 +5288,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5245,11 +5300,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5257,11 +5312,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5269,11 +5324,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A8,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5286,11 +5341,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5298,11 +5353,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5310,11 +5365,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5322,11 +5377,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A9,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5339,11 +5394,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5351,11 +5406,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5363,11 +5418,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5375,11 +5430,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A10,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5392,11 +5447,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5404,11 +5459,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5416,11 +5471,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5428,11 +5483,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A11,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5445,11 +5500,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5457,11 +5512,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5469,11 +5524,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5481,11 +5536,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A12,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5498,11 +5553,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5510,11 +5565,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5522,11 +5577,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5534,11 +5589,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A13,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5551,11 +5606,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5563,11 +5618,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5575,11 +5630,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5587,11 +5642,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A14,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5604,11 +5659,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5616,11 +5671,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5628,11 +5683,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5640,11 +5695,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A15,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5657,11 +5712,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5669,11 +5724,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5681,11 +5736,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5693,11 +5748,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A16,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5710,11 +5765,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5722,11 +5777,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5734,11 +5789,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5746,11 +5801,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A17,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -5763,11 +5818,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -5775,11 +5830,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -5787,11 +5842,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -5799,11 +5854,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A18,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -5816,11 +5871,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -5828,11 +5883,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -5840,11 +5895,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -5852,11 +5907,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A19,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -5869,11 +5924,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$83,Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$83,Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -5881,11 +5936,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$83,Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$83,Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -5893,11 +5948,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$83,Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$83,Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -5905,11 +5960,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$83,$A20,Meals!$M$5:$M$83,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">

</xml_diff>

<commit_message>
Close Day 16 at 2,349 kcal and 140.25 g of protein
Dinner ran ~145 over plan on a larger chicken piece plus a curry
container and a boiled egg. A 320 deficit is corrective while the fitted
scale trend runs ahead of the food log's prediction.

Sixteen days: 2,179 kcal, 114.4 g protein, 490 deficit, 0.45 kg/week.
The last four protein days read 141, 181, 92, 140 - the one miss is the
day the closing scoops went unconfirmed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N84"/>
+  <dimension ref="A1:N85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4907,39 +4907,39 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate (rice halved) + 1-egg omelette + sambar, cabbage thoran, veg curry, curd</t>
+          <t>Grilled chicken piece + chicken curry + 2 chapati + 1 boiled egg</t>
         </is>
       </c>
       <c r="D83" s="7" t="n">
-        <v>615</v>
+        <v>650</v>
       </c>
       <c r="E83" s="7" t="n">
-        <v>960</v>
+        <v>938</v>
       </c>
       <c r="F83" s="8">
         <f>AVERAGE(D83:E83)</f>
         <v/>
       </c>
       <c r="G83" s="9" t="n">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="H83" s="9" t="n">
-        <v>33</v>
+        <v>72.5</v>
       </c>
       <c r="I83" s="10">
         <f>AVERAGE(G83:H83)</f>
         <v/>
       </c>
       <c r="J83" s="9" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="K83" s="9" t="n">
-        <v>47</v>
+        <v>48.5</v>
       </c>
       <c r="L83" s="10">
         <f>AVERAGE(J83:K83)</f>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="N83" s="6" t="inlineStr">
         <is>
-          <t>Corrected - the flat item was a thin 1-egg omelette</t>
+          <t>Sprite can in the photo not identified - counted as zero-sugar</t>
         </is>
       </c>
     </row>
@@ -4962,39 +4962,39 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>Black coffee + 1.5 whey scoops</t>
+          <t>Mess meals plate (rice halved) + 1-egg omelette + sambar, cabbage thoran, veg curry, curd</t>
         </is>
       </c>
       <c r="D84" s="7" t="n">
-        <v>150</v>
+        <v>615</v>
       </c>
       <c r="E84" s="7" t="n">
-        <v>195</v>
+        <v>960</v>
       </c>
       <c r="F84" s="8">
         <f>AVERAGE(D84:E84)</f>
         <v/>
       </c>
       <c r="G84" s="9" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="H84" s="9" t="n">
-        <v>37.5</v>
+        <v>33</v>
       </c>
       <c r="I84" s="10">
         <f>AVERAGE(G84:H84)</f>
         <v/>
       </c>
       <c r="J84" s="9" t="n">
-        <v>1.5</v>
+        <v>26</v>
       </c>
       <c r="K84" s="9" t="n">
-        <v>4.5</v>
+        <v>47</v>
       </c>
       <c r="L84" s="10">
         <f>AVERAGE(J84:K84)</f>
@@ -5006,6 +5006,61 @@
         </is>
       </c>
       <c r="N84" s="6" t="inlineStr">
+        <is>
+          <t>Corrected - the flat item was a thin 1-egg omelette</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1.5 whey scoops</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="E85" s="7" t="n">
+        <v>195</v>
+      </c>
+      <c r="F85" s="8">
+        <f>AVERAGE(D85:E85)</f>
+        <v/>
+      </c>
+      <c r="G85" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="H85" s="9" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="I85" s="10">
+        <f>AVERAGE(G85:H85)</f>
+        <v/>
+      </c>
+      <c r="J85" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K85" s="9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L85" s="10">
+        <f>AVERAGE(J85:K85)</f>
+        <v/>
+      </c>
+      <c r="M85" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N85" s="6" t="inlineStr">
         <is>
           <t>Scoop 1 and a half</t>
         </is>
@@ -5129,11 +5184,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5141,11 +5196,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5153,11 +5208,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5165,11 +5220,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A5,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5182,11 +5237,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5194,11 +5249,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5206,11 +5261,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5218,11 +5273,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A6,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5235,11 +5290,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5247,11 +5302,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5259,11 +5314,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5271,11 +5326,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A7,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5288,11 +5343,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5300,11 +5355,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5312,11 +5367,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5324,11 +5379,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A8,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5341,11 +5396,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5353,11 +5408,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5365,11 +5420,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5377,11 +5432,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A9,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5394,11 +5449,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5406,11 +5461,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5418,11 +5473,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5430,11 +5485,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A10,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5447,11 +5502,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5459,11 +5514,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5471,11 +5526,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5483,11 +5538,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A11,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5500,11 +5555,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5512,11 +5567,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5524,11 +5579,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5536,11 +5591,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A12,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5553,11 +5608,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5565,11 +5620,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5577,11 +5632,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5589,11 +5644,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A13,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5606,11 +5661,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5618,11 +5673,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5630,11 +5685,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5642,11 +5697,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A14,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5659,11 +5714,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5671,11 +5726,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5683,11 +5738,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5695,11 +5750,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A15,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5712,11 +5767,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5724,11 +5779,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5736,11 +5791,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5748,11 +5803,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A16,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5765,11 +5820,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5777,11 +5832,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5789,11 +5844,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5801,11 +5856,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A17,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -5818,11 +5873,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -5830,11 +5885,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -5842,11 +5897,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -5854,11 +5909,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A18,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -5871,11 +5926,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -5883,11 +5938,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -5895,11 +5950,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -5907,11 +5962,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A19,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -5924,11 +5979,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$84,Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$84,Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -5936,11 +5991,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$84,Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$84,Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -5948,11 +6003,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$84,Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$84,Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -5960,11 +6015,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$84,$A20,Meals!$M$5:$M$84,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">

</xml_diff>

<commit_message>
Log Day 17 breakfast: one porotta instead of two
Saves ~205 kcal for ~4 g of protein, taken without prompting.

That makes today the one day not to halve the ghee rice: leaving it
whole lands 10 over target at 152 g of protein and ~83.5 g of fat, where
halving it produces a 729 deficit while the fitted scale trend is
already outrunning the food log.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N85"/>
+  <dimension ref="A1:N86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5066,6 +5066,61 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="4" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>1 porotta + kadala curry</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="n">
+        <v>360</v>
+      </c>
+      <c r="E86" s="7" t="n">
+        <v>550</v>
+      </c>
+      <c r="F86" s="8">
+        <f>AVERAGE(D86:E86)</f>
+        <v/>
+      </c>
+      <c r="G86" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H86" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="I86" s="10">
+        <f>AVERAGE(G86:H86)</f>
+        <v/>
+      </c>
+      <c r="J86" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="K86" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="L86" s="10">
+        <f>AVERAGE(J86:K86)</f>
+        <v/>
+      </c>
+      <c r="M86" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N86" s="6" t="inlineStr">
+        <is>
+          <t>Took 1 porotta rather than the menu's 2 - saves ~205 kcal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -5080,7 +5135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5184,11 +5239,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5196,11 +5251,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5208,11 +5263,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5220,11 +5275,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A5,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5237,11 +5292,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5249,11 +5304,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5261,11 +5316,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5273,11 +5328,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A6,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5290,11 +5345,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5302,11 +5357,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5314,11 +5369,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5326,11 +5381,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A7,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5343,11 +5398,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5355,11 +5410,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5367,11 +5422,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5379,11 +5434,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A8,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5396,11 +5451,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5408,11 +5463,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5420,11 +5475,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5432,11 +5487,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A9,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5449,11 +5504,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5461,11 +5516,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5473,11 +5528,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5485,11 +5540,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A10,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5502,11 +5557,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5514,11 +5569,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5526,11 +5581,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5538,11 +5593,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A11,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5555,11 +5610,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5567,11 +5622,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5579,11 +5634,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5591,11 +5646,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A12,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5608,11 +5663,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5620,11 +5675,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5632,11 +5687,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5644,11 +5699,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A13,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5661,11 +5716,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5673,11 +5728,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5685,11 +5740,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5697,11 +5752,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A14,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5714,11 +5769,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5726,11 +5781,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5738,11 +5793,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5750,11 +5805,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A15,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5767,11 +5822,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5779,11 +5834,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5791,11 +5846,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5803,11 +5858,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A16,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5820,11 +5875,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5832,11 +5887,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5844,11 +5899,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5856,11 +5911,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A17,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -5873,11 +5928,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -5885,11 +5940,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -5897,11 +5952,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -5909,11 +5964,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A18,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -5926,11 +5981,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -5938,11 +5993,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -5950,11 +6005,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -5962,11 +6017,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A19,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -5979,11 +6034,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$85,Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$85,Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -5991,11 +6046,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$85,Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$85,Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6003,11 +6058,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$85,Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$85,Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6015,15 +6070,68 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$85,$A20,Meals!$M$5:$M$85,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
         <f>D20-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B21" s="8">
+        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"logged")</f>
+        <v/>
+      </c>
+      <c r="C21" s="8">
+        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"logged")</f>
+        <v/>
+      </c>
+      <c r="D21" s="8">
+        <f>AVERAGE(B21:C21)</f>
+        <v/>
+      </c>
+      <c r="E21" s="10">
+        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"logged")</f>
+        <v/>
+      </c>
+      <c r="F21" s="10">
+        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"logged")</f>
+        <v/>
+      </c>
+      <c r="G21" s="10">
+        <f>AVERAGE(E21:F21)</f>
+        <v/>
+      </c>
+      <c r="H21" s="10">
+        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"logged")</f>
+        <v/>
+      </c>
+      <c r="I21" s="10">
+        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"logged")</f>
+        <v/>
+      </c>
+      <c r="J21" s="10">
+        <f>AVERAGE(H21:I21)</f>
+        <v/>
+      </c>
+      <c r="K21" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"logged")</f>
+        <v/>
+      </c>
+      <c r="L21" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"pending")</f>
+        <v/>
+      </c>
+      <c r="M21" s="19">
+        <f>D21-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -7057,7 +7165,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$20)</f>
+        <f>COUNT(Daily!$A$5:$A$21)</f>
         <v/>
       </c>
     </row>
@@ -7068,7 +7176,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$20),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$21),0)</f>
         <v/>
       </c>
     </row>
@@ -7079,7 +7187,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$20),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$21),0)</f>
         <v/>
       </c>
     </row>
@@ -7090,7 +7198,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$20),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$21),0)</f>
         <v/>
       </c>
     </row>
@@ -7134,7 +7242,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$20,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$21,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -7145,7 +7253,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$20)</f>
+        <f>SUM(Daily!$L$5:$L$21)</f>
         <v/>
       </c>
     </row>
@@ -7196,19 +7304,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$20,"&gt;="&amp;$A17,Daily!$A$5:$A$20,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$21,"&gt;="&amp;$A17,Daily!$A$5:$A$21,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$20,Daily!$A$5:$A$20,"&gt;="&amp;$A17,Daily!$A$5:$A$20,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$21,Daily!$A$5:$A$21,"&gt;="&amp;$A17,Daily!$A$5:$A$21,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$20,Daily!$A$5:$A$20,"&gt;="&amp;$A17,Daily!$A$5:$A$20,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$21,Daily!$A$5:$A$21,"&gt;="&amp;$A17,Daily!$A$5:$A$21,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$20,Daily!$A$5:$A$20,"&gt;="&amp;$A17,Daily!$A$5:$A$20,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$21,Daily!$A$5:$A$21,"&gt;="&amp;$A17,Daily!$A$5:$A$21,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -7220,19 +7328,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$20,"&gt;="&amp;$A18,Daily!$A$5:$A$20,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$21,"&gt;="&amp;$A18,Daily!$A$5:$A$21,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$20,Daily!$A$5:$A$20,"&gt;="&amp;$A18,Daily!$A$5:$A$20,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$21,Daily!$A$5:$A$21,"&gt;="&amp;$A18,Daily!$A$5:$A$21,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$20,Daily!$A$5:$A$20,"&gt;="&amp;$A18,Daily!$A$5:$A$20,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$21,Daily!$A$5:$A$21,"&gt;="&amp;$A18,Daily!$A$5:$A$21,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$20,Daily!$A$5:$A$20,"&gt;="&amp;$A18,Daily!$A$5:$A$20,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$21,Daily!$A$5:$A$21,"&gt;="&amp;$A18,Daily!$A$5:$A$21,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -7244,19 +7352,19 @@
         <v>46285</v>
       </c>
       <c r="C19" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$20,"&gt;="&amp;$A19,Daily!$A$5:$A$20,"&lt;="&amp;$B19)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$21,"&gt;="&amp;$A19,Daily!$A$5:$A$21,"&lt;="&amp;$B19)</f>
         <v/>
       </c>
       <c r="D19" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$20,Daily!$A$5:$A$20,"&gt;="&amp;$A19,Daily!$A$5:$A$20,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$21,Daily!$A$5:$A$21,"&gt;="&amp;$A19,Daily!$A$5:$A$21,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$20,Daily!$A$5:$A$20,"&gt;="&amp;$A19,Daily!$A$5:$A$20,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$21,Daily!$A$5:$A$21,"&gt;="&amp;$A19,Daily!$A$5:$A$21,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$20,Daily!$A$5:$A$20,"&gt;="&amp;$A19,Daily!$A$5:$A$20,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$21,Daily!$A$5:$A$21,"&gt;="&amp;$A19,Daily!$A$5:$A$21,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
     </row>
@@ -7307,19 +7415,19 @@
         <v>46295</v>
       </c>
       <c r="C23" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$20,"&gt;="&amp;$A23,Daily!$A$5:$A$20,"&lt;="&amp;$B23)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$21,"&gt;="&amp;$A23,Daily!$A$5:$A$21,"&lt;="&amp;$B23)</f>
         <v/>
       </c>
       <c r="D23" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$20,Daily!$A$5:$A$20,"&gt;="&amp;$A23,Daily!$A$5:$A$20,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$21,Daily!$A$5:$A$21,"&gt;="&amp;$A23,Daily!$A$5:$A$21,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$20,Daily!$A$5:$A$20,"&gt;="&amp;$A23,Daily!$A$5:$A$20,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$21,Daily!$A$5:$A$21,"&gt;="&amp;$A23,Daily!$A$5:$A$21,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$20,Daily!$A$5:$A$20,"&gt;="&amp;$A23,Daily!$A$5:$A$20,"&lt;="&amp;$B23),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$21,Daily!$A$5:$A$21,"&gt;="&amp;$A23,Daily!$A$5:$A$21,"&lt;="&amp;$B23),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Day 17 lunch: halved ghee rice with chicken curry
The rice was halved against this morning's suggestion, which is the
better call: the same 190 kcal spent on whey and eggs buys ~35 g of
protein rather than the rice's ~3 g.

Leaves 1,065 kcal and 85 g of protein for the evening - four scoops and
two eggs lands 7 under target at a 556 deficit.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N86"/>
+  <dimension ref="A1:N87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5118,6 +5118,61 @@
       <c r="N86" s="6" t="inlineStr">
         <is>
           <t>Took 1 porotta rather than the menu's 2 - saves ~205 kcal</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>Ghee rice (halved) + chicken curry + curd</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="n">
+        <v>490</v>
+      </c>
+      <c r="E87" s="7" t="n">
+        <v>710</v>
+      </c>
+      <c r="F87" s="8">
+        <f>AVERAGE(D87:E87)</f>
+        <v/>
+      </c>
+      <c r="G87" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="H87" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I87" s="10">
+        <f>AVERAGE(G87:H87)</f>
+        <v/>
+      </c>
+      <c r="J87" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="K87" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="L87" s="10">
+        <f>AVERAGE(J87:K87)</f>
+        <v/>
+      </c>
+      <c r="M87" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N87" s="6" t="inlineStr">
+        <is>
+          <t>Rice halved despite the day having room for it</t>
         </is>
       </c>
     </row>
@@ -5239,11 +5294,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5251,11 +5306,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5263,11 +5318,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5275,11 +5330,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A5,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5292,11 +5347,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5304,11 +5359,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5316,11 +5371,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5328,11 +5383,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A6,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5345,11 +5400,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5357,11 +5412,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5369,11 +5424,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5381,11 +5436,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A7,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5398,11 +5453,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5410,11 +5465,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5422,11 +5477,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5434,11 +5489,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A8,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5451,11 +5506,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5463,11 +5518,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5475,11 +5530,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5487,11 +5542,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A9,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5504,11 +5559,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5516,11 +5571,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5528,11 +5583,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5540,11 +5595,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A10,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5557,11 +5612,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5569,11 +5624,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5581,11 +5636,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5593,11 +5648,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A11,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5610,11 +5665,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5622,11 +5677,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5634,11 +5689,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5646,11 +5701,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A12,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5663,11 +5718,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5675,11 +5730,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5687,11 +5742,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5699,11 +5754,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A13,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5716,11 +5771,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5728,11 +5783,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5740,11 +5795,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5752,11 +5807,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A14,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5769,11 +5824,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5781,11 +5836,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5793,11 +5848,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5805,11 +5860,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A15,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5822,11 +5877,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5834,11 +5889,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5846,11 +5901,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5858,11 +5913,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A16,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5875,11 +5930,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5887,11 +5942,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5899,11 +5954,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5911,11 +5966,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A17,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -5928,11 +5983,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -5940,11 +5995,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -5952,11 +6007,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -5964,11 +6019,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A18,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -5981,11 +6036,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -5993,11 +6048,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6005,11 +6060,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6017,11 +6072,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A19,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6034,11 +6089,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6046,11 +6101,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6058,11 +6113,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6070,11 +6125,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A20,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6087,11 +6142,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$86,Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$86,Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6099,11 +6154,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$86,Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$86,Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6111,11 +6166,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$86,Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$86,Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6123,11 +6178,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$86,$A21,Meals!$M$5:$M$86,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">

</xml_diff>

<commit_message>
Log Day 17 snack: parippu vada and milk coffee
~225 kcal for 8.75 g of protein. The evening drops from four scoops and
two eggs to three scoops and one.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N87"/>
+  <dimension ref="A1:N88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5173,6 +5173,61 @@
       <c r="N87" s="6" t="inlineStr">
         <is>
           <t>Rice halved despite the day having room for it</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>1 parippu vada + milk coffee (no sugar)</t>
+        </is>
+      </c>
+      <c r="D88" s="7" t="n">
+        <v>170</v>
+      </c>
+      <c r="E88" s="7" t="n">
+        <v>280</v>
+      </c>
+      <c r="F88" s="8">
+        <f>AVERAGE(D88:E88)</f>
+        <v/>
+      </c>
+      <c r="G88" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="H88" s="9" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="I88" s="10">
+        <f>AVERAGE(G88:H88)</f>
+        <v/>
+      </c>
+      <c r="J88" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="K88" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="L88" s="10">
+        <f>AVERAGE(J88:K88)</f>
+        <v/>
+      </c>
+      <c r="M88" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N88" s="6" t="inlineStr">
+        <is>
+          <t>First milk coffee logged - black coffee is ~2 kcal against this ~60</t>
         </is>
       </c>
     </row>
@@ -5294,11 +5349,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5306,11 +5361,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5318,11 +5373,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5330,11 +5385,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A5,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5347,11 +5402,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5359,11 +5414,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5371,11 +5426,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5383,11 +5438,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A6,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5400,11 +5455,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5412,11 +5467,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5424,11 +5479,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5436,11 +5491,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A7,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5453,11 +5508,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5465,11 +5520,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5477,11 +5532,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5489,11 +5544,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A8,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5506,11 +5561,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5518,11 +5573,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5530,11 +5585,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5542,11 +5597,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A9,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5559,11 +5614,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5571,11 +5626,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5583,11 +5638,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5595,11 +5650,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A10,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5612,11 +5667,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5624,11 +5679,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5636,11 +5691,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5648,11 +5703,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A11,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5665,11 +5720,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5677,11 +5732,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5689,11 +5744,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5701,11 +5756,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A12,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5718,11 +5773,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5730,11 +5785,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5742,11 +5797,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5754,11 +5809,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A13,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5771,11 +5826,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5783,11 +5838,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5795,11 +5850,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5807,11 +5862,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A14,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5824,11 +5879,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5836,11 +5891,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5848,11 +5903,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5860,11 +5915,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A15,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5877,11 +5932,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5889,11 +5944,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5901,11 +5956,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5913,11 +5968,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A16,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5930,11 +5985,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5942,11 +5997,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -5954,11 +6009,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -5966,11 +6021,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A17,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -5983,11 +6038,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -5995,11 +6050,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6007,11 +6062,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6019,11 +6074,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A18,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6036,11 +6091,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6048,11 +6103,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6060,11 +6115,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6072,11 +6127,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A19,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6089,11 +6144,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6101,11 +6156,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6113,11 +6168,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6125,11 +6180,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A20,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6142,11 +6197,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$87,Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$87,Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6154,11 +6209,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$87,Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$87,Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6166,11 +6221,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$87,Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$87,Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6178,11 +6233,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$87,$A21,Meals!$M$5:$M$87,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">

</xml_diff>

<commit_message>
Log Day 17 squid snack and add it to the reference table
~165 kcal for ~12 g of protein - 7.3 g per 100 kcal, double the mess
average and close to a boiled egg. Squid is very lean; the fat is
frying oil.

The evening drops to two scoops: 2,125 kcal, 131.75 g, a 544 deficit.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N88"/>
+  <dimension ref="A1:N89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5228,6 +5228,61 @@
       <c r="N88" s="6" t="inlineStr">
         <is>
           <t>First milk coffee logged - black coffee is ~2 kcal against this ~60</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="inlineStr">
+        <is>
+          <t>1 small stuffed squid (pan-fried)</t>
+        </is>
+      </c>
+      <c r="D89" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="E89" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="F89" s="8">
+        <f>AVERAGE(D89:E89)</f>
+        <v/>
+      </c>
+      <c r="G89" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H89" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="I89" s="10">
+        <f>AVERAGE(G89:H89)</f>
+        <v/>
+      </c>
+      <c r="J89" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="K89" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="L89" s="10">
+        <f>AVERAGE(J89:K89)</f>
+        <v/>
+      </c>
+      <c r="M89" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N89" s="6" t="inlineStr">
+        <is>
+          <t>7.3 g protein per 100 kcal - double the mess average</t>
         </is>
       </c>
     </row>
@@ -5349,11 +5404,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5361,11 +5416,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5373,11 +5428,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5385,11 +5440,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A5,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5402,11 +5457,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5414,11 +5469,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5426,11 +5481,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5438,11 +5493,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A6,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5455,11 +5510,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5467,11 +5522,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5479,11 +5534,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5491,11 +5546,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A7,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5508,11 +5563,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5520,11 +5575,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5532,11 +5587,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5544,11 +5599,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A8,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5561,11 +5616,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5573,11 +5628,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5585,11 +5640,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5597,11 +5652,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A9,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5614,11 +5669,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5626,11 +5681,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5638,11 +5693,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5650,11 +5705,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A10,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5667,11 +5722,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5679,11 +5734,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5691,11 +5746,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5703,11 +5758,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A11,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5720,11 +5775,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5732,11 +5787,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5744,11 +5799,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5756,11 +5811,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A12,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5773,11 +5828,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5785,11 +5840,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5797,11 +5852,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5809,11 +5864,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A13,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5826,11 +5881,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5838,11 +5893,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5850,11 +5905,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5862,11 +5917,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A14,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5879,11 +5934,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5891,11 +5946,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5903,11 +5958,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5915,11 +5970,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A15,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5932,11 +5987,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5944,11 +5999,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -5956,11 +6011,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -5968,11 +6023,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A16,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -5985,11 +6040,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -5997,11 +6052,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6009,11 +6064,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6021,11 +6076,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A17,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6038,11 +6093,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6050,11 +6105,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6062,11 +6117,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6074,11 +6129,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A18,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6091,11 +6146,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6103,11 +6158,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6115,11 +6170,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6127,11 +6182,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A19,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6144,11 +6199,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6156,11 +6211,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6168,11 +6223,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6180,11 +6235,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A20,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6197,11 +6252,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$88,Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$88,Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6209,11 +6264,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$88,Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$88,Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6221,11 +6276,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$88,Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$88,Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6233,11 +6288,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$88,$A21,Meals!$M$5:$M$88,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -8055,7 +8110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -9549,6 +9604,33 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>Stuffed squid - koonthal nirachathu (1 small)</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="C60" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="D60" s="8">
+        <f>AVERAGE(B60:C60)</f>
+        <v/>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>~10-14 g</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>7.3 g protein per 100 kcal. Squid itself is very lean; nearly all the fat is frying oil</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Log the Day 17 soup and turn the evening into a restaurant budget
580 kcal and 60.25 g of protein left with dinner still to be ordered.
Grilled or tandoori main plus one roti and a scoop lands at 2,190 and
151 g; a rice plate is the one shape that does not fit.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N89"/>
+  <dimension ref="A1:N90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5283,6 +5283,61 @@
       <c r="N89" s="6" t="inlineStr">
         <is>
           <t>7.3 g protein per 100 kcal - double the mess average</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="inlineStr">
+        <is>
+          <t>Clear soup (small bowl)</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="E90" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F90" s="8">
+        <f>AVERAGE(D90:E90)</f>
+        <v/>
+      </c>
+      <c r="G90" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H90" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I90" s="10">
+        <f>AVERAGE(G90:H90)</f>
+        <v/>
+      </c>
+      <c r="J90" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K90" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L90" s="10">
+        <f>AVERAGE(J90:K90)</f>
+        <v/>
+      </c>
+      <c r="M90" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N90" s="6" t="inlineStr">
+        <is>
+          <t>Restaurant starter; thin clear soup with a little oil on top</t>
         </is>
       </c>
     </row>
@@ -5404,11 +5459,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5416,11 +5471,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5428,11 +5483,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5440,11 +5495,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A5,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5457,11 +5512,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5469,11 +5524,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5481,11 +5536,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5493,11 +5548,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A6,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5510,11 +5565,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5522,11 +5577,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5534,11 +5589,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5546,11 +5601,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A7,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5563,11 +5618,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5575,11 +5630,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5587,11 +5642,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5599,11 +5654,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A8,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5616,11 +5671,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5628,11 +5683,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5640,11 +5695,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5652,11 +5707,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A9,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5669,11 +5724,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5681,11 +5736,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5693,11 +5748,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5705,11 +5760,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A10,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5722,11 +5777,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5734,11 +5789,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5746,11 +5801,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5758,11 +5813,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A11,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5775,11 +5830,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5787,11 +5842,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5799,11 +5854,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5811,11 +5866,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A12,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5828,11 +5883,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5840,11 +5895,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5852,11 +5907,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5864,11 +5919,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A13,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5881,11 +5936,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5893,11 +5948,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5905,11 +5960,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5917,11 +5972,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A14,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5934,11 +5989,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -5946,11 +6001,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -5958,11 +6013,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -5970,11 +6025,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A15,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -5987,11 +6042,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -5999,11 +6054,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6011,11 +6066,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6023,11 +6078,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A16,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6040,11 +6095,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6052,11 +6107,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6064,11 +6119,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6076,11 +6131,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A17,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6093,11 +6148,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6105,11 +6160,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6117,11 +6172,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6129,11 +6184,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A18,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6146,11 +6201,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6158,11 +6213,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6170,11 +6225,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6182,11 +6237,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A19,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6199,11 +6254,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6211,11 +6266,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6223,11 +6278,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6235,11 +6290,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A20,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6252,11 +6307,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$89,Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$89,Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6264,11 +6319,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$89,Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$89,Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6276,11 +6331,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$89,Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$89,Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6288,11 +6343,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$89,$A21,Meals!$M$5:$M$89,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">

</xml_diff>

<commit_message>
Log the Day 17 mint juice and revise the restaurant budget
~100 kcal of sugar for zero protein, which displaces the evening scoop.
480 kcal and 60 g of protein left: a grilled main plus one bread lands
at 2,175 and 130.5 g with no scoop needed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N90"/>
+  <dimension ref="A1:N91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5127,39 +5127,39 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Drink</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>Ghee rice (halved) + chicken curry + curd</t>
+          <t>Mint juice (small cup)</t>
         </is>
       </c>
       <c r="D87" s="7" t="n">
-        <v>490</v>
+        <v>60</v>
       </c>
       <c r="E87" s="7" t="n">
-        <v>710</v>
+        <v>140</v>
       </c>
       <c r="F87" s="8">
         <f>AVERAGE(D87:E87)</f>
         <v/>
       </c>
       <c r="G87" s="9" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="H87" s="9" t="n">
-        <v>36</v>
+        <v>0.5</v>
       </c>
       <c r="I87" s="10">
         <f>AVERAGE(G87:H87)</f>
         <v/>
       </c>
       <c r="J87" s="9" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="K87" s="9" t="n">
-        <v>36</v>
+        <v>0.5</v>
       </c>
       <c r="L87" s="10">
         <f>AVERAGE(J87:K87)</f>
@@ -5172,7 +5172,7 @@
       </c>
       <c r="N87" s="6" t="inlineStr">
         <is>
-          <t>Rice halved despite the day having room for it</t>
+          <t>Assumed sweetened - if unsweetened it is nearer 15 kcal</t>
         </is>
       </c>
     </row>
@@ -5182,39 +5182,39 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>1 parippu vada + milk coffee (no sugar)</t>
+          <t>Ghee rice (halved) + chicken curry + curd</t>
         </is>
       </c>
       <c r="D88" s="7" t="n">
-        <v>170</v>
+        <v>490</v>
       </c>
       <c r="E88" s="7" t="n">
-        <v>280</v>
+        <v>710</v>
       </c>
       <c r="F88" s="8">
         <f>AVERAGE(D88:E88)</f>
         <v/>
       </c>
       <c r="G88" s="9" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="H88" s="9" t="n">
-        <v>10.5</v>
+        <v>36</v>
       </c>
       <c r="I88" s="10">
         <f>AVERAGE(G88:H88)</f>
         <v/>
       </c>
       <c r="J88" s="9" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="K88" s="9" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="L88" s="10">
         <f>AVERAGE(J88:K88)</f>
@@ -5227,7 +5227,7 @@
       </c>
       <c r="N88" s="6" t="inlineStr">
         <is>
-          <t>First milk coffee logged - black coffee is ~2 kcal against this ~60</t>
+          <t>Rice halved despite the day having room for it</t>
         </is>
       </c>
     </row>
@@ -5242,34 +5242,34 @@
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>1 small stuffed squid (pan-fried)</t>
+          <t>1 parippu vada + milk coffee (no sugar)</t>
         </is>
       </c>
       <c r="D89" s="7" t="n">
-        <v>130</v>
+        <v>170</v>
       </c>
       <c r="E89" s="7" t="n">
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="F89" s="8">
         <f>AVERAGE(D89:E89)</f>
         <v/>
       </c>
       <c r="G89" s="9" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H89" s="9" t="n">
-        <v>14</v>
+        <v>10.5</v>
       </c>
       <c r="I89" s="10">
         <f>AVERAGE(G89:H89)</f>
         <v/>
       </c>
       <c r="J89" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K89" s="9" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L89" s="10">
         <f>AVERAGE(J89:K89)</f>
@@ -5282,7 +5282,7 @@
       </c>
       <c r="N89" s="6" t="inlineStr">
         <is>
-          <t>7.3 g protein per 100 kcal - double the mess average</t>
+          <t>First milk coffee logged - black coffee is ~2 kcal against this ~60</t>
         </is>
       </c>
     </row>
@@ -5297,34 +5297,34 @@
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>Clear soup (small bowl)</t>
+          <t>1 small stuffed squid (pan-fried)</t>
         </is>
       </c>
       <c r="D90" s="7" t="n">
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="E90" s="7" t="n">
-        <v>130</v>
+        <v>200</v>
       </c>
       <c r="F90" s="8">
         <f>AVERAGE(D90:E90)</f>
         <v/>
       </c>
       <c r="G90" s="9" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H90" s="9" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="I90" s="10">
         <f>AVERAGE(G90:H90)</f>
         <v/>
       </c>
       <c r="J90" s="9" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="K90" s="9" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="L90" s="10">
         <f>AVERAGE(J90:K90)</f>
@@ -5336,6 +5336,61 @@
         </is>
       </c>
       <c r="N90" s="6" t="inlineStr">
+        <is>
+          <t>7.3 g protein per 100 kcal - double the mess average</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>Clear soup (small bowl)</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="E91" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F91" s="8">
+        <f>AVERAGE(D91:E91)</f>
+        <v/>
+      </c>
+      <c r="G91" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H91" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I91" s="10">
+        <f>AVERAGE(G91:H91)</f>
+        <v/>
+      </c>
+      <c r="J91" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K91" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L91" s="10">
+        <f>AVERAGE(J91:K91)</f>
+        <v/>
+      </c>
+      <c r="M91" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N91" s="6" t="inlineStr">
         <is>
           <t>Restaurant starter; thin clear soup with a little oil on top</t>
         </is>
@@ -5459,11 +5514,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5471,11 +5526,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5483,11 +5538,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5495,11 +5550,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A5,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5512,11 +5567,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5524,11 +5579,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5536,11 +5591,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5548,11 +5603,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A6,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5565,11 +5620,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5577,11 +5632,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5589,11 +5644,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5601,11 +5656,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A7,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5618,11 +5673,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5630,11 +5685,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5642,11 +5697,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5654,11 +5709,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A8,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5671,11 +5726,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5683,11 +5738,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5695,11 +5750,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5707,11 +5762,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A9,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5724,11 +5779,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5736,11 +5791,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5748,11 +5803,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5760,11 +5815,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A10,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5777,11 +5832,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5789,11 +5844,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5801,11 +5856,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5813,11 +5868,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A11,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5830,11 +5885,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5842,11 +5897,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5854,11 +5909,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5866,11 +5921,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A12,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5883,11 +5938,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5895,11 +5950,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5907,11 +5962,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5919,11 +5974,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A13,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5936,11 +5991,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -5948,11 +6003,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -5960,11 +6015,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -5972,11 +6027,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A14,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -5989,11 +6044,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6001,11 +6056,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6013,11 +6068,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6025,11 +6080,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A15,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6042,11 +6097,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6054,11 +6109,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6066,11 +6121,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6078,11 +6133,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A16,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6095,11 +6150,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6107,11 +6162,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6119,11 +6174,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6131,11 +6186,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A17,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6148,11 +6203,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6160,11 +6215,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6172,11 +6227,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6184,11 +6239,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A18,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6201,11 +6256,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6213,11 +6268,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6225,11 +6280,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6237,11 +6292,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A19,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6254,11 +6309,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6266,11 +6321,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6278,11 +6333,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6290,11 +6345,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A20,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6307,11 +6362,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$90,Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$90,Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6319,11 +6374,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$90,Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$90,Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6331,11 +6386,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$90,Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$90,Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6343,11 +6398,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$90,$A21,Meals!$M$5:$M$90,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">

</xml_diff>

<commit_message>
Correct the Day 17 soup: one spoonful, not the bowl
~87 kcal back, which brings the closing scoop back into the budget: a
grilled main, one bread and one scoop lands at 2,203 and 149.25 g.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -5352,34 +5352,34 @@
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>Clear soup (small bowl)</t>
+          <t>Clear soup (one spoonful only)</t>
         </is>
       </c>
       <c r="D91" s="7" t="n">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="E91" s="7" t="n">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="F91" s="8">
         <f>AVERAGE(D91:E91)</f>
         <v/>
       </c>
       <c r="G91" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H91" s="9" t="n">
-        <v>6</v>
+        <v>0.5</v>
       </c>
       <c r="I91" s="10">
         <f>AVERAGE(G91:H91)</f>
         <v/>
       </c>
       <c r="J91" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K91" s="9" t="n">
-        <v>6</v>
+        <v>0.5</v>
       </c>
       <c r="L91" s="10">
         <f>AVERAGE(J91:K91)</f>
@@ -5392,7 +5392,7 @@
       </c>
       <c r="N91" s="6" t="inlineStr">
         <is>
-          <t>Restaurant starter; thin clear soup with a little oil on top</t>
+          <t>Corrected - only a spoonful was taken</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log one serving of the low-calorie gelato and add it to the reference
The 86 on the front is per serving, not per tub - a 500 ml tub is about
four servings, ~344 kcal. Also notes the oligofructose load in a whole
tub.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N91"/>
+  <dimension ref="A1:N92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5393,6 +5393,61 @@
       <c r="N91" s="6" t="inlineStr">
         <is>
           <t>Corrected - only a spoonful was taken</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>Brooklyn Creamery guilt-free gelato - coconut creme (1 serving)</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="E92" s="7" t="n">
+        <v>95</v>
+      </c>
+      <c r="F92" s="8">
+        <f>AVERAGE(D92:E92)</f>
+        <v/>
+      </c>
+      <c r="G92" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H92" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I92" s="10">
+        <f>AVERAGE(G92:H92)</f>
+        <v/>
+      </c>
+      <c r="J92" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K92" s="9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L92" s="10">
+        <f>AVERAGE(J92:K92)</f>
+        <v/>
+      </c>
+      <c r="M92" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N92" s="6" t="inlineStr">
+        <is>
+          <t>86 kcal is per serving; a 500 ml tub is about 4 servings</t>
         </is>
       </c>
     </row>
@@ -5514,11 +5569,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5526,11 +5581,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5538,11 +5593,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5550,11 +5605,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A5,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5567,11 +5622,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5579,11 +5634,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5591,11 +5646,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5603,11 +5658,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A6,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5620,11 +5675,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5632,11 +5687,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5644,11 +5699,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5656,11 +5711,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A7,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5673,11 +5728,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5685,11 +5740,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5697,11 +5752,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5709,11 +5764,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A8,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5726,11 +5781,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5738,11 +5793,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5750,11 +5805,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5762,11 +5817,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A9,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5779,11 +5834,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5791,11 +5846,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5803,11 +5858,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5815,11 +5870,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A10,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5832,11 +5887,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5844,11 +5899,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5856,11 +5911,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5868,11 +5923,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A11,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5885,11 +5940,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5897,11 +5952,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5909,11 +5964,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5921,11 +5976,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A12,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5938,11 +5993,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -5950,11 +6005,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -5962,11 +6017,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -5974,11 +6029,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A13,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -5991,11 +6046,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6003,11 +6058,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6015,11 +6070,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6027,11 +6082,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A14,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6044,11 +6099,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6056,11 +6111,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6068,11 +6123,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6080,11 +6135,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A15,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6097,11 +6152,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6109,11 +6164,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6121,11 +6176,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6133,11 +6188,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A16,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6150,11 +6205,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6162,11 +6217,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6174,11 +6229,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6186,11 +6241,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A17,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6203,11 +6258,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6215,11 +6270,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6227,11 +6282,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6239,11 +6294,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A18,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6256,11 +6311,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6268,11 +6323,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6280,11 +6335,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6292,11 +6347,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A19,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6309,11 +6364,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6321,11 +6376,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6333,11 +6388,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6345,11 +6400,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A20,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6362,11 +6417,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$91,Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$91,Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6374,11 +6429,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$91,Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$91,Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6386,11 +6441,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$91,Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$91,Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6398,11 +6453,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$91,$A21,Meals!$M$5:$M$91,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -8220,7 +8275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -9741,6 +9796,60 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>Low-calorie gelato (1 serving ~125 ml)</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="C61" s="7" t="n">
+        <v>95</v>
+      </c>
+      <c r="D61" s="8">
+        <f>AVERAGE(B61:C61)</f>
+        <v/>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>~1-3 g</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>86 kcal per serving - a 500 ml tub is ~4 servings, so ~344 kcal</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>Low-calorie gelato (whole 500 ml tub)</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="n">
+        <v>330</v>
+      </c>
+      <c r="C62" s="7" t="n">
+        <v>360</v>
+      </c>
+      <c r="D62" s="8">
+        <f>AVERAGE(B62:C62)</f>
+        <v/>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>~5-10 g</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>Sweetened with oligofructose; a whole tub is 20-30 g of added fibre and commonly causes bloating</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Log Day 18 breakfast and mark Day 17 incomplete
Day 17's restaurant main and closing scoop were never reported, so it
stands at 1,641 kcal - implausible for a day that included a restaurant
soup and juice. Marked incomplete and excluded from the averages, the
same treatment as Day 8.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N92"/>
+  <dimension ref="A1:N93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5451,6 +5451,61 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" s="4" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="inlineStr">
+        <is>
+          <t>2 poori + potato bhaji</t>
+        </is>
+      </c>
+      <c r="D93" s="7" t="n">
+        <v>290</v>
+      </c>
+      <c r="E93" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="F93" s="8">
+        <f>AVERAGE(D93:E93)</f>
+        <v/>
+      </c>
+      <c r="G93" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="H93" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="I93" s="10">
+        <f>AVERAGE(G93:H93)</f>
+        <v/>
+      </c>
+      <c r="J93" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="K93" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="L93" s="10">
+        <f>AVERAGE(J93:K93)</f>
+        <v/>
+      </c>
+      <c r="M93" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N93" s="6" t="inlineStr">
+        <is>
+          <t>Monday mess breakfast as served</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -5465,7 +5520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5569,11 +5624,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5581,11 +5636,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5593,11 +5648,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5605,11 +5660,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A5,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5622,11 +5677,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5634,11 +5689,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5646,11 +5701,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5658,11 +5713,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A6,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5675,11 +5730,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5687,11 +5742,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5699,11 +5754,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5711,11 +5766,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A7,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5728,11 +5783,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5740,11 +5795,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5752,11 +5807,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5764,11 +5819,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A8,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5781,11 +5836,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5793,11 +5848,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5805,11 +5860,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5817,11 +5872,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A9,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5834,11 +5889,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5846,11 +5901,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5858,11 +5913,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5870,11 +5925,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A10,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5887,11 +5942,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5899,11 +5954,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5911,11 +5966,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5923,11 +5978,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A11,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5940,11 +5995,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -5952,11 +6007,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -5964,11 +6019,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -5976,11 +6031,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A12,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -5993,11 +6048,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6005,11 +6060,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6017,11 +6072,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6029,11 +6084,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A13,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6046,11 +6101,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6058,11 +6113,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6070,11 +6125,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6082,11 +6137,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A14,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6099,11 +6154,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6111,11 +6166,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6123,11 +6178,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6135,11 +6190,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A15,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6152,11 +6207,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6164,11 +6219,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6176,11 +6231,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6188,11 +6243,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A16,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6205,11 +6260,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6217,11 +6272,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6229,11 +6284,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6241,11 +6296,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A17,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6258,11 +6313,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6270,11 +6325,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6282,11 +6337,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6294,11 +6349,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A18,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6311,11 +6366,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6323,11 +6378,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6335,11 +6390,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6347,11 +6402,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A19,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6364,11 +6419,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6376,11 +6431,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6388,11 +6443,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6400,11 +6455,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A20,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6417,11 +6472,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$92,Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$92,Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6429,11 +6484,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$92,Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$92,Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6441,11 +6496,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$92,Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$92,Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6453,15 +6508,68 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$92,$A21,Meals!$M$5:$M$92,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
         <f>D21-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B22" s="21">
+        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"logged")</f>
+        <v/>
+      </c>
+      <c r="C22" s="21">
+        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"logged")</f>
+        <v/>
+      </c>
+      <c r="D22" s="21">
+        <f>AVERAGE(B22:C22)</f>
+        <v/>
+      </c>
+      <c r="E22" s="22">
+        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"logged")</f>
+        <v/>
+      </c>
+      <c r="F22" s="22">
+        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"logged")</f>
+        <v/>
+      </c>
+      <c r="G22" s="22">
+        <f>AVERAGE(E22:F22)</f>
+        <v/>
+      </c>
+      <c r="H22" s="22">
+        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"logged")</f>
+        <v/>
+      </c>
+      <c r="I22" s="22">
+        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"logged")</f>
+        <v/>
+      </c>
+      <c r="J22" s="22">
+        <f>AVERAGE(H22:I22)</f>
+        <v/>
+      </c>
+      <c r="K22" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"logged")</f>
+        <v/>
+      </c>
+      <c r="L22" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"pending")</f>
+        <v/>
+      </c>
+      <c r="M22" s="23">
+        <f>D22-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -7456,7 +7564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7495,7 +7603,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$21)</f>
+        <f>COUNT(Daily!$A$5:$A$22)</f>
         <v/>
       </c>
     </row>
@@ -7506,7 +7614,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$21),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$22),0)</f>
         <v/>
       </c>
     </row>
@@ -7517,7 +7625,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$21),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$22),0)</f>
         <v/>
       </c>
     </row>
@@ -7528,7 +7636,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$21),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$22),0)</f>
         <v/>
       </c>
     </row>
@@ -7572,7 +7680,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$21,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$22,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -7583,7 +7691,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$21)</f>
+        <f>SUM(Daily!$L$5:$L$22)</f>
         <v/>
       </c>
     </row>
@@ -7634,19 +7742,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$21,"&gt;="&amp;$A17,Daily!$A$5:$A$21,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$22,"&gt;="&amp;$A17,Daily!$A$5:$A$22,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$21,Daily!$A$5:$A$21,"&gt;="&amp;$A17,Daily!$A$5:$A$21,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$22,Daily!$A$5:$A$22,"&gt;="&amp;$A17,Daily!$A$5:$A$22,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$21,Daily!$A$5:$A$21,"&gt;="&amp;$A17,Daily!$A$5:$A$21,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$22,Daily!$A$5:$A$22,"&gt;="&amp;$A17,Daily!$A$5:$A$22,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$21,Daily!$A$5:$A$21,"&gt;="&amp;$A17,Daily!$A$5:$A$21,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$22,Daily!$A$5:$A$22,"&gt;="&amp;$A17,Daily!$A$5:$A$22,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -7658,19 +7766,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$21,"&gt;="&amp;$A18,Daily!$A$5:$A$21,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$22,"&gt;="&amp;$A18,Daily!$A$5:$A$22,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$21,Daily!$A$5:$A$21,"&gt;="&amp;$A18,Daily!$A$5:$A$21,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$22,Daily!$A$5:$A$22,"&gt;="&amp;$A18,Daily!$A$5:$A$22,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$21,Daily!$A$5:$A$21,"&gt;="&amp;$A18,Daily!$A$5:$A$21,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$22,Daily!$A$5:$A$22,"&gt;="&amp;$A18,Daily!$A$5:$A$22,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$21,Daily!$A$5:$A$21,"&gt;="&amp;$A18,Daily!$A$5:$A$21,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$22,Daily!$A$5:$A$22,"&gt;="&amp;$A18,Daily!$A$5:$A$22,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -7682,87 +7790,111 @@
         <v>46285</v>
       </c>
       <c r="C19" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$21,"&gt;="&amp;$A19,Daily!$A$5:$A$21,"&lt;="&amp;$B19)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$22,"&gt;="&amp;$A19,Daily!$A$5:$A$22,"&lt;="&amp;$B19)</f>
         <v/>
       </c>
       <c r="D19" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$21,Daily!$A$5:$A$21,"&gt;="&amp;$A19,Daily!$A$5:$A$21,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$22,Daily!$A$5:$A$22,"&gt;="&amp;$A19,Daily!$A$5:$A$22,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$21,Daily!$A$5:$A$21,"&gt;="&amp;$A19,Daily!$A$5:$A$21,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$22,Daily!$A$5:$A$22,"&gt;="&amp;$A19,Daily!$A$5:$A$22,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$21,Daily!$A$5:$A$21,"&gt;="&amp;$A19,Daily!$A$5:$A$21,"&lt;="&amp;$B19),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="28" t="inlineStr">
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$22,Daily!$A$5:$A$22,"&gt;="&amp;$A19,Daily!$A$5:$A$22,"&lt;="&amp;$B19),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>46292</v>
+      </c>
+      <c r="C20" s="18">
+        <f>COUNTIFS(Daily!$A$5:$A$22,"&gt;="&amp;$A20,Daily!$A$5:$A$22,"&lt;="&amp;$B20)</f>
+        <v/>
+      </c>
+      <c r="D20" s="8">
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$22,Daily!$A$5:$A$22,"&gt;="&amp;$A20,Daily!$A$5:$A$22,"&lt;="&amp;$B20),0)</f>
+        <v/>
+      </c>
+      <c r="E20" s="10">
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$22,Daily!$A$5:$A$22,"&gt;="&amp;$A20,Daily!$A$5:$A$22,"&lt;="&amp;$B20),0)</f>
+        <v/>
+      </c>
+      <c r="F20" s="10">
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$22,Daily!$A$5:$A$22,"&gt;="&amp;$A20,Daily!$A$5:$A$22,"&lt;="&amp;$B20),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="28" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Month start</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Month end</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Days logged</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>Avg cal/day (mid)</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>Avg protein/day (mid, g)</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Avg fat/day (mid, g)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
+    <row r="24">
+      <c r="A24" s="4" t="n">
         <v>46266</v>
       </c>
-      <c r="B23" s="4" t="n">
+      <c r="B24" s="4" t="n">
         <v>46295</v>
       </c>
-      <c r="C23" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$21,"&gt;="&amp;$A23,Daily!$A$5:$A$21,"&lt;="&amp;$B23)</f>
-        <v/>
-      </c>
-      <c r="D23" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$21,Daily!$A$5:$A$21,"&gt;="&amp;$A23,Daily!$A$5:$A$21,"&lt;="&amp;$B23),0)</f>
-        <v/>
-      </c>
-      <c r="E23" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$21,Daily!$A$5:$A$21,"&gt;="&amp;$A23,Daily!$A$5:$A$21,"&lt;="&amp;$B23),0)</f>
-        <v/>
-      </c>
-      <c r="F23" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$21,Daily!$A$5:$A$21,"&gt;="&amp;$A23,Daily!$A$5:$A$21,"&lt;="&amp;$B23),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="27" t="inlineStr">
+      <c r="C24" s="18">
+        <f>COUNTIFS(Daily!$A$5:$A$22,"&gt;="&amp;$A24,Daily!$A$5:$A$22,"&lt;="&amp;$B24)</f>
+        <v/>
+      </c>
+      <c r="D24" s="8">
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$22,Daily!$A$5:$A$22,"&gt;="&amp;$A24,Daily!$A$5:$A$22,"&lt;="&amp;$B24),0)</f>
+        <v/>
+      </c>
+      <c r="E24" s="10">
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$22,Daily!$A$5:$A$22,"&gt;="&amp;$A24,Daily!$A$5:$A$22,"&lt;="&amp;$B24),0)</f>
+        <v/>
+      </c>
+      <c r="F24" s="10">
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$22,Daily!$A$5:$A$22,"&gt;="&amp;$A24,Daily!$A$5:$A$22,"&lt;="&amp;$B24),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="27" t="inlineStr">
         <is>
           <t>Averages cover only the days present in the log; a part-logged day (today's dinner still to come) drags its average down.</t>
         </is>

</xml_diff>

<commit_message>
Close Day 17 with the restaurant dinner: 2,491 kcal, 158.25 g protein
Quarter grilled chicken and a mixed grill, ~850 kcal for ~90 g of
protein. The day lands at only -178, but the dinner is not why: the
~585 kcal of vada, squid, gelato and mint juice before it delivered
25 g of protein between them.

Sixteen complete days: 2,198 kcal, 117.1 g protein, 470 deficit,
0.43 kg/week. The protein average has climbed from 105.6 in a week.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N93"/>
+  <dimension ref="A1:N94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5127,39 +5127,39 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>Drink</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>Mint juice (small cup)</t>
+          <t>Quarter grilled chicken + mixed grill</t>
         </is>
       </c>
       <c r="D87" s="7" t="n">
-        <v>60</v>
+        <v>650</v>
       </c>
       <c r="E87" s="7" t="n">
-        <v>140</v>
+        <v>1050</v>
       </c>
       <c r="F87" s="8">
         <f>AVERAGE(D87:E87)</f>
         <v/>
       </c>
       <c r="G87" s="9" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H87" s="9" t="n">
-        <v>0.5</v>
+        <v>105</v>
       </c>
       <c r="I87" s="10">
         <f>AVERAGE(G87:H87)</f>
         <v/>
       </c>
       <c r="J87" s="9" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="K87" s="9" t="n">
-        <v>0.5</v>
+        <v>63</v>
       </c>
       <c r="L87" s="10">
         <f>AVERAGE(J87:K87)</f>
@@ -5172,7 +5172,7 @@
       </c>
       <c r="N87" s="6" t="inlineStr">
         <is>
-          <t>Assumed sweetened - if unsweetened it is nearer 15 kcal</t>
+          <t>Restaurant dinner at Panoor; closing scoop not taken</t>
         </is>
       </c>
     </row>
@@ -5182,39 +5182,39 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Drink</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>Ghee rice (halved) + chicken curry + curd</t>
+          <t>Mint juice (small cup)</t>
         </is>
       </c>
       <c r="D88" s="7" t="n">
-        <v>490</v>
+        <v>60</v>
       </c>
       <c r="E88" s="7" t="n">
-        <v>710</v>
+        <v>140</v>
       </c>
       <c r="F88" s="8">
         <f>AVERAGE(D88:E88)</f>
         <v/>
       </c>
       <c r="G88" s="9" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="H88" s="9" t="n">
-        <v>36</v>
+        <v>0.5</v>
       </c>
       <c r="I88" s="10">
         <f>AVERAGE(G88:H88)</f>
         <v/>
       </c>
       <c r="J88" s="9" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="K88" s="9" t="n">
-        <v>36</v>
+        <v>0.5</v>
       </c>
       <c r="L88" s="10">
         <f>AVERAGE(J88:K88)</f>
@@ -5227,7 +5227,7 @@
       </c>
       <c r="N88" s="6" t="inlineStr">
         <is>
-          <t>Rice halved despite the day having room for it</t>
+          <t>Assumed sweetened - if unsweetened it is nearer 15 kcal</t>
         </is>
       </c>
     </row>
@@ -5237,39 +5237,39 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>1 parippu vada + milk coffee (no sugar)</t>
+          <t>Ghee rice (halved) + chicken curry + curd</t>
         </is>
       </c>
       <c r="D89" s="7" t="n">
-        <v>170</v>
+        <v>490</v>
       </c>
       <c r="E89" s="7" t="n">
-        <v>280</v>
+        <v>710</v>
       </c>
       <c r="F89" s="8">
         <f>AVERAGE(D89:E89)</f>
         <v/>
       </c>
       <c r="G89" s="9" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="H89" s="9" t="n">
-        <v>10.5</v>
+        <v>36</v>
       </c>
       <c r="I89" s="10">
         <f>AVERAGE(G89:H89)</f>
         <v/>
       </c>
       <c r="J89" s="9" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="K89" s="9" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="L89" s="10">
         <f>AVERAGE(J89:K89)</f>
@@ -5282,7 +5282,7 @@
       </c>
       <c r="N89" s="6" t="inlineStr">
         <is>
-          <t>First milk coffee logged - black coffee is ~2 kcal against this ~60</t>
+          <t>Rice halved despite the day having room for it</t>
         </is>
       </c>
     </row>
@@ -5297,34 +5297,34 @@
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>1 small stuffed squid (pan-fried)</t>
+          <t>1 parippu vada + milk coffee (no sugar)</t>
         </is>
       </c>
       <c r="D90" s="7" t="n">
-        <v>130</v>
+        <v>170</v>
       </c>
       <c r="E90" s="7" t="n">
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="F90" s="8">
         <f>AVERAGE(D90:E90)</f>
         <v/>
       </c>
       <c r="G90" s="9" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H90" s="9" t="n">
-        <v>14</v>
+        <v>10.5</v>
       </c>
       <c r="I90" s="10">
         <f>AVERAGE(G90:H90)</f>
         <v/>
       </c>
       <c r="J90" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K90" s="9" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L90" s="10">
         <f>AVERAGE(J90:K90)</f>
@@ -5337,7 +5337,7 @@
       </c>
       <c r="N90" s="6" t="inlineStr">
         <is>
-          <t>7.3 g protein per 100 kcal - double the mess average</t>
+          <t>First milk coffee logged - black coffee is ~2 kcal against this ~60</t>
         </is>
       </c>
     </row>
@@ -5352,34 +5352,34 @@
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>Clear soup (one spoonful only)</t>
+          <t>1 small stuffed squid (pan-fried)</t>
         </is>
       </c>
       <c r="D91" s="7" t="n">
-        <v>5</v>
+        <v>130</v>
       </c>
       <c r="E91" s="7" t="n">
-        <v>12</v>
+        <v>200</v>
       </c>
       <c r="F91" s="8">
         <f>AVERAGE(D91:E91)</f>
         <v/>
       </c>
       <c r="G91" s="9" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H91" s="9" t="n">
-        <v>0.5</v>
+        <v>14</v>
       </c>
       <c r="I91" s="10">
         <f>AVERAGE(G91:H91)</f>
         <v/>
       </c>
       <c r="J91" s="9" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K91" s="9" t="n">
-        <v>0.5</v>
+        <v>15</v>
       </c>
       <c r="L91" s="10">
         <f>AVERAGE(J91:K91)</f>
@@ -5392,7 +5392,7 @@
       </c>
       <c r="N91" s="6" t="inlineStr">
         <is>
-          <t>Corrected - only a spoonful was taken</t>
+          <t>7.3 g protein per 100 kcal - double the mess average</t>
         </is>
       </c>
     </row>
@@ -5407,34 +5407,34 @@
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>Brooklyn Creamery guilt-free gelato - coconut creme (1 serving)</t>
+          <t>Clear soup (one spoonful only)</t>
         </is>
       </c>
       <c r="D92" s="7" t="n">
-        <v>80</v>
+        <v>5</v>
       </c>
       <c r="E92" s="7" t="n">
-        <v>95</v>
+        <v>12</v>
       </c>
       <c r="F92" s="8">
         <f>AVERAGE(D92:E92)</f>
         <v/>
       </c>
       <c r="G92" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H92" s="9" t="n">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="I92" s="10">
         <f>AVERAGE(G92:H92)</f>
         <v/>
       </c>
       <c r="J92" s="9" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="K92" s="9" t="n">
-        <v>4.5</v>
+        <v>0.5</v>
       </c>
       <c r="L92" s="10">
         <f>AVERAGE(J92:K92)</f>
@@ -5447,49 +5447,49 @@
       </c>
       <c r="N92" s="6" t="inlineStr">
         <is>
-          <t>86 kcal is per serving; a 500 ml tub is about 4 servings</t>
+          <t>Corrected - only a spoonful was taken</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>Breakfast</t>
+          <t>Snack</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>2 poori + potato bhaji</t>
+          <t>Brooklyn Creamery guilt-free gelato - coconut creme (1 serving)</t>
         </is>
       </c>
       <c r="D93" s="7" t="n">
-        <v>290</v>
+        <v>80</v>
       </c>
       <c r="E93" s="7" t="n">
-        <v>420</v>
+        <v>95</v>
       </c>
       <c r="F93" s="8">
         <f>AVERAGE(D93:E93)</f>
         <v/>
       </c>
       <c r="G93" s="9" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H93" s="9" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I93" s="10">
         <f>AVERAGE(G93:H93)</f>
         <v/>
       </c>
       <c r="J93" s="9" t="n">
-        <v>14</v>
+        <v>2.5</v>
       </c>
       <c r="K93" s="9" t="n">
-        <v>24</v>
+        <v>4.5</v>
       </c>
       <c r="L93" s="10">
         <f>AVERAGE(J93:K93)</f>
@@ -5501,6 +5501,61 @@
         </is>
       </c>
       <c r="N93" s="6" t="inlineStr">
+        <is>
+          <t>86 kcal is per serving; a 500 ml tub is about 4 servings</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="inlineStr">
+        <is>
+          <t>2 poori + potato bhaji</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="n">
+        <v>290</v>
+      </c>
+      <c r="E94" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="F94" s="8">
+        <f>AVERAGE(D94:E94)</f>
+        <v/>
+      </c>
+      <c r="G94" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="H94" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="I94" s="10">
+        <f>AVERAGE(G94:H94)</f>
+        <v/>
+      </c>
+      <c r="J94" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="K94" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="L94" s="10">
+        <f>AVERAGE(J94:K94)</f>
+        <v/>
+      </c>
+      <c r="M94" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N94" s="6" t="inlineStr">
         <is>
           <t>Monday mess breakfast as served</t>
         </is>
@@ -5624,11 +5679,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5636,11 +5691,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5648,11 +5703,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5660,11 +5715,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A5,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5677,11 +5732,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5689,11 +5744,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5701,11 +5756,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5713,11 +5768,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A6,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5730,11 +5785,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5742,11 +5797,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5754,11 +5809,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5766,11 +5821,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A7,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5783,11 +5838,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5795,11 +5850,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5807,11 +5862,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5819,11 +5874,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A8,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5836,11 +5891,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5848,11 +5903,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5860,11 +5915,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5872,11 +5927,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A9,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5889,11 +5944,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5901,11 +5956,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5913,11 +5968,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5925,11 +5980,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A10,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5942,11 +5997,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -5954,11 +6009,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -5966,11 +6021,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -5978,11 +6033,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A11,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -5995,11 +6050,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6007,11 +6062,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6019,11 +6074,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6031,11 +6086,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A12,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6048,11 +6103,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6060,11 +6115,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6072,11 +6127,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6084,11 +6139,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A13,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6101,11 +6156,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6113,11 +6168,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6125,11 +6180,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6137,11 +6192,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A14,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6154,11 +6209,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6166,11 +6221,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6178,11 +6233,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6190,11 +6245,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A15,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6207,11 +6262,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6219,11 +6274,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6231,11 +6286,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6243,11 +6298,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A16,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6260,11 +6315,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6272,11 +6327,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6284,11 +6339,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6296,11 +6351,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A17,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6313,11 +6368,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6325,11 +6380,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6337,11 +6392,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6349,11 +6404,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A18,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6366,11 +6421,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6378,11 +6433,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6390,11 +6445,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6402,11 +6457,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A19,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6419,11 +6474,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6431,11 +6486,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6443,11 +6498,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6455,11 +6510,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A20,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6472,11 +6527,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6484,11 +6539,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6496,11 +6551,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6508,11 +6563,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A21,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -6525,11 +6580,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$93,Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$93,Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -6537,11 +6592,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$93,Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$93,Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -6549,11 +6604,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$93,Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$93,Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -6561,11 +6616,11 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$93,$A22,Meals!$M$5:$M$93,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">

</xml_diff>

<commit_message>
Log Day 18 lunch: fullest meals plate since Day 13
Rice not stated as halved and costed as a near-full portion; the plate
also carried two pappadam and every side container. The omelette roll is
the only real protein on it.

Lands on one chapati at dinner plus three scoops: 2,120 exactly, 134.5 g.
Identical calories to two chapati and two scoops, but 19 g more protein.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N94"/>
+  <dimension ref="A1:N95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5558,6 +5558,61 @@
       <c r="N94" s="6" t="inlineStr">
         <is>
           <t>Monday mess breakfast as served</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>Mess meals plate + 1-egg omelette roll, 2 pappadam, sambar, kadala, chammanthi, veg curry</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="n">
+        <v>750</v>
+      </c>
+      <c r="E95" s="7" t="n">
+        <v>1160</v>
+      </c>
+      <c r="F95" s="8">
+        <f>AVERAGE(D95:E95)</f>
+        <v/>
+      </c>
+      <c r="G95" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="H95" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I95" s="10">
+        <f>AVERAGE(G95:H95)</f>
+        <v/>
+      </c>
+      <c r="J95" s="9" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="K95" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="L95" s="10">
+        <f>AVERAGE(J95:K95)</f>
+        <v/>
+      </c>
+      <c r="M95" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N95" s="6" t="inlineStr">
+        <is>
+          <t>Rice not stated as halved - costed as a near-full portion</t>
         </is>
       </c>
     </row>
@@ -5679,11 +5734,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5691,11 +5746,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5703,11 +5758,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5715,11 +5770,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A5,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5732,11 +5787,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5744,11 +5799,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5756,11 +5811,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5768,11 +5823,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A6,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5785,11 +5840,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5797,11 +5852,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5809,11 +5864,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5821,11 +5876,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A7,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5838,11 +5893,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5850,11 +5905,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5862,11 +5917,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5874,11 +5929,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A8,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5891,11 +5946,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5903,11 +5958,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5915,11 +5970,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5927,11 +5982,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A9,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5944,11 +5999,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -5956,11 +6011,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -5968,11 +6023,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -5980,11 +6035,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A10,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -5997,11 +6052,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6009,11 +6064,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6021,11 +6076,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6033,11 +6088,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A11,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6050,11 +6105,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6062,11 +6117,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6074,11 +6129,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6086,11 +6141,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A12,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6103,11 +6158,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6115,11 +6170,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6127,11 +6182,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6139,11 +6194,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A13,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6156,11 +6211,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6168,11 +6223,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6180,11 +6235,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6192,11 +6247,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A14,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6209,11 +6264,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6221,11 +6276,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6233,11 +6288,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6245,11 +6300,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A15,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6262,11 +6317,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6274,11 +6329,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6286,11 +6341,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6298,11 +6353,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A16,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6315,11 +6370,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6327,11 +6382,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6339,11 +6394,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6351,11 +6406,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A17,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6368,11 +6423,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6380,11 +6435,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6392,11 +6447,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6404,11 +6459,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A18,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6421,11 +6476,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6433,11 +6488,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6445,11 +6500,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6457,11 +6512,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A19,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6474,11 +6529,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6486,11 +6541,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6498,11 +6553,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6510,11 +6565,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A20,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6527,11 +6582,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6539,11 +6594,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6551,11 +6606,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6563,11 +6618,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A21,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -6580,11 +6635,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$94,Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$94,Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -6592,11 +6647,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$94,Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$94,Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -6604,11 +6659,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$94,Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$94,Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -6616,11 +6671,11 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$94,$A22,Meals!$M$5:$M$94,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">

</xml_diff>

<commit_message>
Log the Day 18 rasam
~37 kcal - the best-value item in the container set, against the coconut
chammanthi's ~125 for barely more protein. Evening plan unchanged at one
chapati and three scoops.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N95"/>
+  <dimension ref="A1:N96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5613,6 +5613,61 @@
       <c r="N95" s="6" t="inlineStr">
         <is>
           <t>Rice not stated as halved - costed as a near-full portion</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="inlineStr">
+        <is>
+          <t>Rasam (small container)</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="E96" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="F96" s="8">
+        <f>AVERAGE(D96:E96)</f>
+        <v/>
+      </c>
+      <c r="G96" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H96" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I96" s="10">
+        <f>AVERAGE(G96:H96)</f>
+        <v/>
+      </c>
+      <c r="J96" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K96" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L96" s="10">
+        <f>AVERAGE(J96:K96)</f>
+        <v/>
+      </c>
+      <c r="M96" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N96" s="6" t="inlineStr">
+        <is>
+          <t>Thin tamarind broth - the cheapest item in the container set</t>
         </is>
       </c>
     </row>
@@ -5734,11 +5789,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5746,11 +5801,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5758,11 +5813,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5770,11 +5825,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A5,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5787,11 +5842,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5799,11 +5854,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5811,11 +5866,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5823,11 +5878,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A6,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5840,11 +5895,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5852,11 +5907,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5864,11 +5919,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5876,11 +5931,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A7,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5893,11 +5948,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5905,11 +5960,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5917,11 +5972,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5929,11 +5984,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A8,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -5946,11 +6001,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -5958,11 +6013,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -5970,11 +6025,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -5982,11 +6037,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A9,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -5999,11 +6054,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -6011,11 +6066,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -6023,11 +6078,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -6035,11 +6090,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A10,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -6052,11 +6107,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6064,11 +6119,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6076,11 +6131,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6088,11 +6143,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A11,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6105,11 +6160,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6117,11 +6172,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6129,11 +6184,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6141,11 +6196,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A12,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6158,11 +6213,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6170,11 +6225,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6182,11 +6237,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6194,11 +6249,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A13,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6211,11 +6266,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6223,11 +6278,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6235,11 +6290,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6247,11 +6302,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A14,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6264,11 +6319,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6276,11 +6331,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6288,11 +6343,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6300,11 +6355,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A15,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6317,11 +6372,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6329,11 +6384,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6341,11 +6396,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6353,11 +6408,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A16,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6370,11 +6425,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6382,11 +6437,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6394,11 +6449,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6406,11 +6461,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A17,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6423,11 +6478,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6435,11 +6490,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6447,11 +6502,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6459,11 +6514,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A18,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6476,11 +6531,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6488,11 +6543,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6500,11 +6555,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6512,11 +6567,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A19,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6529,11 +6584,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6541,11 +6596,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6553,11 +6608,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6565,11 +6620,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A20,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6582,11 +6637,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6594,11 +6649,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6606,11 +6661,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6618,11 +6673,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A21,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -6635,11 +6690,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$95,Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$95,Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -6647,11 +6702,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$95,Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$95,Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -6659,11 +6714,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$95,Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$95,Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -6671,11 +6726,11 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$95,$A22,Meals!$M$5:$M$95,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">

</xml_diff>

<commit_message>
Log Day 18 dinner: half grilled chicken with the fries and kubboos left
Skipping those two is worth ~400-600 kcal, more than every deliberate
cut made at lunch.

The creamy garlic sauce is now the expensive item: ~190 kcal for ~1 g of
protein, 0.5 g per 100 kcal, the worst rate in eighteen days. Leaving it
and taking one chapati puts the day at 2,245 and 138.25 g.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N96"/>
+  <dimension ref="A1:N97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5567,39 +5567,39 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate + 1-egg omelette roll, 2 pappadam, sambar, kadala, chammanthi, veg curry</t>
+          <t>Half grilled chicken + 2 chapati + chicken curry + salad + creamy garlic sauce</t>
         </is>
       </c>
       <c r="D95" s="7" t="n">
-        <v>750</v>
+        <v>865</v>
       </c>
       <c r="E95" s="7" t="n">
-        <v>1160</v>
+        <v>1310</v>
       </c>
       <c r="F95" s="8">
         <f>AVERAGE(D95:E95)</f>
         <v/>
       </c>
       <c r="G95" s="9" t="n">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="H95" s="9" t="n">
-        <v>37</v>
+        <v>92</v>
       </c>
       <c r="I95" s="10">
         <f>AVERAGE(G95:H95)</f>
         <v/>
       </c>
       <c r="J95" s="9" t="n">
-        <v>31.5</v>
+        <v>46</v>
       </c>
       <c r="K95" s="9" t="n">
-        <v>55</v>
+        <v>78.5</v>
       </c>
       <c r="L95" s="10">
         <f>AVERAGE(J95:K95)</f>
@@ -5612,7 +5612,7 @@
       </c>
       <c r="N95" s="6" t="inlineStr">
         <is>
-          <t>Rice not stated as halved - costed as a near-full portion</t>
+          <t>Fries and kubboos skipped - saves ~400-600 kcal</t>
         </is>
       </c>
     </row>
@@ -5627,34 +5627,34 @@
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>Rasam (small container)</t>
+          <t>Mess meals plate + 1-egg omelette roll, 2 pappadam, sambar, kadala, chammanthi, veg curry</t>
         </is>
       </c>
       <c r="D96" s="7" t="n">
-        <v>25</v>
+        <v>750</v>
       </c>
       <c r="E96" s="7" t="n">
-        <v>50</v>
+        <v>1160</v>
       </c>
       <c r="F96" s="8">
         <f>AVERAGE(D96:E96)</f>
         <v/>
       </c>
       <c r="G96" s="9" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="H96" s="9" t="n">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="I96" s="10">
         <f>AVERAGE(G96:H96)</f>
         <v/>
       </c>
       <c r="J96" s="9" t="n">
-        <v>1</v>
+        <v>31.5</v>
       </c>
       <c r="K96" s="9" t="n">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="L96" s="10">
         <f>AVERAGE(J96:K96)</f>
@@ -5666,6 +5666,61 @@
         </is>
       </c>
       <c r="N96" s="6" t="inlineStr">
+        <is>
+          <t>Rice not stated as halved - costed as a near-full portion</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="inlineStr">
+        <is>
+          <t>Rasam (small container)</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="E97" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="F97" s="8">
+        <f>AVERAGE(D97:E97)</f>
+        <v/>
+      </c>
+      <c r="G97" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H97" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I97" s="10">
+        <f>AVERAGE(G97:H97)</f>
+        <v/>
+      </c>
+      <c r="J97" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K97" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L97" s="10">
+        <f>AVERAGE(J97:K97)</f>
+        <v/>
+      </c>
+      <c r="M97" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N97" s="6" t="inlineStr">
         <is>
           <t>Thin tamarind broth - the cheapest item in the container set</t>
         </is>
@@ -5789,11 +5844,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5801,11 +5856,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5813,11 +5868,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5825,11 +5880,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A5,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5842,11 +5897,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5854,11 +5909,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5866,11 +5921,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5878,11 +5933,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A6,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5895,11 +5950,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5907,11 +5962,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5919,11 +5974,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5931,11 +5986,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A7,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -5948,11 +6003,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -5960,11 +6015,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -5972,11 +6027,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -5984,11 +6039,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A8,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -6001,11 +6056,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -6013,11 +6068,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -6025,11 +6080,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -6037,11 +6092,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A9,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -6054,11 +6109,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -6066,11 +6121,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -6078,11 +6133,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -6090,11 +6145,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A10,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -6107,11 +6162,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6119,11 +6174,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6131,11 +6186,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6143,11 +6198,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A11,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6160,11 +6215,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6172,11 +6227,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6184,11 +6239,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6196,11 +6251,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A12,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6213,11 +6268,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6225,11 +6280,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6237,11 +6292,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6249,11 +6304,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A13,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6266,11 +6321,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6278,11 +6333,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6290,11 +6345,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6302,11 +6357,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A14,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6319,11 +6374,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6331,11 +6386,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6343,11 +6398,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6355,11 +6410,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A15,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6372,11 +6427,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6384,11 +6439,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6396,11 +6451,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6408,11 +6463,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A16,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6425,11 +6480,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6437,11 +6492,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6449,11 +6504,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6461,11 +6516,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A17,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6478,11 +6533,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6490,11 +6545,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6502,11 +6557,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6514,11 +6569,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A18,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6531,11 +6586,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6543,11 +6598,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6555,11 +6610,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6567,11 +6622,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A19,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6584,11 +6639,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6596,11 +6651,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6608,11 +6663,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6620,11 +6675,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A20,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6637,11 +6692,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6649,11 +6704,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6661,11 +6716,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6673,11 +6728,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A21,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -6690,11 +6745,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$96,Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$96,Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -6702,11 +6757,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$96,Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$96,Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -6714,11 +6769,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$96,Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$96,Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -6726,11 +6781,11 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$96,$A22,Meals!$M$5:$M$96,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">

</xml_diff>

<commit_message>
Close Day 18 and log Day 19 breakfast
Day 18 closed at 2,435 kcal and 120.5 g of protein - no closing scoop
reported and the creamy sauce taken as plated, so a 234 deficit.

Seventeen complete days: 2,212 kcal, 117.3 g protein, 457 deficit,
0.42 kg/week.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N97"/>
+  <dimension ref="A1:N98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5726,6 +5726,61 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" s="4" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>Large masala dosa + sambar</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="n">
+        <v>410</v>
+      </c>
+      <c r="E98" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="F98" s="8">
+        <f>AVERAGE(D98:E98)</f>
+        <v/>
+      </c>
+      <c r="G98" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H98" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="I98" s="10">
+        <f>AVERAGE(G98:H98)</f>
+        <v/>
+      </c>
+      <c r="J98" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="K98" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="L98" s="10">
+        <f>AVERAGE(J98:K98)</f>
+        <v/>
+      </c>
+      <c r="M98" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N98" s="6" t="inlineStr">
+        <is>
+          <t>Tuesday mess breakfast</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -5740,7 +5795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5844,11 +5899,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5856,11 +5911,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5868,11 +5923,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5880,11 +5935,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A5,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5897,11 +5952,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5909,11 +5964,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5921,11 +5976,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5933,11 +5988,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A6,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -5950,11 +6005,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -5962,11 +6017,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -5974,11 +6029,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -5986,11 +6041,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A7,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -6003,11 +6058,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -6015,11 +6070,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -6027,11 +6082,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -6039,11 +6094,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A8,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -6056,11 +6111,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -6068,11 +6123,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -6080,11 +6135,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -6092,11 +6147,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A9,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -6109,11 +6164,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -6121,11 +6176,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -6133,11 +6188,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -6145,11 +6200,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A10,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -6162,11 +6217,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6174,11 +6229,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6186,11 +6241,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6198,11 +6253,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A11,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6215,11 +6270,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6227,11 +6282,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6239,11 +6294,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6251,11 +6306,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A12,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6268,11 +6323,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6280,11 +6335,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6292,11 +6347,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6304,11 +6359,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A13,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6321,11 +6376,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6333,11 +6388,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6345,11 +6400,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6357,11 +6412,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A14,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6374,11 +6429,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6386,11 +6441,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6398,11 +6453,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6410,11 +6465,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A15,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6427,11 +6482,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6439,11 +6494,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6451,11 +6506,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6463,11 +6518,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A16,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6480,11 +6535,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6492,11 +6547,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6504,11 +6559,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6516,11 +6571,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A17,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6533,11 +6588,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6545,11 +6600,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6557,11 +6612,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6569,11 +6624,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A18,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6586,11 +6641,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6598,11 +6653,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6610,11 +6665,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6622,11 +6677,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A19,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6639,11 +6694,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6651,11 +6706,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6663,11 +6718,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6675,11 +6730,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A20,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6692,11 +6747,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6704,11 +6759,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6716,11 +6771,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6728,11 +6783,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A21,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -6745,11 +6800,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$97,Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$97,Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -6757,11 +6812,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$97,Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$97,Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -6769,11 +6824,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$97,Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$97,Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -6781,15 +6836,68 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$97,$A22,Meals!$M$5:$M$97,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">
         <f>D22-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B23" s="8">
+        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"logged")</f>
+        <v/>
+      </c>
+      <c r="C23" s="8">
+        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"logged")</f>
+        <v/>
+      </c>
+      <c r="D23" s="8">
+        <f>AVERAGE(B23:C23)</f>
+        <v/>
+      </c>
+      <c r="E23" s="10">
+        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"logged")</f>
+        <v/>
+      </c>
+      <c r="F23" s="10">
+        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"logged")</f>
+        <v/>
+      </c>
+      <c r="G23" s="10">
+        <f>AVERAGE(E23:F23)</f>
+        <v/>
+      </c>
+      <c r="H23" s="10">
+        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"logged")</f>
+        <v/>
+      </c>
+      <c r="I23" s="10">
+        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"logged")</f>
+        <v/>
+      </c>
+      <c r="J23" s="10">
+        <f>AVERAGE(H23:I23)</f>
+        <v/>
+      </c>
+      <c r="K23" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"logged")</f>
+        <v/>
+      </c>
+      <c r="L23" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"pending")</f>
+        <v/>
+      </c>
+      <c r="M23" s="19">
+        <f>D23-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -7823,7 +7931,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$22)</f>
+        <f>COUNT(Daily!$A$5:$A$23)</f>
         <v/>
       </c>
     </row>
@@ -7834,7 +7942,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$22),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$23),0)</f>
         <v/>
       </c>
     </row>
@@ -7845,7 +7953,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$22),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$23),0)</f>
         <v/>
       </c>
     </row>
@@ -7856,7 +7964,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$22),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$23),0)</f>
         <v/>
       </c>
     </row>
@@ -7900,7 +8008,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$22,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$23,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -7911,7 +8019,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$22)</f>
+        <f>SUM(Daily!$L$5:$L$23)</f>
         <v/>
       </c>
     </row>
@@ -7962,19 +8070,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$22,"&gt;="&amp;$A17,Daily!$A$5:$A$22,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$23,"&gt;="&amp;$A17,Daily!$A$5:$A$23,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$22,Daily!$A$5:$A$22,"&gt;="&amp;$A17,Daily!$A$5:$A$22,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$23,Daily!$A$5:$A$23,"&gt;="&amp;$A17,Daily!$A$5:$A$23,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$22,Daily!$A$5:$A$22,"&gt;="&amp;$A17,Daily!$A$5:$A$22,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$23,Daily!$A$5:$A$23,"&gt;="&amp;$A17,Daily!$A$5:$A$23,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$22,Daily!$A$5:$A$22,"&gt;="&amp;$A17,Daily!$A$5:$A$22,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$23,Daily!$A$5:$A$23,"&gt;="&amp;$A17,Daily!$A$5:$A$23,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -7986,19 +8094,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$22,"&gt;="&amp;$A18,Daily!$A$5:$A$22,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$23,"&gt;="&amp;$A18,Daily!$A$5:$A$23,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$22,Daily!$A$5:$A$22,"&gt;="&amp;$A18,Daily!$A$5:$A$22,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$23,Daily!$A$5:$A$23,"&gt;="&amp;$A18,Daily!$A$5:$A$23,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$22,Daily!$A$5:$A$22,"&gt;="&amp;$A18,Daily!$A$5:$A$22,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$23,Daily!$A$5:$A$23,"&gt;="&amp;$A18,Daily!$A$5:$A$23,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$22,Daily!$A$5:$A$22,"&gt;="&amp;$A18,Daily!$A$5:$A$22,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$23,Daily!$A$5:$A$23,"&gt;="&amp;$A18,Daily!$A$5:$A$23,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -8010,19 +8118,19 @@
         <v>46285</v>
       </c>
       <c r="C19" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$22,"&gt;="&amp;$A19,Daily!$A$5:$A$22,"&lt;="&amp;$B19)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$23,"&gt;="&amp;$A19,Daily!$A$5:$A$23,"&lt;="&amp;$B19)</f>
         <v/>
       </c>
       <c r="D19" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$22,Daily!$A$5:$A$22,"&gt;="&amp;$A19,Daily!$A$5:$A$22,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$23,Daily!$A$5:$A$23,"&gt;="&amp;$A19,Daily!$A$5:$A$23,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$22,Daily!$A$5:$A$22,"&gt;="&amp;$A19,Daily!$A$5:$A$22,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$23,Daily!$A$5:$A$23,"&gt;="&amp;$A19,Daily!$A$5:$A$23,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$22,Daily!$A$5:$A$22,"&gt;="&amp;$A19,Daily!$A$5:$A$22,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$23,Daily!$A$5:$A$23,"&gt;="&amp;$A19,Daily!$A$5:$A$23,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
     </row>
@@ -8034,19 +8142,19 @@
         <v>46292</v>
       </c>
       <c r="C20" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$22,"&gt;="&amp;$A20,Daily!$A$5:$A$22,"&lt;="&amp;$B20)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$23,"&gt;="&amp;$A20,Daily!$A$5:$A$23,"&lt;="&amp;$B20)</f>
         <v/>
       </c>
       <c r="D20" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$22,Daily!$A$5:$A$22,"&gt;="&amp;$A20,Daily!$A$5:$A$22,"&lt;="&amp;$B20),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$23,Daily!$A$5:$A$23,"&gt;="&amp;$A20,Daily!$A$5:$A$23,"&lt;="&amp;$B20),0)</f>
         <v/>
       </c>
       <c r="E20" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$22,Daily!$A$5:$A$22,"&gt;="&amp;$A20,Daily!$A$5:$A$22,"&lt;="&amp;$B20),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$23,Daily!$A$5:$A$23,"&gt;="&amp;$A20,Daily!$A$5:$A$23,"&lt;="&amp;$B20),0)</f>
         <v/>
       </c>
       <c r="F20" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$22,Daily!$A$5:$A$22,"&gt;="&amp;$A20,Daily!$A$5:$A$22,"&lt;="&amp;$B20),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$23,Daily!$A$5:$A$23,"&gt;="&amp;$A20,Daily!$A$5:$A$23,"&lt;="&amp;$B20),0)</f>
         <v/>
       </c>
     </row>
@@ -8097,19 +8205,19 @@
         <v>46295</v>
       </c>
       <c r="C24" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$22,"&gt;="&amp;$A24,Daily!$A$5:$A$22,"&lt;="&amp;$B24)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$23,"&gt;="&amp;$A24,Daily!$A$5:$A$23,"&lt;="&amp;$B24)</f>
         <v/>
       </c>
       <c r="D24" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$22,Daily!$A$5:$A$22,"&gt;="&amp;$A24,Daily!$A$5:$A$22,"&lt;="&amp;$B24),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$23,Daily!$A$5:$A$23,"&gt;="&amp;$A24,Daily!$A$5:$A$23,"&lt;="&amp;$B24),0)</f>
         <v/>
       </c>
       <c r="E24" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$22,Daily!$A$5:$A$22,"&gt;="&amp;$A24,Daily!$A$5:$A$22,"&lt;="&amp;$B24),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$23,Daily!$A$5:$A$23,"&gt;="&amp;$A24,Daily!$A$5:$A$23,"&lt;="&amp;$B24),0)</f>
         <v/>
       </c>
       <c r="F24" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$22,Daily!$A$5:$A$22,"&gt;="&amp;$A24,Daily!$A$5:$A$22,"&lt;="&amp;$B24),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$23,Daily!$A$5:$A$23,"&gt;="&amp;$A24,Daily!$A$5:$A$23,"&lt;="&amp;$B24),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Day 19 lunch: halved ghee rice with chicken curry
1,015 kcal and 86.5 g of protein left. Four scoops and one egg lands 31
under target at a 580 deficit - the right direction after five of seven
days above target.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N98"/>
+  <dimension ref="A1:N99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5778,6 +5778,61 @@
       <c r="N98" s="6" t="inlineStr">
         <is>
           <t>Tuesday mess breakfast</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>Ghee rice (halved) + chicken curry + raita</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="n">
+        <v>490</v>
+      </c>
+      <c r="E99" s="7" t="n">
+        <v>710</v>
+      </c>
+      <c r="F99" s="8">
+        <f>AVERAGE(D99:E99)</f>
+        <v/>
+      </c>
+      <c r="G99" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="H99" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I99" s="10">
+        <f>AVERAGE(G99:H99)</f>
+        <v/>
+      </c>
+      <c r="J99" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="K99" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="L99" s="10">
+        <f>AVERAGE(J99:K99)</f>
+        <v/>
+      </c>
+      <c r="M99" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N99" s="6" t="inlineStr">
+        <is>
+          <t>Rice halved; generous chicken portion</t>
         </is>
       </c>
     </row>
@@ -5899,11 +5954,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5911,11 +5966,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5923,11 +5978,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5935,11 +5990,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A5,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -5952,11 +6007,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -5964,11 +6019,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -5976,11 +6031,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -5988,11 +6043,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A6,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -6005,11 +6060,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -6017,11 +6072,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -6029,11 +6084,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -6041,11 +6096,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A7,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -6058,11 +6113,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -6070,11 +6125,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -6082,11 +6137,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -6094,11 +6149,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A8,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -6111,11 +6166,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -6123,11 +6178,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -6135,11 +6190,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -6147,11 +6202,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A9,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -6164,11 +6219,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -6176,11 +6231,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -6188,11 +6243,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -6200,11 +6255,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A10,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -6217,11 +6272,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6229,11 +6284,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6241,11 +6296,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6253,11 +6308,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A11,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6270,11 +6325,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6282,11 +6337,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6294,11 +6349,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6306,11 +6361,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A12,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6323,11 +6378,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6335,11 +6390,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6347,11 +6402,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6359,11 +6414,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A13,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6376,11 +6431,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6388,11 +6443,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6400,11 +6455,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6412,11 +6467,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A14,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6429,11 +6484,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6441,11 +6496,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6453,11 +6508,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6465,11 +6520,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A15,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6482,11 +6537,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6494,11 +6549,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6506,11 +6561,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6518,11 +6573,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A16,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6535,11 +6590,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6547,11 +6602,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6559,11 +6614,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6571,11 +6626,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A17,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6588,11 +6643,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6600,11 +6655,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6612,11 +6667,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6624,11 +6679,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A18,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6641,11 +6696,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6653,11 +6708,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6665,11 +6720,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6677,11 +6732,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A19,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6694,11 +6749,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6706,11 +6761,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6718,11 +6773,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6730,11 +6785,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A20,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6747,11 +6802,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6759,11 +6814,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6771,11 +6826,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6783,11 +6838,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A21,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -6800,11 +6855,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -6812,11 +6867,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -6824,11 +6879,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -6836,11 +6891,11 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A22,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">
@@ -6853,11 +6908,11 @@
         <v>46287</v>
       </c>
       <c r="B23" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$98,Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="C23" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$98,Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="D23" s="8">
@@ -6865,11 +6920,11 @@
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$98,Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$98,Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="G23" s="10">
@@ -6877,11 +6932,11 @@
         <v/>
       </c>
       <c r="H23" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$98,Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="I23" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$98,Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="J23" s="10">
@@ -6889,11 +6944,11 @@
         <v/>
       </c>
       <c r="K23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"logged")</f>
         <v/>
       </c>
       <c r="L23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$98,$A23,Meals!$M$5:$M$98,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"pending")</f>
         <v/>
       </c>
       <c r="M23" s="19">

</xml_diff>

<commit_message>
Log Day 19 dinner: grilled chicken added to the green peas mess dinner
Tuesday serves 54.5 g of protein; a quarter grilled chicken plus one
chapati instead of two puts the day at 95.25 g before any whey - the
biggest structural fix made to a mess day in nineteen days.

Three scoops with the creamy sauce left lands 7 over target at 162.75 g
and a 541 deficit.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N99"/>
+  <dimension ref="A1:N100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5787,39 +5787,39 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>Ghee rice (halved) + chicken curry + raita</t>
+          <t>Quarter grilled chicken + green peas curry + 1 chapati + salad</t>
         </is>
       </c>
       <c r="D99" s="7" t="n">
-        <v>490</v>
+        <v>545</v>
       </c>
       <c r="E99" s="7" t="n">
-        <v>710</v>
+        <v>810</v>
       </c>
       <c r="F99" s="8">
         <f>AVERAGE(D99:E99)</f>
         <v/>
       </c>
       <c r="G99" s="9" t="n">
-        <v>26</v>
+        <v>44.5</v>
       </c>
       <c r="H99" s="9" t="n">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I99" s="10">
         <f>AVERAGE(G99:H99)</f>
         <v/>
       </c>
       <c r="J99" s="9" t="n">
-        <v>21</v>
+        <v>23.5</v>
       </c>
       <c r="K99" s="9" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="L99" s="10">
         <f>AVERAGE(J99:K99)</f>
@@ -5831,6 +5831,61 @@
         </is>
       </c>
       <c r="N99" s="6" t="inlineStr">
+        <is>
+          <t>Grilled chicken added to the mess dinner; 1 chapati not 2; creamy sauce container not counted</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>Ghee rice (halved) + chicken curry + raita</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="n">
+        <v>490</v>
+      </c>
+      <c r="E100" s="7" t="n">
+        <v>710</v>
+      </c>
+      <c r="F100" s="8">
+        <f>AVERAGE(D100:E100)</f>
+        <v/>
+      </c>
+      <c r="G100" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="H100" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I100" s="10">
+        <f>AVERAGE(G100:H100)</f>
+        <v/>
+      </c>
+      <c r="J100" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="K100" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="L100" s="10">
+        <f>AVERAGE(J100:K100)</f>
+        <v/>
+      </c>
+      <c r="M100" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N100" s="6" t="inlineStr">
         <is>
           <t>Rice halved; generous chicken portion</t>
         </is>
@@ -5954,11 +6009,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -5966,11 +6021,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -5978,11 +6033,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -5990,11 +6045,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A5,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -6007,11 +6062,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -6019,11 +6074,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -6031,11 +6086,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -6043,11 +6098,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A6,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -6060,11 +6115,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -6072,11 +6127,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -6084,11 +6139,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -6096,11 +6151,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A7,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -6113,11 +6168,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -6125,11 +6180,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -6137,11 +6192,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -6149,11 +6204,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A8,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -6166,11 +6221,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -6178,11 +6233,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -6190,11 +6245,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -6202,11 +6257,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A9,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -6219,11 +6274,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -6231,11 +6286,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -6243,11 +6298,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -6255,11 +6310,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A10,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -6272,11 +6327,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6284,11 +6339,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6296,11 +6351,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6308,11 +6363,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A11,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6325,11 +6380,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6337,11 +6392,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6349,11 +6404,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6361,11 +6416,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A12,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6378,11 +6433,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6390,11 +6445,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6402,11 +6457,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6414,11 +6469,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A13,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6431,11 +6486,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6443,11 +6498,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6455,11 +6510,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6467,11 +6522,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A14,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6484,11 +6539,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6496,11 +6551,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6508,11 +6563,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6520,11 +6575,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A15,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6537,11 +6592,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6549,11 +6604,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6561,11 +6616,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6573,11 +6628,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A16,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6590,11 +6645,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6602,11 +6657,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6614,11 +6669,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6626,11 +6681,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A17,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6643,11 +6698,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6655,11 +6710,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6667,11 +6722,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6679,11 +6734,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A18,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6696,11 +6751,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6708,11 +6763,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6720,11 +6775,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6732,11 +6787,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A19,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6749,11 +6804,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6761,11 +6816,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6773,11 +6828,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6785,11 +6840,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A20,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6802,11 +6857,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6814,11 +6869,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6826,11 +6881,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6838,11 +6893,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A21,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -6855,11 +6910,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -6867,11 +6922,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -6879,11 +6934,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -6891,11 +6946,11 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A22,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">
@@ -6908,11 +6963,11 @@
         <v>46287</v>
       </c>
       <c r="B23" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$99,Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="C23" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$99,Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="D23" s="8">
@@ -6920,11 +6975,11 @@
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$99,Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$99,Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="G23" s="10">
@@ -6932,11 +6987,11 @@
         <v/>
       </c>
       <c r="H23" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$99,Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="I23" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$99,Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="J23" s="10">
@@ -6944,11 +6999,11 @@
         <v/>
       </c>
       <c r="K23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"logged")</f>
         <v/>
       </c>
       <c r="L23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$99,$A23,Meals!$M$5:$M$99,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"pending")</f>
         <v/>
       </c>
       <c r="M23" s="19">

</xml_diff>

<commit_message>
Record two weigh-ins and reverse the trend reading
89.50 on 09-22 and 89.60 on 09-23. The scale has been flat for five days
and the last seven logged days average 2,343 kcal against a 2,120
target, predicting only 0.296 kg/wk - the two agree.

Four days ago the fit was running ahead of the food log and I read
above-target days as corrective. That is now wrong and the guidance is
reversed: back to 2,120. Every mess-based day in the week landed on
target; the overage is the snack layer, two garlic sauces and three
restaurant dinners.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -7025,7 +7025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7279,8 +7279,58 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B13" s="24" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="C13" s="25">
+        <f>B13-B12</f>
+        <v/>
+      </c>
+      <c r="D13" s="25">
+        <f>B13-$B$5</f>
+        <v/>
+      </c>
+      <c r="E13" s="26">
+        <f>AVERAGE(B7:B13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Morning weigh-in</t>
+        </is>
+      </c>
+    </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="4" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B14" s="24" t="n">
+        <v>89.59999999999999</v>
+      </c>
+      <c r="C14" s="25">
+        <f>B14-B13</f>
+        <v/>
+      </c>
+      <c r="D14" s="25">
+        <f>B14-$B$5</f>
+        <v/>
+      </c>
+      <c r="E14" s="26">
+        <f>AVERAGE(B8:B14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Morning weigh-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>A drop in the first week is mostly water and glycogen, not fat. Judge the trend over 2-3 weeks, and change the activity multiplier on Targets only then.</t>
         </is>

</xml_diff>

<commit_message>
Close Day 19 and log Day 20 breakfast
Day 19 closed at 1,782 kcal - the closing scoops went unreported again,
so 95.25 g of protein on an -886 deficit rather than 2,127 and 162.75 g.

Day 20 is Wednesday, a tight day. Rice halved, one chapati at dinner and
three scoops lands 40 under target at a 589 deficit.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N100"/>
+  <dimension ref="A1:N101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5891,6 +5891,61 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" s="4" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="inlineStr">
+        <is>
+          <t>Large plain dosa + sambar + red chutney (white chutney skipped)</t>
+        </is>
+      </c>
+      <c r="D101" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="E101" s="7" t="n">
+        <v>620</v>
+      </c>
+      <c r="F101" s="8">
+        <f>AVERAGE(D101:E101)</f>
+        <v/>
+      </c>
+      <c r="G101" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H101" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="I101" s="10">
+        <f>AVERAGE(G101:H101)</f>
+        <v/>
+      </c>
+      <c r="J101" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="K101" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="L101" s="10">
+        <f>AVERAGE(J101:K101)</f>
+        <v/>
+      </c>
+      <c r="M101" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N101" s="6" t="inlineStr">
+        <is>
+          <t>Plain rather than masala - no potato filling; tenth skip of the white chutney</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -5905,7 +5960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6009,11 +6064,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -6021,11 +6076,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -6033,11 +6088,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -6045,11 +6100,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A5,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -6062,11 +6117,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -6074,11 +6129,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -6086,11 +6141,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -6098,11 +6153,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A6,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -6115,11 +6170,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -6127,11 +6182,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -6139,11 +6194,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -6151,11 +6206,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A7,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -6168,11 +6223,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -6180,11 +6235,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -6192,11 +6247,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -6204,11 +6259,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A8,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -6221,11 +6276,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -6233,11 +6288,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -6245,11 +6300,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -6257,11 +6312,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A9,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -6274,11 +6329,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -6286,11 +6341,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -6298,11 +6353,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -6310,11 +6365,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A10,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -6327,11 +6382,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6339,11 +6394,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6351,11 +6406,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6363,11 +6418,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A11,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6380,11 +6435,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6392,11 +6447,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6404,11 +6459,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6416,11 +6471,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A12,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6433,11 +6488,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6445,11 +6500,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6457,11 +6512,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6469,11 +6524,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A13,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6486,11 +6541,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6498,11 +6553,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6510,11 +6565,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6522,11 +6577,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A14,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6539,11 +6594,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6551,11 +6606,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6563,11 +6618,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6575,11 +6630,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A15,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6592,11 +6647,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6604,11 +6659,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6616,11 +6671,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6628,11 +6683,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A16,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6645,11 +6700,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6657,11 +6712,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6669,11 +6724,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6681,11 +6736,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A17,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6698,11 +6753,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6710,11 +6765,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6722,11 +6777,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6734,11 +6789,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A18,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6751,11 +6806,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6763,11 +6818,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6775,11 +6830,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6787,11 +6842,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A19,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6804,11 +6859,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6816,11 +6871,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6828,11 +6883,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6840,11 +6895,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A20,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6857,11 +6912,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6869,11 +6924,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6881,11 +6936,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6893,11 +6948,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A21,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -6910,11 +6965,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -6922,11 +6977,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -6934,11 +6989,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -6946,11 +7001,11 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A22,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">
@@ -6963,11 +7018,11 @@
         <v>46287</v>
       </c>
       <c r="B23" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$100,Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="C23" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$100,Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="D23" s="8">
@@ -6975,11 +7030,11 @@
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$100,Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$100,Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="G23" s="10">
@@ -6987,11 +7042,11 @@
         <v/>
       </c>
       <c r="H23" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$100,Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="I23" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$100,Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="J23" s="10">
@@ -6999,15 +7054,68 @@
         <v/>
       </c>
       <c r="K23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"logged")</f>
         <v/>
       </c>
       <c r="L23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$100,$A23,Meals!$M$5:$M$100,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"pending")</f>
         <v/>
       </c>
       <c r="M23" s="19">
         <f>D23-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B24" s="21">
+        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"logged")</f>
+        <v/>
+      </c>
+      <c r="C24" s="21">
+        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"logged")</f>
+        <v/>
+      </c>
+      <c r="D24" s="21">
+        <f>AVERAGE(B24:C24)</f>
+        <v/>
+      </c>
+      <c r="E24" s="22">
+        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"logged")</f>
+        <v/>
+      </c>
+      <c r="F24" s="22">
+        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"logged")</f>
+        <v/>
+      </c>
+      <c r="G24" s="22">
+        <f>AVERAGE(E24:F24)</f>
+        <v/>
+      </c>
+      <c r="H24" s="22">
+        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"logged")</f>
+        <v/>
+      </c>
+      <c r="I24" s="22">
+        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"logged")</f>
+        <v/>
+      </c>
+      <c r="J24" s="22">
+        <f>AVERAGE(H24:I24)</f>
+        <v/>
+      </c>
+      <c r="K24" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"logged")</f>
+        <v/>
+      </c>
+      <c r="L24" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"pending")</f>
+        <v/>
+      </c>
+      <c r="M24" s="23">
+        <f>D24-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -8091,7 +8199,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$23)</f>
+        <f>COUNT(Daily!$A$5:$A$24)</f>
         <v/>
       </c>
     </row>
@@ -8102,7 +8210,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$23),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$24),0)</f>
         <v/>
       </c>
     </row>
@@ -8113,7 +8221,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$23),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$24),0)</f>
         <v/>
       </c>
     </row>
@@ -8124,7 +8232,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$23),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$24),0)</f>
         <v/>
       </c>
     </row>
@@ -8168,7 +8276,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$23,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$24,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -8179,7 +8287,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$23)</f>
+        <f>SUM(Daily!$L$5:$L$24)</f>
         <v/>
       </c>
     </row>
@@ -8230,19 +8338,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$23,"&gt;="&amp;$A17,Daily!$A$5:$A$23,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$24,"&gt;="&amp;$A17,Daily!$A$5:$A$24,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$23,Daily!$A$5:$A$23,"&gt;="&amp;$A17,Daily!$A$5:$A$23,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$24,Daily!$A$5:$A$24,"&gt;="&amp;$A17,Daily!$A$5:$A$24,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$23,Daily!$A$5:$A$23,"&gt;="&amp;$A17,Daily!$A$5:$A$23,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$24,Daily!$A$5:$A$24,"&gt;="&amp;$A17,Daily!$A$5:$A$24,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$23,Daily!$A$5:$A$23,"&gt;="&amp;$A17,Daily!$A$5:$A$23,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$24,Daily!$A$5:$A$24,"&gt;="&amp;$A17,Daily!$A$5:$A$24,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -8254,19 +8362,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$23,"&gt;="&amp;$A18,Daily!$A$5:$A$23,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$24,"&gt;="&amp;$A18,Daily!$A$5:$A$24,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$23,Daily!$A$5:$A$23,"&gt;="&amp;$A18,Daily!$A$5:$A$23,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$24,Daily!$A$5:$A$24,"&gt;="&amp;$A18,Daily!$A$5:$A$24,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$23,Daily!$A$5:$A$23,"&gt;="&amp;$A18,Daily!$A$5:$A$23,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$24,Daily!$A$5:$A$24,"&gt;="&amp;$A18,Daily!$A$5:$A$24,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$23,Daily!$A$5:$A$23,"&gt;="&amp;$A18,Daily!$A$5:$A$23,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$24,Daily!$A$5:$A$24,"&gt;="&amp;$A18,Daily!$A$5:$A$24,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -8278,19 +8386,19 @@
         <v>46285</v>
       </c>
       <c r="C19" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$23,"&gt;="&amp;$A19,Daily!$A$5:$A$23,"&lt;="&amp;$B19)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$24,"&gt;="&amp;$A19,Daily!$A$5:$A$24,"&lt;="&amp;$B19)</f>
         <v/>
       </c>
       <c r="D19" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$23,Daily!$A$5:$A$23,"&gt;="&amp;$A19,Daily!$A$5:$A$23,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$24,Daily!$A$5:$A$24,"&gt;="&amp;$A19,Daily!$A$5:$A$24,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$23,Daily!$A$5:$A$23,"&gt;="&amp;$A19,Daily!$A$5:$A$23,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$24,Daily!$A$5:$A$24,"&gt;="&amp;$A19,Daily!$A$5:$A$24,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$23,Daily!$A$5:$A$23,"&gt;="&amp;$A19,Daily!$A$5:$A$23,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$24,Daily!$A$5:$A$24,"&gt;="&amp;$A19,Daily!$A$5:$A$24,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
     </row>
@@ -8302,19 +8410,19 @@
         <v>46292</v>
       </c>
       <c r="C20" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$23,"&gt;="&amp;$A20,Daily!$A$5:$A$23,"&lt;="&amp;$B20)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$24,"&gt;="&amp;$A20,Daily!$A$5:$A$24,"&lt;="&amp;$B20)</f>
         <v/>
       </c>
       <c r="D20" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$23,Daily!$A$5:$A$23,"&gt;="&amp;$A20,Daily!$A$5:$A$23,"&lt;="&amp;$B20),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$24,Daily!$A$5:$A$24,"&gt;="&amp;$A20,Daily!$A$5:$A$24,"&lt;="&amp;$B20),0)</f>
         <v/>
       </c>
       <c r="E20" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$23,Daily!$A$5:$A$23,"&gt;="&amp;$A20,Daily!$A$5:$A$23,"&lt;="&amp;$B20),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$24,Daily!$A$5:$A$24,"&gt;="&amp;$A20,Daily!$A$5:$A$24,"&lt;="&amp;$B20),0)</f>
         <v/>
       </c>
       <c r="F20" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$23,Daily!$A$5:$A$23,"&gt;="&amp;$A20,Daily!$A$5:$A$23,"&lt;="&amp;$B20),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$24,Daily!$A$5:$A$24,"&gt;="&amp;$A20,Daily!$A$5:$A$24,"&lt;="&amp;$B20),0)</f>
         <v/>
       </c>
     </row>
@@ -8365,19 +8473,19 @@
         <v>46295</v>
       </c>
       <c r="C24" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$23,"&gt;="&amp;$A24,Daily!$A$5:$A$23,"&lt;="&amp;$B24)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$24,"&gt;="&amp;$A24,Daily!$A$5:$A$24,"&lt;="&amp;$B24)</f>
         <v/>
       </c>
       <c r="D24" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$23,Daily!$A$5:$A$23,"&gt;="&amp;$A24,Daily!$A$5:$A$23,"&lt;="&amp;$B24),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$24,Daily!$A$5:$A$24,"&gt;="&amp;$A24,Daily!$A$5:$A$24,"&lt;="&amp;$B24),0)</f>
         <v/>
       </c>
       <c r="E24" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$23,Daily!$A$5:$A$23,"&gt;="&amp;$A24,Daily!$A$5:$A$23,"&lt;="&amp;$B24),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$24,Daily!$A$5:$A$24,"&gt;="&amp;$A24,Daily!$A$5:$A$24,"&lt;="&amp;$B24),0)</f>
         <v/>
       </c>
       <c r="F24" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$23,Daily!$A$5:$A$23,"&gt;="&amp;$A24,Daily!$A$5:$A$23,"&lt;="&amp;$B24),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$24,Daily!$A$5:$A$24,"&gt;="&amp;$A24,Daily!$A$5:$A$24,"&lt;="&amp;$B24),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Day 20 lunch: meals plate with a 2-egg omelette
Plate only - the three side containers are uncounted and the rice was
not stated as halved, together worth ~370 kcal.

One chapati at dinner and three scoops lands 15 under target at 135 g
and a 564 deficit; eating the containers would take that to 314.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N101"/>
+  <dimension ref="A1:N102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5943,6 +5943,61 @@
       <c r="N101" s="6" t="inlineStr">
         <is>
           <t>Plain rather than masala - no potato filling; tenth skip of the white chutney</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>Mess meals plate + 2-egg omelette, pappadam, veg curry, chammanthi, pickle</t>
+        </is>
+      </c>
+      <c r="D102" s="7" t="n">
+        <v>630</v>
+      </c>
+      <c r="E102" s="7" t="n">
+        <v>940</v>
+      </c>
+      <c r="F102" s="8">
+        <f>AVERAGE(D102:E102)</f>
+        <v/>
+      </c>
+      <c r="G102" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="H102" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="I102" s="10">
+        <f>AVERAGE(G102:H102)</f>
+        <v/>
+      </c>
+      <c r="J102" s="9" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="K102" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="L102" s="10">
+        <f>AVERAGE(J102:K102)</f>
+        <v/>
+      </c>
+      <c r="M102" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N102" s="6" t="inlineStr">
+        <is>
+          <t>Plate only - three side containers not counted; rice not stated as halved</t>
         </is>
       </c>
     </row>
@@ -6064,11 +6119,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -6076,11 +6131,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -6088,11 +6143,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -6100,11 +6155,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A5,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -6117,11 +6172,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -6129,11 +6184,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -6141,11 +6196,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -6153,11 +6208,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A6,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -6170,11 +6225,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -6182,11 +6237,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -6194,11 +6249,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -6206,11 +6261,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A7,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -6223,11 +6278,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -6235,11 +6290,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -6247,11 +6302,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -6259,11 +6314,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A8,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -6276,11 +6331,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -6288,11 +6343,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -6300,11 +6355,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -6312,11 +6367,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A9,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -6329,11 +6384,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -6341,11 +6396,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -6353,11 +6408,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -6365,11 +6420,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A10,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -6382,11 +6437,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6394,11 +6449,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6406,11 +6461,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6418,11 +6473,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A11,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6435,11 +6490,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6447,11 +6502,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6459,11 +6514,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6471,11 +6526,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A12,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6488,11 +6543,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6500,11 +6555,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6512,11 +6567,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6524,11 +6579,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A13,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6541,11 +6596,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6553,11 +6608,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6565,11 +6620,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6577,11 +6632,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A14,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6594,11 +6649,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6606,11 +6661,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6618,11 +6673,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6630,11 +6685,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A15,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6647,11 +6702,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6659,11 +6714,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6671,11 +6726,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6683,11 +6738,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A16,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6700,11 +6755,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6712,11 +6767,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6724,11 +6779,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6736,11 +6791,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A17,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6753,11 +6808,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6765,11 +6820,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6777,11 +6832,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6789,11 +6844,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A18,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6806,11 +6861,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6818,11 +6873,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6830,11 +6885,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6842,11 +6897,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A19,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6859,11 +6914,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6871,11 +6926,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6883,11 +6938,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6895,11 +6950,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A20,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6912,11 +6967,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6924,11 +6979,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6936,11 +6991,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -6948,11 +7003,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A21,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -6965,11 +7020,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -6977,11 +7032,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -6989,11 +7044,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -7001,11 +7056,11 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A22,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">
@@ -7018,11 +7073,11 @@
         <v>46287</v>
       </c>
       <c r="B23" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C23" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D23" s="8">
@@ -7030,11 +7085,11 @@
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G23" s="10">
@@ -7042,11 +7097,11 @@
         <v/>
       </c>
       <c r="H23" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I23" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J23" s="10">
@@ -7054,11 +7109,11 @@
         <v/>
       </c>
       <c r="K23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A23,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M23" s="19">
@@ -7071,11 +7126,11 @@
         <v>46288</v>
       </c>
       <c r="B24" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$101,Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="C24" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$101,Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="D24" s="21">
@@ -7083,11 +7138,11 @@
         <v/>
       </c>
       <c r="E24" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$101,Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="F24" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$101,Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="G24" s="22">
@@ -7095,11 +7150,11 @@
         <v/>
       </c>
       <c r="H24" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$101,Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="I24" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$101,Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="J24" s="22">
@@ -7107,11 +7162,11 @@
         <v/>
       </c>
       <c r="K24" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"logged")</f>
         <v/>
       </c>
       <c r="L24" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$101,$A24,Meals!$M$5:$M$101,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"pending")</f>
         <v/>
       </c>
       <c r="M24" s="23">

</xml_diff>

<commit_message>
Log a second omelette on Day 20
Three eggs' worth so far, which is what has kept protein moving on a
lunch plate with no meat or fish.

Closing on chicken curry without the chapati plus three scoops: 2,105
and 138.5 g, against 119.5 g for the same calories with the chapati.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N102"/>
+  <dimension ref="A1:N103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5998,6 +5998,61 @@
       <c r="N102" s="6" t="inlineStr">
         <is>
           <t>Plate only - three side containers not counted; rice not stated as halved</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C103" s="6" t="inlineStr">
+        <is>
+          <t>1-egg omelette</t>
+        </is>
+      </c>
+      <c r="D103" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="E103" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="F103" s="8">
+        <f>AVERAGE(D103:E103)</f>
+        <v/>
+      </c>
+      <c r="G103" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H103" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="I103" s="10">
+        <f>AVERAGE(G103:H103)</f>
+        <v/>
+      </c>
+      <c r="J103" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="K103" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="L103" s="10">
+        <f>AVERAGE(J103:K103)</f>
+        <v/>
+      </c>
+      <c r="M103" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N103" s="6" t="inlineStr">
+        <is>
+          <t>Second omelette of the day</t>
         </is>
       </c>
     </row>
@@ -6119,11 +6174,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -6131,11 +6186,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -6143,11 +6198,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -6155,11 +6210,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A5,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -6172,11 +6227,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -6184,11 +6239,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -6196,11 +6251,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -6208,11 +6263,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A6,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -6225,11 +6280,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -6237,11 +6292,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -6249,11 +6304,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -6261,11 +6316,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A7,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -6278,11 +6333,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -6290,11 +6345,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -6302,11 +6357,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -6314,11 +6369,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A8,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -6331,11 +6386,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -6343,11 +6398,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -6355,11 +6410,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -6367,11 +6422,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A9,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -6384,11 +6439,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -6396,11 +6451,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -6408,11 +6463,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -6420,11 +6475,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A10,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -6437,11 +6492,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6449,11 +6504,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6461,11 +6516,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6473,11 +6528,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A11,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6490,11 +6545,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6502,11 +6557,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6514,11 +6569,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6526,11 +6581,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A12,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6543,11 +6598,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6555,11 +6610,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6567,11 +6622,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6579,11 +6634,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A13,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6596,11 +6651,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6608,11 +6663,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6620,11 +6675,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6632,11 +6687,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A14,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6649,11 +6704,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6661,11 +6716,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6673,11 +6728,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6685,11 +6740,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A15,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6702,11 +6757,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6714,11 +6769,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6726,11 +6781,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6738,11 +6793,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A16,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6755,11 +6810,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6767,11 +6822,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6779,11 +6834,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6791,11 +6846,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A17,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6808,11 +6863,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6820,11 +6875,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6832,11 +6887,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6844,11 +6899,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A18,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6861,11 +6916,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6873,11 +6928,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6885,11 +6940,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6897,11 +6952,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A19,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6914,11 +6969,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6926,11 +6981,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6938,11 +6993,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -6950,11 +7005,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A20,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -6967,11 +7022,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -6979,11 +7034,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -6991,11 +7046,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -7003,11 +7058,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A21,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -7020,11 +7075,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -7032,11 +7087,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -7044,11 +7099,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -7056,11 +7111,11 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A22,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">
@@ -7073,11 +7128,11 @@
         <v>46287</v>
       </c>
       <c r="B23" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C23" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D23" s="8">
@@ -7085,11 +7140,11 @@
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G23" s="10">
@@ -7097,11 +7152,11 @@
         <v/>
       </c>
       <c r="H23" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I23" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J23" s="10">
@@ -7109,11 +7164,11 @@
         <v/>
       </c>
       <c r="K23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A23,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M23" s="19">
@@ -7126,11 +7181,11 @@
         <v>46288</v>
       </c>
       <c r="B24" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$102,Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="C24" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$102,Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="D24" s="21">
@@ -7138,11 +7193,11 @@
         <v/>
       </c>
       <c r="E24" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$102,Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="F24" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$102,Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="G24" s="22">
@@ -7150,11 +7205,11 @@
         <v/>
       </c>
       <c r="H24" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$102,Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="I24" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$102,Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="J24" s="22">
@@ -7162,11 +7217,11 @@
         <v/>
       </c>
       <c r="K24" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"logged")</f>
         <v/>
       </c>
       <c r="L24" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$102,$A24,Meals!$M$5:$M$102,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"pending")</f>
         <v/>
       </c>
       <c r="M24" s="23">

</xml_diff>

<commit_message>
Log Day 20 dinner: 2 chapati with a small chicken curry
Came in ~120 under the menu on a two-piece chicken portion. Closing on
three scoops: 2,215 kcal and 138.5 g, still below the last seven days'
2,286 average, against 116 g for two scoops on target.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N103"/>
+  <dimension ref="A1:N104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5952,39 +5952,39 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C102" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate + 2-egg omelette, pappadam, veg curry, chammanthi, pickle</t>
+          <t>2 chapati + chicken curry (2 small pieces)</t>
         </is>
       </c>
       <c r="D102" s="7" t="n">
-        <v>630</v>
+        <v>380</v>
       </c>
       <c r="E102" s="7" t="n">
-        <v>940</v>
+        <v>540</v>
       </c>
       <c r="F102" s="8">
         <f>AVERAGE(D102:E102)</f>
         <v/>
       </c>
       <c r="G102" s="9" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H102" s="9" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="I102" s="10">
         <f>AVERAGE(G102:H102)</f>
         <v/>
       </c>
       <c r="J102" s="9" t="n">
-        <v>27.5</v>
+        <v>16</v>
       </c>
       <c r="K102" s="9" t="n">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="L102" s="10">
         <f>AVERAGE(J102:K102)</f>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="N102" s="6" t="inlineStr">
         <is>
-          <t>Plate only - three side containers not counted; rice not stated as halved</t>
+          <t>Small chicken portion; gravy poured over both chapati</t>
         </is>
       </c>
     </row>
@@ -6007,39 +6007,39 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
         <is>
-          <t>1-egg omelette</t>
+          <t>Mess meals plate + 2-egg omelette, pappadam, veg curry, chammanthi, pickle</t>
         </is>
       </c>
       <c r="D103" s="7" t="n">
-        <v>90</v>
+        <v>630</v>
       </c>
       <c r="E103" s="7" t="n">
-        <v>140</v>
+        <v>940</v>
       </c>
       <c r="F103" s="8">
         <f>AVERAGE(D103:E103)</f>
         <v/>
       </c>
       <c r="G103" s="9" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="H103" s="9" t="n">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="I103" s="10">
         <f>AVERAGE(G103:H103)</f>
         <v/>
       </c>
       <c r="J103" s="9" t="n">
-        <v>7</v>
+        <v>27.5</v>
       </c>
       <c r="K103" s="9" t="n">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="L103" s="10">
         <f>AVERAGE(J103:K103)</f>
@@ -6051,6 +6051,61 @@
         </is>
       </c>
       <c r="N103" s="6" t="inlineStr">
+        <is>
+          <t>Plate only - three side containers not counted; rice not stated as halved</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="inlineStr">
+        <is>
+          <t>1-egg omelette</t>
+        </is>
+      </c>
+      <c r="D104" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="E104" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="F104" s="8">
+        <f>AVERAGE(D104:E104)</f>
+        <v/>
+      </c>
+      <c r="G104" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H104" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="I104" s="10">
+        <f>AVERAGE(G104:H104)</f>
+        <v/>
+      </c>
+      <c r="J104" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="K104" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="L104" s="10">
+        <f>AVERAGE(J104:K104)</f>
+        <v/>
+      </c>
+      <c r="M104" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N104" s="6" t="inlineStr">
         <is>
           <t>Second omelette of the day</t>
         </is>
@@ -6174,11 +6229,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -6186,11 +6241,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -6198,11 +6253,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -6210,11 +6265,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A5,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -6227,11 +6282,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -6239,11 +6294,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -6251,11 +6306,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -6263,11 +6318,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A6,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -6280,11 +6335,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -6292,11 +6347,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -6304,11 +6359,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -6316,11 +6371,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A7,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -6333,11 +6388,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -6345,11 +6400,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -6357,11 +6412,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -6369,11 +6424,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A8,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -6386,11 +6441,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -6398,11 +6453,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -6410,11 +6465,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -6422,11 +6477,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A9,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -6439,11 +6494,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -6451,11 +6506,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -6463,11 +6518,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -6475,11 +6530,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A10,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -6492,11 +6547,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6504,11 +6559,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6516,11 +6571,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6528,11 +6583,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A11,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6545,11 +6600,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6557,11 +6612,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6569,11 +6624,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6581,11 +6636,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A12,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6598,11 +6653,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6610,11 +6665,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6622,11 +6677,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6634,11 +6689,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A13,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6651,11 +6706,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6663,11 +6718,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6675,11 +6730,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6687,11 +6742,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A14,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6704,11 +6759,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6716,11 +6771,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6728,11 +6783,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6740,11 +6795,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A15,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6757,11 +6812,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6769,11 +6824,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6781,11 +6836,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6793,11 +6848,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A16,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6810,11 +6865,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6822,11 +6877,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6834,11 +6889,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6846,11 +6901,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A17,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6863,11 +6918,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6875,11 +6930,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6887,11 +6942,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6899,11 +6954,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A18,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6916,11 +6971,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6928,11 +6983,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6940,11 +6995,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -6952,11 +7007,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A19,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -6969,11 +7024,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -6981,11 +7036,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -6993,11 +7048,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -7005,11 +7060,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A20,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -7022,11 +7077,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -7034,11 +7089,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -7046,11 +7101,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -7058,11 +7113,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A21,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -7075,11 +7130,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -7087,11 +7142,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -7099,11 +7154,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -7111,11 +7166,11 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A22,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">
@@ -7128,11 +7183,11 @@
         <v>46287</v>
       </c>
       <c r="B23" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C23" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D23" s="8">
@@ -7140,11 +7195,11 @@
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G23" s="10">
@@ -7152,11 +7207,11 @@
         <v/>
       </c>
       <c r="H23" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I23" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J23" s="10">
@@ -7164,11 +7219,11 @@
         <v/>
       </c>
       <c r="K23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A23,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M23" s="19">
@@ -7181,11 +7236,11 @@
         <v>46288</v>
       </c>
       <c r="B24" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$103,Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="C24" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$103,Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="D24" s="21">
@@ -7193,11 +7248,11 @@
         <v/>
       </c>
       <c r="E24" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$103,Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="F24" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$103,Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="G24" s="22">
@@ -7205,11 +7260,11 @@
         <v/>
       </c>
       <c r="H24" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$103,Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="I24" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$103,Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="J24" s="22">
@@ -7217,11 +7272,11 @@
         <v/>
       </c>
       <c r="K24" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"logged")</f>
         <v/>
       </c>
       <c r="L24" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$103,$A24,Meals!$M$5:$M$103,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"pending")</f>
         <v/>
       </c>
       <c r="M24" s="23">

</xml_diff>

<commit_message>
Log 89.15 weigh-in and close Day 20 at 71 g protein
The five-day flat patch breaks, but a single reading swings the fitted
rate by 0.22 kg/wk, so guidance stays at 2,120. Day 20 closed without
the planned scoops - lowest protein day of the twenty logged.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -7298,7 +7298,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7602,8 +7602,33 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="27" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B15" s="24" t="n">
+        <v>89.15000000000001</v>
+      </c>
+      <c r="C15" s="25">
+        <f>B15-B14</f>
+        <v/>
+      </c>
+      <c r="D15" s="25">
+        <f>B15-$B$5</f>
+        <v/>
+      </c>
+      <c r="E15" s="26">
+        <f>AVERAGE(B9:B15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Morning weigh-in - largest single-day drop in the log</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="inlineStr">
         <is>
           <t>A drop in the first week is mostly water and glycogen, not fat. Judge the trend over 2-3 weeks, and change the activity multiplier on Targets only then.</t>
         </is>

</xml_diff>

<commit_message>
Log Day 21 breakfast: ghee roast dosa, white chutney skipped
Opens Thursday, the second protein desert on the mess menu, the day
after the lowest-protein day of the log.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N104"/>
+  <dimension ref="A1:N105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6111,6 +6111,61 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" s="4" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C105" s="6" t="inlineStr">
+        <is>
+          <t>Large ghee roast dosa + sambar + red chutney (white chutney skipped)</t>
+        </is>
+      </c>
+      <c r="D105" s="7" t="n">
+        <v>440</v>
+      </c>
+      <c r="E105" s="7" t="n">
+        <v>680</v>
+      </c>
+      <c r="F105" s="8">
+        <f>AVERAGE(D105:E105)</f>
+        <v/>
+      </c>
+      <c r="G105" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H105" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="I105" s="10">
+        <f>AVERAGE(G105:H105)</f>
+        <v/>
+      </c>
+      <c r="J105" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="K105" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="L105" s="10">
+        <f>AVERAGE(J105:K105)</f>
+        <v/>
+      </c>
+      <c r="M105" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N105" s="6" t="inlineStr">
+        <is>
+          <t>Restaurant ghee roast - larger and ghee-fried; eleventh consecutive white chutney skip</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -6125,7 +6180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6229,11 +6284,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -6241,11 +6296,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -6253,11 +6308,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -6265,11 +6320,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A5,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -6282,11 +6337,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -6294,11 +6349,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -6306,11 +6361,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -6318,11 +6373,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A6,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -6335,11 +6390,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -6347,11 +6402,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -6359,11 +6414,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -6371,11 +6426,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A7,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -6388,11 +6443,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -6400,11 +6455,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -6412,11 +6467,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -6424,11 +6479,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A8,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -6441,11 +6496,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -6453,11 +6508,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -6465,11 +6520,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -6477,11 +6532,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A9,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -6494,11 +6549,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -6506,11 +6561,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -6518,11 +6573,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -6530,11 +6585,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A10,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -6547,11 +6602,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6559,11 +6614,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6571,11 +6626,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6583,11 +6638,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A11,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6600,11 +6655,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6612,11 +6667,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6624,11 +6679,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6636,11 +6691,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A12,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6653,11 +6708,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6665,11 +6720,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6677,11 +6732,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6689,11 +6744,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A13,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6706,11 +6761,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6718,11 +6773,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6730,11 +6785,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6742,11 +6797,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A14,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6759,11 +6814,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6771,11 +6826,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6783,11 +6838,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6795,11 +6850,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A15,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6812,11 +6867,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6824,11 +6879,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6836,11 +6891,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6848,11 +6903,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A16,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6865,11 +6920,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6877,11 +6932,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6889,11 +6944,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6901,11 +6956,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A17,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6918,11 +6973,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6930,11 +6985,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6942,11 +6997,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -6954,11 +7009,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A18,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -6971,11 +7026,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -6983,11 +7038,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -6995,11 +7050,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -7007,11 +7062,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A19,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -7024,11 +7079,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -7036,11 +7091,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -7048,11 +7103,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -7060,11 +7115,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A20,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -7077,11 +7132,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -7089,11 +7144,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -7101,11 +7156,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -7113,11 +7168,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A21,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -7130,11 +7185,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -7142,11 +7197,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -7154,11 +7209,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -7166,11 +7221,11 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A22,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">
@@ -7183,11 +7238,11 @@
         <v>46287</v>
       </c>
       <c r="B23" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C23" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D23" s="8">
@@ -7195,11 +7250,11 @@
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G23" s="10">
@@ -7207,11 +7262,11 @@
         <v/>
       </c>
       <c r="H23" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I23" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J23" s="10">
@@ -7219,11 +7274,11 @@
         <v/>
       </c>
       <c r="K23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A23,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M23" s="19">
@@ -7236,11 +7291,11 @@
         <v>46288</v>
       </c>
       <c r="B24" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$104,Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="C24" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$104,Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="D24" s="21">
@@ -7248,11 +7303,11 @@
         <v/>
       </c>
       <c r="E24" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$104,Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="F24" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$104,Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="G24" s="22">
@@ -7260,11 +7315,11 @@
         <v/>
       </c>
       <c r="H24" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$104,Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="I24" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$104,Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="J24" s="22">
@@ -7272,15 +7327,68 @@
         <v/>
       </c>
       <c r="K24" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"logged")</f>
         <v/>
       </c>
       <c r="L24" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$104,$A24,Meals!$M$5:$M$104,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"pending")</f>
         <v/>
       </c>
       <c r="M24" s="23">
         <f>D24-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B25" s="8">
+        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"logged")</f>
+        <v/>
+      </c>
+      <c r="C25" s="8">
+        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"logged")</f>
+        <v/>
+      </c>
+      <c r="D25" s="8">
+        <f>AVERAGE(B25:C25)</f>
+        <v/>
+      </c>
+      <c r="E25" s="10">
+        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"logged")</f>
+        <v/>
+      </c>
+      <c r="F25" s="10">
+        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"logged")</f>
+        <v/>
+      </c>
+      <c r="G25" s="10">
+        <f>AVERAGE(E25:F25)</f>
+        <v/>
+      </c>
+      <c r="H25" s="10">
+        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"logged")</f>
+        <v/>
+      </c>
+      <c r="I25" s="10">
+        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"logged")</f>
+        <v/>
+      </c>
+      <c r="J25" s="10">
+        <f>AVERAGE(H25:I25)</f>
+        <v/>
+      </c>
+      <c r="K25" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"logged")</f>
+        <v/>
+      </c>
+      <c r="L25" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"pending")</f>
+        <v/>
+      </c>
+      <c r="M25" s="19">
+        <f>D25-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -8389,7 +8497,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$24)</f>
+        <f>COUNT(Daily!$A$5:$A$25)</f>
         <v/>
       </c>
     </row>
@@ -8400,7 +8508,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$24),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$25),0)</f>
         <v/>
       </c>
     </row>
@@ -8411,7 +8519,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$24),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$25),0)</f>
         <v/>
       </c>
     </row>
@@ -8422,7 +8530,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$24),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$25),0)</f>
         <v/>
       </c>
     </row>
@@ -8466,7 +8574,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$24,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$25,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -8477,7 +8585,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$24)</f>
+        <f>SUM(Daily!$L$5:$L$25)</f>
         <v/>
       </c>
     </row>
@@ -8528,19 +8636,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$24,"&gt;="&amp;$A17,Daily!$A$5:$A$24,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$25,"&gt;="&amp;$A17,Daily!$A$5:$A$25,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$24,Daily!$A$5:$A$24,"&gt;="&amp;$A17,Daily!$A$5:$A$24,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$25,Daily!$A$5:$A$25,"&gt;="&amp;$A17,Daily!$A$5:$A$25,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$24,Daily!$A$5:$A$24,"&gt;="&amp;$A17,Daily!$A$5:$A$24,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$25,Daily!$A$5:$A$25,"&gt;="&amp;$A17,Daily!$A$5:$A$25,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$24,Daily!$A$5:$A$24,"&gt;="&amp;$A17,Daily!$A$5:$A$24,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$25,Daily!$A$5:$A$25,"&gt;="&amp;$A17,Daily!$A$5:$A$25,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -8552,19 +8660,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$24,"&gt;="&amp;$A18,Daily!$A$5:$A$24,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$25,"&gt;="&amp;$A18,Daily!$A$5:$A$25,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$24,Daily!$A$5:$A$24,"&gt;="&amp;$A18,Daily!$A$5:$A$24,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$25,Daily!$A$5:$A$25,"&gt;="&amp;$A18,Daily!$A$5:$A$25,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$24,Daily!$A$5:$A$24,"&gt;="&amp;$A18,Daily!$A$5:$A$24,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$25,Daily!$A$5:$A$25,"&gt;="&amp;$A18,Daily!$A$5:$A$25,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$24,Daily!$A$5:$A$24,"&gt;="&amp;$A18,Daily!$A$5:$A$24,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$25,Daily!$A$5:$A$25,"&gt;="&amp;$A18,Daily!$A$5:$A$25,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -8576,19 +8684,19 @@
         <v>46285</v>
       </c>
       <c r="C19" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$24,"&gt;="&amp;$A19,Daily!$A$5:$A$24,"&lt;="&amp;$B19)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$25,"&gt;="&amp;$A19,Daily!$A$5:$A$25,"&lt;="&amp;$B19)</f>
         <v/>
       </c>
       <c r="D19" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$24,Daily!$A$5:$A$24,"&gt;="&amp;$A19,Daily!$A$5:$A$24,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$25,Daily!$A$5:$A$25,"&gt;="&amp;$A19,Daily!$A$5:$A$25,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$24,Daily!$A$5:$A$24,"&gt;="&amp;$A19,Daily!$A$5:$A$24,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$25,Daily!$A$5:$A$25,"&gt;="&amp;$A19,Daily!$A$5:$A$25,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$24,Daily!$A$5:$A$24,"&gt;="&amp;$A19,Daily!$A$5:$A$24,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$25,Daily!$A$5:$A$25,"&gt;="&amp;$A19,Daily!$A$5:$A$25,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
     </row>
@@ -8600,19 +8708,19 @@
         <v>46292</v>
       </c>
       <c r="C20" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$24,"&gt;="&amp;$A20,Daily!$A$5:$A$24,"&lt;="&amp;$B20)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$25,"&gt;="&amp;$A20,Daily!$A$5:$A$25,"&lt;="&amp;$B20)</f>
         <v/>
       </c>
       <c r="D20" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$24,Daily!$A$5:$A$24,"&gt;="&amp;$A20,Daily!$A$5:$A$24,"&lt;="&amp;$B20),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$25,Daily!$A$5:$A$25,"&gt;="&amp;$A20,Daily!$A$5:$A$25,"&lt;="&amp;$B20),0)</f>
         <v/>
       </c>
       <c r="E20" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$24,Daily!$A$5:$A$24,"&gt;="&amp;$A20,Daily!$A$5:$A$24,"&lt;="&amp;$B20),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$25,Daily!$A$5:$A$25,"&gt;="&amp;$A20,Daily!$A$5:$A$25,"&lt;="&amp;$B20),0)</f>
         <v/>
       </c>
       <c r="F20" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$24,Daily!$A$5:$A$24,"&gt;="&amp;$A20,Daily!$A$5:$A$24,"&lt;="&amp;$B20),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$25,Daily!$A$5:$A$25,"&gt;="&amp;$A20,Daily!$A$5:$A$25,"&lt;="&amp;$B20),0)</f>
         <v/>
       </c>
     </row>
@@ -8663,19 +8771,19 @@
         <v>46295</v>
       </c>
       <c r="C24" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$24,"&gt;="&amp;$A24,Daily!$A$5:$A$24,"&lt;="&amp;$B24)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$25,"&gt;="&amp;$A24,Daily!$A$5:$A$25,"&lt;="&amp;$B24)</f>
         <v/>
       </c>
       <c r="D24" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$24,Daily!$A$5:$A$24,"&gt;="&amp;$A24,Daily!$A$5:$A$24,"&lt;="&amp;$B24),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$25,Daily!$A$5:$A$25,"&gt;="&amp;$A24,Daily!$A$5:$A$25,"&lt;="&amp;$B24),0)</f>
         <v/>
       </c>
       <c r="E24" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$24,Daily!$A$5:$A$24,"&gt;="&amp;$A24,Daily!$A$5:$A$24,"&lt;="&amp;$B24),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$25,Daily!$A$5:$A$25,"&gt;="&amp;$A24,Daily!$A$5:$A$25,"&lt;="&amp;$B24),0)</f>
         <v/>
       </c>
       <c r="F24" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$24,Daily!$A$5:$A$24,"&gt;="&amp;$A24,Daily!$A$5:$A$24,"&lt;="&amp;$B24),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$25,Daily!$A$5:$A$25,"&gt;="&amp;$A24,Daily!$A$5:$A$25,"&lt;="&amp;$B24),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct Day 21 breakfast: plain dosa, not ghee roast
Drops the day's opening from 560 to 510 kcal and the fat from 29 to 25 g.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -6122,14 +6122,14 @@
       </c>
       <c r="C105" s="6" t="inlineStr">
         <is>
-          <t>Large ghee roast dosa + sambar + red chutney (white chutney skipped)</t>
+          <t>Large plain dosa + sambar + red chutney (white chutney skipped)</t>
         </is>
       </c>
       <c r="D105" s="7" t="n">
-        <v>440</v>
+        <v>400</v>
       </c>
       <c r="E105" s="7" t="n">
-        <v>680</v>
+        <v>620</v>
       </c>
       <c r="F105" s="8">
         <f>AVERAGE(D105:E105)</f>
@@ -6146,10 +6146,10 @@
         <v/>
       </c>
       <c r="J105" s="9" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K105" s="9" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="L105" s="10">
         <f>AVERAGE(J105:K105)</f>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="N105" s="6" t="inlineStr">
         <is>
-          <t>Restaurant ghee roast - larger and ghee-fried; eleventh consecutive white chutney skip</t>
+          <t>Plain dosa - not the menu's ghee roast; eleventh consecutive white chutney skip</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Day 21 lunch: halved mess plate with a chicken fry piece
710 kcal against the menu's 950; the chicken fry supplies most of the
plate's protein on a menu day that lists no meat.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N105"/>
+  <dimension ref="A1:N106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6163,6 +6163,61 @@
       <c r="N105" s="6" t="inlineStr">
         <is>
           <t>Plain dosa - not the menu's ghee roast; eleventh consecutive white chutney skip</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="inlineStr">
+        <is>
+          <t>Mess meals plate - rice halved, pappadam, cabbage thoran, dal, curry gravy, 1 small chicken fry piece, small curd</t>
+        </is>
+      </c>
+      <c r="D106" s="7" t="n">
+        <v>570</v>
+      </c>
+      <c r="E106" s="7" t="n">
+        <v>850</v>
+      </c>
+      <c r="F106" s="8">
+        <f>AVERAGE(D106:E106)</f>
+        <v/>
+      </c>
+      <c r="G106" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="H106" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I106" s="10">
+        <f>AVERAGE(G106:H106)</f>
+        <v/>
+      </c>
+      <c r="J106" s="9" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="K106" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="L106" s="10">
+        <f>AVERAGE(J106:K106)</f>
+        <v/>
+      </c>
+      <c r="M106" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N106" s="6" t="inlineStr">
+        <is>
+          <t>Rice halved; chicken fry is the protein anchor on a menu day with no meat listed</t>
         </is>
       </c>
     </row>
@@ -6284,11 +6339,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -6296,11 +6351,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -6308,11 +6363,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -6320,11 +6375,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A5,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -6337,11 +6392,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -6349,11 +6404,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -6361,11 +6416,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -6373,11 +6428,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A6,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -6390,11 +6445,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -6402,11 +6457,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -6414,11 +6469,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -6426,11 +6481,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A7,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -6443,11 +6498,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -6455,11 +6510,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -6467,11 +6522,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -6479,11 +6534,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A8,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -6496,11 +6551,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -6508,11 +6563,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -6520,11 +6575,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -6532,11 +6587,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A9,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -6549,11 +6604,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -6561,11 +6616,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -6573,11 +6628,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -6585,11 +6640,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A10,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -6602,11 +6657,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6614,11 +6669,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6626,11 +6681,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6638,11 +6693,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A11,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6655,11 +6710,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6667,11 +6722,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6679,11 +6734,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6691,11 +6746,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A12,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6708,11 +6763,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6720,11 +6775,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6732,11 +6787,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6744,11 +6799,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A13,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6761,11 +6816,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6773,11 +6828,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6785,11 +6840,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6797,11 +6852,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A14,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6814,11 +6869,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6826,11 +6881,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6838,11 +6893,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6850,11 +6905,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A15,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6867,11 +6922,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6879,11 +6934,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6891,11 +6946,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6903,11 +6958,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A16,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6920,11 +6975,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6932,11 +6987,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6944,11 +6999,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -6956,11 +7011,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A17,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -6973,11 +7028,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -6985,11 +7040,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -6997,11 +7052,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -7009,11 +7064,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A18,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -7026,11 +7081,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -7038,11 +7093,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -7050,11 +7105,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -7062,11 +7117,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A19,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -7079,11 +7134,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -7091,11 +7146,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -7103,11 +7158,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -7115,11 +7170,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A20,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -7132,11 +7187,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -7144,11 +7199,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -7156,11 +7211,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -7168,11 +7223,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A21,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -7185,11 +7240,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -7197,11 +7252,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -7209,11 +7264,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -7221,11 +7276,11 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A22,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">
@@ -7238,11 +7293,11 @@
         <v>46287</v>
       </c>
       <c r="B23" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C23" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D23" s="8">
@@ -7250,11 +7305,11 @@
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G23" s="10">
@@ -7262,11 +7317,11 @@
         <v/>
       </c>
       <c r="H23" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I23" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J23" s="10">
@@ -7274,11 +7329,11 @@
         <v/>
       </c>
       <c r="K23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A23,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M23" s="19">
@@ -7291,11 +7346,11 @@
         <v>46288</v>
       </c>
       <c r="B24" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C24" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D24" s="21">
@@ -7303,11 +7358,11 @@
         <v/>
       </c>
       <c r="E24" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F24" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G24" s="22">
@@ -7315,11 +7370,11 @@
         <v/>
       </c>
       <c r="H24" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I24" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J24" s="22">
@@ -7327,11 +7382,11 @@
         <v/>
       </c>
       <c r="K24" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L24" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A24,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M24" s="23">
@@ -7344,11 +7399,11 @@
         <v>46289</v>
       </c>
       <c r="B25" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$105,Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="C25" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$105,Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="D25" s="8">
@@ -7356,11 +7411,11 @@
         <v/>
       </c>
       <c r="E25" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$105,Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="F25" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$105,Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="G25" s="10">
@@ -7368,11 +7423,11 @@
         <v/>
       </c>
       <c r="H25" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$105,Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="I25" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$105,Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="J25" s="10">
@@ -7380,11 +7435,11 @@
         <v/>
       </c>
       <c r="K25" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"logged")</f>
         <v/>
       </c>
       <c r="L25" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$105,$A25,Meals!$M$5:$M$105,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"pending")</f>
         <v/>
       </c>
       <c r="M25" s="19">

</xml_diff>

<commit_message>
Log Day 21 snack and dinner; add pazham pori and beef reference rows
Day sits at 1,975 kcal and 72.5 g protein before whey. The pazham pori
is the lowest protein density in the reference table at 1.4 g/100 kcal.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N106"/>
+  <dimension ref="A1:N108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6172,39 +6172,39 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C106" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate - rice halved, pappadam, cabbage thoran, dal, curry gravy, 1 small chicken fry piece, small curd</t>
+          <t>Gobi chilly + 2 chapati</t>
         </is>
       </c>
       <c r="D106" s="7" t="n">
-        <v>570</v>
+        <v>400</v>
       </c>
       <c r="E106" s="7" t="n">
-        <v>850</v>
+        <v>560</v>
       </c>
       <c r="F106" s="8">
         <f>AVERAGE(D106:E106)</f>
         <v/>
       </c>
       <c r="G106" s="9" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="H106" s="9" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="I106" s="10">
         <f>AVERAGE(G106:H106)</f>
         <v/>
       </c>
       <c r="J106" s="9" t="n">
-        <v>22.5</v>
+        <v>16</v>
       </c>
       <c r="K106" s="9" t="n">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="L106" s="10">
         <f>AVERAGE(J106:K106)</f>
@@ -6217,7 +6217,117 @@
       </c>
       <c r="N106" s="6" t="inlineStr">
         <is>
+          <t>Thursday menu dinner as served; no meat on the menu</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C107" s="6" t="inlineStr">
+        <is>
+          <t>Mess meals plate - rice halved, pappadam, cabbage thoran, dal, curry gravy, 1 small chicken fry piece, small curd</t>
+        </is>
+      </c>
+      <c r="D107" s="7" t="n">
+        <v>570</v>
+      </c>
+      <c r="E107" s="7" t="n">
+        <v>850</v>
+      </c>
+      <c r="F107" s="8">
+        <f>AVERAGE(D107:E107)</f>
+        <v/>
+      </c>
+      <c r="G107" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="H107" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I107" s="10">
+        <f>AVERAGE(G107:H107)</f>
+        <v/>
+      </c>
+      <c r="J107" s="9" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="K107" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="L107" s="10">
+        <f>AVERAGE(J107:K107)</f>
+        <v/>
+      </c>
+      <c r="M107" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N107" s="6" t="inlineStr">
+        <is>
           <t>Rice halved; chicken fry is the protein anchor on a menu day with no meat listed</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="inlineStr">
+        <is>
+          <t>2 small pieces of beef from curry + 1 pazham pori</t>
+        </is>
+      </c>
+      <c r="D108" s="7" t="n">
+        <v>220</v>
+      </c>
+      <c r="E108" s="7" t="n">
+        <v>330</v>
+      </c>
+      <c r="F108" s="8">
+        <f>AVERAGE(D108:E108)</f>
+        <v/>
+      </c>
+      <c r="G108" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H108" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="I108" s="10">
+        <f>AVERAGE(G108:H108)</f>
+        <v/>
+      </c>
+      <c r="J108" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="K108" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="L108" s="10">
+        <f>AVERAGE(J108:K108)</f>
+        <v/>
+      </c>
+      <c r="M108" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N108" s="6" t="inlineStr">
+        <is>
+          <t>Pazham pori is deep-fried banana in batter; beef pieces are the only protein in the snack</t>
         </is>
       </c>
     </row>
@@ -6339,11 +6449,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -6351,11 +6461,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -6363,11 +6473,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -6375,11 +6485,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A5,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -6392,11 +6502,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -6404,11 +6514,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -6416,11 +6526,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -6428,11 +6538,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A6,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -6445,11 +6555,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -6457,11 +6567,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -6469,11 +6579,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -6481,11 +6591,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A7,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -6498,11 +6608,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -6510,11 +6620,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -6522,11 +6632,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -6534,11 +6644,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A8,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -6551,11 +6661,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -6563,11 +6673,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -6575,11 +6685,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -6587,11 +6697,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A9,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -6604,11 +6714,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -6616,11 +6726,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -6628,11 +6738,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -6640,11 +6750,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A10,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -6657,11 +6767,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6669,11 +6779,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6681,11 +6791,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6693,11 +6803,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A11,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6710,11 +6820,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6722,11 +6832,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6734,11 +6844,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6746,11 +6856,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A12,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6763,11 +6873,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6775,11 +6885,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6787,11 +6897,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6799,11 +6909,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A13,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6816,11 +6926,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6828,11 +6938,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6840,11 +6950,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6852,11 +6962,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A14,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6869,11 +6979,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6881,11 +6991,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -6893,11 +7003,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -6905,11 +7015,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A15,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -6922,11 +7032,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -6934,11 +7044,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -6946,11 +7056,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -6958,11 +7068,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A16,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -6975,11 +7085,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -6987,11 +7097,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -6999,11 +7109,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -7011,11 +7121,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A17,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -7028,11 +7138,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -7040,11 +7150,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -7052,11 +7162,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -7064,11 +7174,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A18,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -7081,11 +7191,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -7093,11 +7203,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -7105,11 +7215,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -7117,11 +7227,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A19,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -7134,11 +7244,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -7146,11 +7256,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -7158,11 +7268,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -7170,11 +7280,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A20,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -7187,11 +7297,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -7199,11 +7309,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -7211,11 +7321,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -7223,11 +7333,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A21,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -7240,11 +7350,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -7252,11 +7362,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -7264,11 +7374,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -7276,11 +7386,11 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A22,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">
@@ -7293,11 +7403,11 @@
         <v>46287</v>
       </c>
       <c r="B23" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C23" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D23" s="8">
@@ -7305,11 +7415,11 @@
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G23" s="10">
@@ -7317,11 +7427,11 @@
         <v/>
       </c>
       <c r="H23" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I23" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J23" s="10">
@@ -7329,11 +7439,11 @@
         <v/>
       </c>
       <c r="K23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A23,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M23" s="19">
@@ -7346,11 +7456,11 @@
         <v>46288</v>
       </c>
       <c r="B24" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C24" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D24" s="21">
@@ -7358,11 +7468,11 @@
         <v/>
       </c>
       <c r="E24" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F24" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G24" s="22">
@@ -7370,11 +7480,11 @@
         <v/>
       </c>
       <c r="H24" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I24" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J24" s="22">
@@ -7382,11 +7492,11 @@
         <v/>
       </c>
       <c r="K24" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L24" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A24,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M24" s="23">
@@ -7399,11 +7509,11 @@
         <v>46289</v>
       </c>
       <c r="B25" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$106,Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="C25" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$106,Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="D25" s="8">
@@ -7411,11 +7521,11 @@
         <v/>
       </c>
       <c r="E25" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$106,Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="F25" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$106,Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="G25" s="10">
@@ -7423,11 +7533,11 @@
         <v/>
       </c>
       <c r="H25" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$106,Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="I25" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$106,Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="J25" s="10">
@@ -7435,11 +7545,11 @@
         <v/>
       </c>
       <c r="K25" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"logged")</f>
         <v/>
       </c>
       <c r="L25" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$106,$A25,Meals!$M$5:$M$106,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"pending")</f>
         <v/>
       </c>
       <c r="M25" s="19">
@@ -9356,7 +9466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -10931,6 +11041,60 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>Pazham pori (banana fritter)</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="C63" s="7" t="n">
+        <v>220</v>
+      </c>
+      <c r="D63" s="8">
+        <f>AVERAGE(B63:C63)</f>
+        <v/>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>~2-3 g</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>Ripe banana in sweetened batter, deep fried. 1.4 g protein per 100 kcal - the lowest density logged</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>Beef curry (2 small pieces)</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="C64" s="7" t="n">
+        <v>110</v>
+      </c>
+      <c r="D64" s="8">
+        <f>AVERAGE(B64:C64)</f>
+        <v/>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>~8-12 g</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>Meat only, gravy not counted. ~11 g protein per 100 kcal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Log 88.75 weigh-in and close Day 21 at 72.5 g protein
First reading under 89. The seven-day intake average is 2,112 against a
2,120 target - the first rolling week to land on target. Protein is now
the only unsolved line at 107 g against a 130 g floor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -7571,7 +7571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7900,8 +7900,33 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="27" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B16" s="24" t="n">
+        <v>88.75</v>
+      </c>
+      <c r="C16" s="25">
+        <f>B16-B15</f>
+        <v/>
+      </c>
+      <c r="D16" s="25">
+        <f>B16-$B$5</f>
+        <v/>
+      </c>
+      <c r="E16" s="26">
+        <f>AVERAGE(B10:B16)</f>
+        <v/>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Morning weigh-in - second consecutive drop; second sub-89.3 reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t>A drop in the first week is mostly water and glycogen, not fat. Judge the trend over 2-3 weeks, and change the activity multiplier on Targets only then.</t>
         </is>

</xml_diff>

<commit_message>
Log Day 22 breakfast: idli set, white chutney skipped
345 kcal - the cheapest breakfast on the weekly rotation, and Friday is
the only day where three scoops fit inside target with room spare.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N108"/>
+  <dimension ref="A1:N109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6331,6 +6331,61 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" s="4" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C109" s="6" t="inlineStr">
+        <is>
+          <t>3 idli + sambar + red chutney (white chutney skipped)</t>
+        </is>
+      </c>
+      <c r="D109" s="7" t="n">
+        <v>280</v>
+      </c>
+      <c r="E109" s="7" t="n">
+        <v>410</v>
+      </c>
+      <c r="F109" s="8">
+        <f>AVERAGE(D109:E109)</f>
+        <v/>
+      </c>
+      <c r="G109" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H109" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="I109" s="10">
+        <f>AVERAGE(G109:H109)</f>
+        <v/>
+      </c>
+      <c r="J109" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="K109" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="L109" s="10">
+        <f>AVERAGE(J109:K109)</f>
+        <v/>
+      </c>
+      <c r="M109" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N109" s="6" t="inlineStr">
+        <is>
+          <t>Steamed not fried - cheapest breakfast on the weekly menu; twelfth consecutive white chutney skip</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -6345,7 +6400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6449,11 +6504,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -6461,11 +6516,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -6473,11 +6528,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -6485,11 +6540,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A5,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -6502,11 +6557,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -6514,11 +6569,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -6526,11 +6581,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -6538,11 +6593,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A6,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -6555,11 +6610,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -6567,11 +6622,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -6579,11 +6634,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -6591,11 +6646,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A7,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -6608,11 +6663,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -6620,11 +6675,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -6632,11 +6687,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -6644,11 +6699,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A8,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -6661,11 +6716,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -6673,11 +6728,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -6685,11 +6740,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -6697,11 +6752,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A9,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -6714,11 +6769,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -6726,11 +6781,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -6738,11 +6793,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -6750,11 +6805,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A10,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -6767,11 +6822,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6779,11 +6834,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6791,11 +6846,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6803,11 +6858,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A11,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6820,11 +6875,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6832,11 +6887,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6844,11 +6899,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6856,11 +6911,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A12,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6873,11 +6928,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6885,11 +6940,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6897,11 +6952,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6909,11 +6964,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A13,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6926,11 +6981,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6938,11 +6993,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -6950,11 +7005,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -6962,11 +7017,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A14,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -6979,11 +7034,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A15,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A15,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -6991,11 +7046,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A15,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A15,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -7003,11 +7058,11 @@
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A15,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A15,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J15" s="10">
@@ -7015,11 +7070,11 @@
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A15,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A15,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A15,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M15" s="19">
@@ -7032,11 +7087,11 @@
         <v>46280</v>
       </c>
       <c r="B16" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A16,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A16,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -7044,11 +7099,11 @@
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A16,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A16,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G16" s="22">
@@ -7056,11 +7111,11 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A16,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A16,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J16" s="22">
@@ -7068,11 +7123,11 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A16,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A16,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A16,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M16" s="23">
@@ -7085,11 +7140,11 @@
         <v>46281</v>
       </c>
       <c r="B17" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A17,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A17,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -7097,11 +7152,11 @@
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A17,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A17,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -7109,11 +7164,11 @@
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A17,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A17,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J17" s="10">
@@ -7121,11 +7176,11 @@
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A17,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A17,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A17,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M17" s="19">
@@ -7138,11 +7193,11 @@
         <v>46282</v>
       </c>
       <c r="B18" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A18,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A18,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -7150,11 +7205,11 @@
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A18,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A18,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G18" s="22">
@@ -7162,11 +7217,11 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A18,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A18,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J18" s="22">
@@ -7174,11 +7229,11 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A18,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A18,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A18,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M18" s="23">
@@ -7191,11 +7246,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A19,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A19,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -7203,11 +7258,11 @@
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A19,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A19,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -7215,11 +7270,11 @@
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A19,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A19,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J19" s="10">
@@ -7227,11 +7282,11 @@
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A19,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A19,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A19,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M19" s="19">
@@ -7244,11 +7299,11 @@
         <v>46284</v>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A20,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A20,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -7256,11 +7311,11 @@
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A20,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A20,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G20" s="22">
@@ -7268,11 +7323,11 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A20,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A20,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J20" s="22">
@@ -7280,11 +7335,11 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A20,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A20,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A20,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M20" s="23">
@@ -7297,11 +7352,11 @@
         <v>46285</v>
       </c>
       <c r="B21" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A21,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A21,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -7309,11 +7364,11 @@
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A21,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A21,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -7321,11 +7376,11 @@
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A21,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A21,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J21" s="10">
@@ -7333,11 +7388,11 @@
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A21,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A21,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A21,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M21" s="19">
@@ -7350,11 +7405,11 @@
         <v>46286</v>
       </c>
       <c r="B22" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A22,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A22,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -7362,11 +7417,11 @@
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A22,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A22,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G22" s="22">
@@ -7374,11 +7429,11 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A22,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A22,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J22" s="22">
@@ -7386,11 +7441,11 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A22,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A22,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A22,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M22" s="23">
@@ -7403,11 +7458,11 @@
         <v>46287</v>
       </c>
       <c r="B23" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A23,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C23" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A23,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D23" s="8">
@@ -7415,11 +7470,11 @@
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A23,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A23,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G23" s="10">
@@ -7427,11 +7482,11 @@
         <v/>
       </c>
       <c r="H23" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A23,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I23" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A23,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J23" s="10">
@@ -7439,11 +7494,11 @@
         <v/>
       </c>
       <c r="K23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A23,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L23" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A23,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A23,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M23" s="19">
@@ -7456,11 +7511,11 @@
         <v>46288</v>
       </c>
       <c r="B24" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A24,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C24" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A24,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D24" s="21">
@@ -7468,11 +7523,11 @@
         <v/>
       </c>
       <c r="E24" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A24,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F24" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A24,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G24" s="22">
@@ -7480,11 +7535,11 @@
         <v/>
       </c>
       <c r="H24" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A24,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I24" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A24,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J24" s="22">
@@ -7492,11 +7547,11 @@
         <v/>
       </c>
       <c r="K24" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A24,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L24" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A24,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A24,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M24" s="23">
@@ -7509,11 +7564,11 @@
         <v>46289</v>
       </c>
       <c r="B25" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$108,Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A25,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="C25" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$108,Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A25,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="D25" s="8">
@@ -7521,11 +7576,11 @@
         <v/>
       </c>
       <c r="E25" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$108,Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A25,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="F25" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$108,Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A25,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="G25" s="10">
@@ -7533,11 +7588,11 @@
         <v/>
       </c>
       <c r="H25" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$108,Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A25,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="I25" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$108,Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A25,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="J25" s="10">
@@ -7545,15 +7600,68 @@
         <v/>
       </c>
       <c r="K25" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A25,Meals!$M$5:$M$109,"logged")</f>
         <v/>
       </c>
       <c r="L25" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$108,$A25,Meals!$M$5:$M$108,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A25,Meals!$M$5:$M$109,"pending")</f>
         <v/>
       </c>
       <c r="M25" s="19">
         <f>D25-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B26" s="21">
+        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A26,Meals!$M$5:$M$109,"logged")</f>
+        <v/>
+      </c>
+      <c r="C26" s="21">
+        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A26,Meals!$M$5:$M$109,"logged")</f>
+        <v/>
+      </c>
+      <c r="D26" s="21">
+        <f>AVERAGE(B26:C26)</f>
+        <v/>
+      </c>
+      <c r="E26" s="22">
+        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A26,Meals!$M$5:$M$109,"logged")</f>
+        <v/>
+      </c>
+      <c r="F26" s="22">
+        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A26,Meals!$M$5:$M$109,"logged")</f>
+        <v/>
+      </c>
+      <c r="G26" s="22">
+        <f>AVERAGE(E26:F26)</f>
+        <v/>
+      </c>
+      <c r="H26" s="22">
+        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A26,Meals!$M$5:$M$109,"logged")</f>
+        <v/>
+      </c>
+      <c r="I26" s="22">
+        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A26,Meals!$M$5:$M$109,"logged")</f>
+        <v/>
+      </c>
+      <c r="J26" s="22">
+        <f>AVERAGE(H26:I26)</f>
+        <v/>
+      </c>
+      <c r="K26" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A26,Meals!$M$5:$M$109,"logged")</f>
+        <v/>
+      </c>
+      <c r="L26" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$109,$A26,Meals!$M$5:$M$109,"pending")</f>
+        <v/>
+      </c>
+      <c r="M26" s="23">
+        <f>D26-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -8687,7 +8795,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$25)</f>
+        <f>COUNT(Daily!$A$5:$A$26)</f>
         <v/>
       </c>
     </row>
@@ -8698,7 +8806,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$25),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$26),0)</f>
         <v/>
       </c>
     </row>
@@ -8709,7 +8817,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$25),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$26),0)</f>
         <v/>
       </c>
     </row>
@@ -8720,7 +8828,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$25),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$26),0)</f>
         <v/>
       </c>
     </row>
@@ -8764,7 +8872,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$25,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$26,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -8775,7 +8883,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$25)</f>
+        <f>SUM(Daily!$L$5:$L$26)</f>
         <v/>
       </c>
     </row>
@@ -8826,19 +8934,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$25,"&gt;="&amp;$A17,Daily!$A$5:$A$25,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$26,"&gt;="&amp;$A17,Daily!$A$5:$A$26,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$25,Daily!$A$5:$A$25,"&gt;="&amp;$A17,Daily!$A$5:$A$25,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$26,Daily!$A$5:$A$26,"&gt;="&amp;$A17,Daily!$A$5:$A$26,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$25,Daily!$A$5:$A$25,"&gt;="&amp;$A17,Daily!$A$5:$A$25,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$26,Daily!$A$5:$A$26,"&gt;="&amp;$A17,Daily!$A$5:$A$26,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$25,Daily!$A$5:$A$25,"&gt;="&amp;$A17,Daily!$A$5:$A$25,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$26,Daily!$A$5:$A$26,"&gt;="&amp;$A17,Daily!$A$5:$A$26,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -8850,19 +8958,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$25,"&gt;="&amp;$A18,Daily!$A$5:$A$25,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$26,"&gt;="&amp;$A18,Daily!$A$5:$A$26,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$25,Daily!$A$5:$A$25,"&gt;="&amp;$A18,Daily!$A$5:$A$25,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$26,Daily!$A$5:$A$26,"&gt;="&amp;$A18,Daily!$A$5:$A$26,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$25,Daily!$A$5:$A$25,"&gt;="&amp;$A18,Daily!$A$5:$A$25,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$26,Daily!$A$5:$A$26,"&gt;="&amp;$A18,Daily!$A$5:$A$26,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$25,Daily!$A$5:$A$25,"&gt;="&amp;$A18,Daily!$A$5:$A$25,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$26,Daily!$A$5:$A$26,"&gt;="&amp;$A18,Daily!$A$5:$A$26,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -8874,19 +8982,19 @@
         <v>46285</v>
       </c>
       <c r="C19" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$25,"&gt;="&amp;$A19,Daily!$A$5:$A$25,"&lt;="&amp;$B19)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$26,"&gt;="&amp;$A19,Daily!$A$5:$A$26,"&lt;="&amp;$B19)</f>
         <v/>
       </c>
       <c r="D19" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$25,Daily!$A$5:$A$25,"&gt;="&amp;$A19,Daily!$A$5:$A$25,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$26,Daily!$A$5:$A$26,"&gt;="&amp;$A19,Daily!$A$5:$A$26,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$25,Daily!$A$5:$A$25,"&gt;="&amp;$A19,Daily!$A$5:$A$25,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$26,Daily!$A$5:$A$26,"&gt;="&amp;$A19,Daily!$A$5:$A$26,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$25,Daily!$A$5:$A$25,"&gt;="&amp;$A19,Daily!$A$5:$A$25,"&lt;="&amp;$B19),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$26,Daily!$A$5:$A$26,"&gt;="&amp;$A19,Daily!$A$5:$A$26,"&lt;="&amp;$B19),0)</f>
         <v/>
       </c>
     </row>
@@ -8898,19 +9006,19 @@
         <v>46292</v>
       </c>
       <c r="C20" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$25,"&gt;="&amp;$A20,Daily!$A$5:$A$25,"&lt;="&amp;$B20)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$26,"&gt;="&amp;$A20,Daily!$A$5:$A$26,"&lt;="&amp;$B20)</f>
         <v/>
       </c>
       <c r="D20" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$25,Daily!$A$5:$A$25,"&gt;="&amp;$A20,Daily!$A$5:$A$25,"&lt;="&amp;$B20),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$26,Daily!$A$5:$A$26,"&gt;="&amp;$A20,Daily!$A$5:$A$26,"&lt;="&amp;$B20),0)</f>
         <v/>
       </c>
       <c r="E20" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$25,Daily!$A$5:$A$25,"&gt;="&amp;$A20,Daily!$A$5:$A$25,"&lt;="&amp;$B20),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$26,Daily!$A$5:$A$26,"&gt;="&amp;$A20,Daily!$A$5:$A$26,"&lt;="&amp;$B20),0)</f>
         <v/>
       </c>
       <c r="F20" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$25,Daily!$A$5:$A$25,"&gt;="&amp;$A20,Daily!$A$5:$A$25,"&lt;="&amp;$B20),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$26,Daily!$A$5:$A$26,"&gt;="&amp;$A20,Daily!$A$5:$A$26,"&lt;="&amp;$B20),0)</f>
         <v/>
       </c>
     </row>
@@ -8961,19 +9069,19 @@
         <v>46295</v>
       </c>
       <c r="C24" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$25,"&gt;="&amp;$A24,Daily!$A$5:$A$25,"&lt;="&amp;$B24)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$26,"&gt;="&amp;$A24,Daily!$A$5:$A$26,"&lt;="&amp;$B24)</f>
         <v/>
       </c>
       <c r="D24" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$25,Daily!$A$5:$A$25,"&gt;="&amp;$A24,Daily!$A$5:$A$25,"&lt;="&amp;$B24),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$26,Daily!$A$5:$A$26,"&gt;="&amp;$A24,Daily!$A$5:$A$26,"&lt;="&amp;$B24),0)</f>
         <v/>
       </c>
       <c r="E24" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$25,Daily!$A$5:$A$25,"&gt;="&amp;$A24,Daily!$A$5:$A$25,"&lt;="&amp;$B24),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$26,Daily!$A$5:$A$26,"&gt;="&amp;$A24,Daily!$A$5:$A$26,"&lt;="&amp;$B24),0)</f>
         <v/>
       </c>
       <c r="F24" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$25,Daily!$A$5:$A$25,"&gt;="&amp;$A24,Daily!$A$5:$A$25,"&lt;="&amp;$B24),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$26,Daily!$A$5:$A$26,"&gt;="&amp;$A24,Daily!$A$5:$A$26,"&lt;="&amp;$B24),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Day 22 lunch: biriyani with rice halved and both chicken pieces
670 kcal at 6.3 g protein per 100 kcal - the highest-protein lunch of
the twenty-two days.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N109"/>
+  <dimension ref="A1:N110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6383,6 +6383,61 @@
       <c r="N109" s="6" t="inlineStr">
         <is>
           <t>Steamed not fried - cheapest breakfast on the weekly menu; twelfth consecutive white chutney skip</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr">
+        <is>
+          <t>Chicken biriyani - rice halved, 2 chicken pieces, pappadam, salad/raita</t>
+        </is>
+      </c>
+      <c r="D110" s="7" t="n">
+        <v>550</v>
+      </c>
+      <c r="E110" s="7" t="n">
+        <v>790</v>
+      </c>
+      <c r="F110" s="8">
+        <f>AVERAGE(D110:E110)</f>
+        <v/>
+      </c>
+      <c r="G110" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="H110" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="I110" s="10">
+        <f>AVERAGE(G110:H110)</f>
+        <v/>
+      </c>
+      <c r="J110" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="K110" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="L110" s="10">
+        <f>AVERAGE(J110:K110)</f>
+        <v/>
+      </c>
+      <c r="M110" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N110" s="6" t="inlineStr">
+        <is>
+          <t>Rice halved but both chicken pieces kept; 6.3 g protein per 100 kcal</t>
         </is>
       </c>
     </row>
@@ -6504,11 +6559,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$110,Meals!$A$5:$A$110,$A5,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$110,Meals!$A$5:$A$110,$A5,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -6516,11 +6571,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$110,Meals!$A$5:$A$110,$A5,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$110,Meals!$A$5:$A$110,$A5,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -6528,11 +6583,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$110,Meals!$A$5:$A$110,$A5,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$110,Meals!$A$5:$A$110,$A5,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -6540,11 +6595,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A5,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A5,Meals!$M$5:$M$109,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A5,Meals!$M$5:$M$110,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -6557,11 +6612,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$110,Meals!$A$5:$A$110,$A6,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$110,Meals!$A$5:$A$110,$A6,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -6569,11 +6624,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$110,Meals!$A$5:$A$110,$A6,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$110,Meals!$A$5:$A$110,$A6,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -6581,11 +6636,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$110,Meals!$A$5:$A$110,$A6,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$110,Meals!$A$5:$A$110,$A6,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -6593,11 +6648,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A6,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A6,Meals!$M$5:$M$109,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A6,Meals!$M$5:$M$110,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -6610,11 +6665,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$110,Meals!$A$5:$A$110,$A7,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$110,Meals!$A$5:$A$110,$A7,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -6622,11 +6677,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$110,Meals!$A$5:$A$110,$A7,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$110,Meals!$A$5:$A$110,$A7,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -6634,11 +6689,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$110,Meals!$A$5:$A$110,$A7,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$110,Meals!$A$5:$A$110,$A7,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -6646,11 +6701,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A7,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A7,Meals!$M$5:$M$109,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A7,Meals!$M$5:$M$110,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -6663,11 +6718,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$110,Meals!$A$5:$A$110,$A8,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$110,Meals!$A$5:$A$110,$A8,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -6675,11 +6730,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$110,Meals!$A$5:$A$110,$A8,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$110,Meals!$A$5:$A$110,$A8,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -6687,11 +6742,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$110,Meals!$A$5:$A$110,$A8,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$110,Meals!$A$5:$A$110,$A8,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -6699,11 +6754,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A8,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A8,Meals!$M$5:$M$109,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A8,Meals!$M$5:$M$110,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -6716,11 +6771,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$110,Meals!$A$5:$A$110,$A9,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$110,Meals!$A$5:$A$110,$A9,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -6728,11 +6783,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$110,Meals!$A$5:$A$110,$A9,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$110,Meals!$A$5:$A$110,$A9,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -6740,11 +6795,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$110,Meals!$A$5:$A$110,$A9,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$110,Meals!$A$5:$A$110,$A9,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -6752,11 +6807,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A9,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A9,Meals!$M$5:$M$109,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A9,Meals!$M$5:$M$110,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -6769,11 +6824,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$110,Meals!$A$5:$A$110,$A10,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$110,Meals!$A$5:$A$110,$A10,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -6781,11 +6836,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$110,Meals!$A$5:$A$110,$A10,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$110,Meals!$A$5:$A$110,$A10,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -6793,11 +6848,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$110,Meals!$A$5:$A$110,$A10,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$110,Meals!$A$5:$A$110,$A10,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -6805,11 +6860,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A10,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A10,Meals!$M$5:$M$109,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A10,Meals!$M$5:$M$110,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -6822,11 +6877,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$110,Meals!$A$5:$A$110,$A11,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$110,Meals!$A$5:$A$110,$A11,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -6834,11 +6889,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$110,Meals!$A$5:$A$110,$A11,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$110,Meals!$A$5:$A$110,$A11,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -6846,11 +6901,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$110,Meals!$A$5:$A$110,$A11,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$110,Meals!$A$5:$A$110,$A11,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -6858,11 +6913,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A11,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A11,Meals!$M$5:$M$109,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A11,Meals!$M$5:$M$110,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -6875,11 +6930,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$110,Meals!$A$5:$A$110,$A12,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$110,Meals!$A$5:$A$110,$A12,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -6887,11 +6942,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$110,Meals!$A$5:$A$110,$A12,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$110,Meals!$A$5:$A$110,$A12,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -6899,11 +6954,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$110,Meals!$A$5:$A$110,$A12,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$110,Meals!$A$5:$A$110,$A12,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -6911,11 +6966,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A12,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A12,Meals!$M$5:$M$109,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A12,Meals!$M$5:$M$110,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -6928,11 +6983,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$110,Meals!$A$5:$A$110,$A13,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$110,Meals!$A$5:$A$110,$A13,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -6940,11 +6995,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$110,Meals!$A$5:$A$110,$A13,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$110,Meals!$A$5:$A$110,$A13,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -6952,11 +7007,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$110,Meals!$A$5:$A$110,$A13,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$110,Meals!$A$5:$A$110,$A13,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -6964,11 +7019,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A13,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A13,Meals!$M$5:$M$109,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A13,Meals!$M$5:$M$110,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">
@@ -6981,11 +7036,11 @@
         <v>46278</v>
       </c>
       <c r="B14" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$110,Meals!$A$5:$A$110,$A14,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$110,Meals!$A$5:$A$110,$A14,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -6993,11 +7048,11 @@
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$109,Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$110,Meals!$A$5:$A$110,$A14,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$109,Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$110,Meals!$A$5:$A$110,$A14,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="G14" s="22">
@@ -7005,11 +7060,11 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$109,Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$110,Meals!$A$5:$A$110,$A14,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$109,Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$110,Meals!$A$5:$A$110,$A14,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="J14" s="22">
@@ -7017,11 +7072,11 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A14,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$109,$A14,Meals!$M$5:$M$109,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$110,$A14,Meals!$M$5:$M$110,"pending")</f>
         <v/>
       </c>
       <c r="M14" s="23">
@@ -7034,11 +7089,11 @@
         <v>46279</v>
       </c>
       <c r="B15" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$109,Meals!$A$5:$A$109,$A15,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$110,Meals!$A$5:$A$110,$A15,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$109,Meals!$A$5:$A$109,$A15,Meals!$M$5:$M$109,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$110,Meals!$A$5:$A$110,$A15,Meals!$M$5:$M$110,"logged")</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -7046,11 +7101,11 @@
         <v/>
       </c>
       <c r="E15" s="10">
-